<commit_message>
extended metrics reported in .*evaluation.json files
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M18"/>
+  <dimension ref="A1:M19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -828,8 +828,8 @@
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>Title: App crashes when applying the "Use percent values" display option for the Incomes by Articles report.
-Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks "View values," checks "Use percent values," and taps "OK," the application crashes.
+          <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
+Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
 Expected Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
@@ -866,11 +866,11 @@
         </is>
       </c>
       <c r="L11" s="1">
-        <f>IFERROR(COUNTIF(K11:K18,"CS")/COUNTA(K11:K18),"")</f>
+        <f>IFERROR(COUNTIF(K11:K19,"CS")/COUNTA(K11:K19),"")</f>
         <v/>
       </c>
       <c r="M11" s="1">
-        <f>COUNTIF(K11:K18,"CS")/8</f>
+        <f>COUNTIF(K11:K19,"CS")/8</f>
         <v/>
       </c>
     </row>
@@ -884,7 +884,7 @@
       <c r="G12" s="1" t="inlineStr"/>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>Tap "Allow" on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
@@ -915,7 +915,7 @@
       <c r="G13" s="1" t="inlineStr"/>
       <c r="H13" s="1" t="inlineStr">
         <is>
-          <t>Tap "Reports" from the dashboard. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
         </is>
       </c>
       <c r="I13" s="1" t="inlineStr">
@@ -946,7 +946,7 @@
       <c r="G14" s="1" t="inlineStr"/>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>Tap "Incomes by Articles" on the Reports screen. &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Open the Incomes by Articles tab. &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
         </is>
       </c>
       <c r="I14" s="1" t="inlineStr">
@@ -977,7 +977,7 @@
       <c r="G15" s="1" t="inlineStr"/>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>Tap "Display" on the Incomes by Articles report screen. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Tap Display. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
         </is>
       </c>
       <c r="I15" s="1" t="inlineStr">
@@ -1008,7 +1008,7 @@
       <c r="G16" s="1" t="inlineStr"/>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>Check the "View values" checkbox. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Check View values. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
         </is>
       </c>
       <c r="I16" s="1" t="inlineStr">
@@ -1039,7 +1039,7 @@
       <c r="G17" s="1" t="inlineStr"/>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>Check the "Use percent values" checkbox. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Check Use percent values. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
         </is>
       </c>
       <c r="I17" s="1" t="inlineStr">
@@ -1070,7 +1070,7 @@
       <c r="G18" s="1" t="inlineStr"/>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>Tap "OK." &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Tap OK. &lt;ef26a526444b0c0827ef99ce6360670c18cb2ac563b206cf97bd84c9479fa5f6&gt;</t>
         </is>
       </c>
       <c r="I18" s="1" t="inlineStr">
@@ -1090,6 +1090,33 @@
       </c>
       <c r="L18" s="1" t="inlineStr"/>
       <c r="M18" s="1" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr"/>
+      <c r="B19" s="1" t="inlineStr"/>
+      <c r="C19" s="1" t="inlineStr"/>
+      <c r="D19" s="1" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr"/>
+      <c r="F19" s="1" t="inlineStr"/>
+      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>If a crash dialog appears, tap OK. &lt;6aa06c426f17d83ac768c98cc6d31a987166d855462845d0b306e83f26fa76f9&gt;</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr"/>
+      <c r="K19" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L19" s="1" t="inlineStr"/>
+      <c r="M19" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1289,8 +1316,8 @@
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>Title: App crashes when applying the "Use percent values" display option for the Incomes by Articles report.
-Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks "View values," checks "Use percent values," and taps "OK," the application crashes.
+          <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
+Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
 Expected Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
@@ -1305,7 +1332,7 @@
       <c r="H4" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
-Triggering GUI Interactions: checks "View values," checks "Use percent values," and taps "OK"
+Triggering GUI Interactions: checks the View values checkbox, checks the Use percent values checkbox, and taps OK
 Triggering Screen Reference: On the Display of Incomes by Articles pop-up of the Reports screen
 Correct Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>

</xml_diff>

<commit_message>
fixed summary csv, added f1
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="S2R Review" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Info Elements Review" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -439,6 +440,8 @@
     <col width="18" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col hidden="1" width="14" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,6 +508,16 @@
       <c r="M1" t="inlineStr">
         <is>
           <t>Recall</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>GT Step Count</t>
         </is>
       </c>
     </row>
@@ -576,6 +589,13 @@
       <c r="M2" s="1">
         <f>COUNTIF(K2:K9,"CS")/6</f>
         <v/>
+      </c>
+      <c r="N2" s="1">
+        <f>IFERROR(2*(L2*M2)/(L2+M2),"")</f>
+        <v/>
+      </c>
+      <c r="O2" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -608,6 +628,8 @@
       </c>
       <c r="L3" s="1" t="inlineStr"/>
       <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr"/>
+      <c r="O3" s="1" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr"/>
@@ -639,6 +661,8 @@
       </c>
       <c r="L4" s="1" t="inlineStr"/>
       <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="inlineStr"/>
+      <c r="O4" s="1" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr"/>
@@ -670,6 +694,8 @@
       </c>
       <c r="L5" s="1" t="inlineStr"/>
       <c r="M5" s="1" t="inlineStr"/>
+      <c r="N5" s="1" t="inlineStr"/>
+      <c r="O5" s="1" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr"/>
@@ -701,6 +727,8 @@
       </c>
       <c r="L6" s="1" t="inlineStr"/>
       <c r="M6" s="1" t="inlineStr"/>
+      <c r="N6" s="1" t="inlineStr"/>
+      <c r="O6" s="1" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr"/>
@@ -732,6 +760,8 @@
       </c>
       <c r="L7" s="1" t="inlineStr"/>
       <c r="M7" s="1" t="inlineStr"/>
+      <c r="N7" s="1" t="inlineStr"/>
+      <c r="O7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr"/>
@@ -759,6 +789,8 @@
       </c>
       <c r="L8" s="1" t="inlineStr"/>
       <c r="M8" s="1" t="inlineStr"/>
+      <c r="N8" s="1" t="inlineStr"/>
+      <c r="O8" s="1" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr"/>
@@ -786,6 +818,8 @@
       </c>
       <c r="L9" s="1" t="inlineStr"/>
       <c r="M9" s="1" t="inlineStr"/>
+      <c r="N9" s="1" t="inlineStr"/>
+      <c r="O9" s="1" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr"/>
@@ -801,6 +835,8 @@
       <c r="K10" s="2" t="inlineStr"/>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -872,6 +908,13 @@
       <c r="M11" s="1">
         <f>COUNTIF(K11:K19,"CS")/8</f>
         <v/>
+      </c>
+      <c r="N11" s="1">
+        <f>IFERROR(2*(L11*M11)/(L11+M11),"")</f>
+        <v/>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>8</v>
       </c>
     </row>
     <row r="12">
@@ -904,6 +947,8 @@
       </c>
       <c r="L12" s="1" t="inlineStr"/>
       <c r="M12" s="1" t="inlineStr"/>
+      <c r="N12" s="1" t="inlineStr"/>
+      <c r="O12" s="1" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="1" t="inlineStr"/>
@@ -935,6 +980,8 @@
       </c>
       <c r="L13" s="1" t="inlineStr"/>
       <c r="M13" s="1" t="inlineStr"/>
+      <c r="N13" s="1" t="inlineStr"/>
+      <c r="O13" s="1" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr"/>
@@ -966,6 +1013,8 @@
       </c>
       <c r="L14" s="1" t="inlineStr"/>
       <c r="M14" s="1" t="inlineStr"/>
+      <c r="N14" s="1" t="inlineStr"/>
+      <c r="O14" s="1" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="1" t="inlineStr"/>
@@ -997,6 +1046,8 @@
       </c>
       <c r="L15" s="1" t="inlineStr"/>
       <c r="M15" s="1" t="inlineStr"/>
+      <c r="N15" s="1" t="inlineStr"/>
+      <c r="O15" s="1" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr"/>
@@ -1028,6 +1079,8 @@
       </c>
       <c r="L16" s="1" t="inlineStr"/>
       <c r="M16" s="1" t="inlineStr"/>
+      <c r="N16" s="1" t="inlineStr"/>
+      <c r="O16" s="1" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="1" t="inlineStr"/>
@@ -1059,6 +1112,8 @@
       </c>
       <c r="L17" s="1" t="inlineStr"/>
       <c r="M17" s="1" t="inlineStr"/>
+      <c r="N17" s="1" t="inlineStr"/>
+      <c r="O17" s="1" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="1" t="inlineStr"/>
@@ -1090,6 +1145,8 @@
       </c>
       <c r="L18" s="1" t="inlineStr"/>
       <c r="M18" s="1" t="inlineStr"/>
+      <c r="N18" s="1" t="inlineStr"/>
+      <c r="O18" s="1" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="1" t="inlineStr"/>
@@ -1117,6 +1174,8 @@
       </c>
       <c r="L19" s="1" t="inlineStr"/>
       <c r="M19" s="1" t="inlineStr"/>
+      <c r="N19" s="1" t="inlineStr"/>
+      <c r="O19" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1262,7 +1321,7 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Correct</t>
+          <t>Incorrect</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
@@ -1361,4 +1420,172 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:O2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="19" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="34" customWidth="1" min="13" max="13"/>
+    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="26" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>agent_version</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>s2r_cs_count</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>s2r_ms_count</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>s2r_es_count</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>average_s2r_precision</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>average_s2r_recall</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>average_s2r_f1</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>info_correct_count</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>info_incomplete_count</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>info_ambiguous_count</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>info_missing_count</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>info_incorrect_count</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>average_total_tokens_consumed_per_conv</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>average_conversation_time_in_seconds</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>average_conversation_turns</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="B2">
+        <f>COUNTIF('S2R Review'!$K:$K,"CS")</f>
+        <v/>
+      </c>
+      <c r="C2">
+        <f>SUM('S2R Review'!$O:$O)-B2</f>
+        <v/>
+      </c>
+      <c r="D2">
+        <f>COUNTIF('S2R Review'!$K:$K,"ES")</f>
+        <v/>
+      </c>
+      <c r="E2">
+        <f>IFERROR(SUM('S2R Review'!$L$2:$L$1048576)/COUNTIF('S2R Review'!$L$2:$L$1048576,"&lt;&gt;"),"")</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>IFERROR(SUM('S2R Review'!$M$2:$M$1048576)/COUNTIF('S2R Review'!$M$2:$M$1048576,"&lt;&gt;"),"")</f>
+        <v/>
+      </c>
+      <c r="G2">
+        <f>IFERROR(SUM('S2R Review'!$N$2:$N$1048576)/COUNTIF('S2R Review'!$N$2:$N$1048576,"&lt;&gt;"),"")</f>
+        <v/>
+      </c>
+      <c r="H2">
+        <f>COUNTIF('Info Elements Review'!$I:$I,"Correct")+COUNTIF('Info Elements Review'!$J:$J,"Correct")+COUNTIF('Info Elements Review'!$K:$K,"Correct")+COUNTIF('Info Elements Review'!$L:$L,"Correct")</f>
+        <v/>
+      </c>
+      <c r="I2">
+        <f>COUNTIF('Info Elements Review'!$I:$I,"Incomplete")+COUNTIF('Info Elements Review'!$J:$J,"Incomplete")+COUNTIF('Info Elements Review'!$K:$K,"Incomplete")+COUNTIF('Info Elements Review'!$L:$L,"Incomplete")</f>
+        <v/>
+      </c>
+      <c r="J2">
+        <f>COUNTIF('Info Elements Review'!$I:$I,"Ambiguous")+COUNTIF('Info Elements Review'!$J:$J,"Ambiguous")+COUNTIF('Info Elements Review'!$K:$K,"Ambiguous")+COUNTIF('Info Elements Review'!$L:$L,"Ambiguous")</f>
+        <v/>
+      </c>
+      <c r="K2">
+        <f>COUNTIF('Info Elements Review'!$I:$I,"Missing")+COUNTIF('Info Elements Review'!$J:$J,"Missing")+COUNTIF('Info Elements Review'!$K:$K,"Missing")+COUNTIF('Info Elements Review'!$L:$L,"Missing")</f>
+        <v/>
+      </c>
+      <c r="L2">
+        <f>COUNTIF('Info Elements Review'!$I:$I,"Incorrect")+COUNTIF('Info Elements Review'!$J:$J,"Incorrect")+COUNTIF('Info Elements Review'!$K:$K,"Incorrect")+COUNTIF('Info Elements Review'!$L:$L,"Incorrect")</f>
+        <v/>
+      </c>
+      <c r="M2" t="n">
+        <v>155648</v>
+      </c>
+      <c r="N2" t="n">
+        <v>204.5602267084996</v>
+      </c>
+      <c r="O2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
updated run_all_burt to fully collect/eval burt++ runs
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O19"/>
+  <dimension ref="A1:O35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -840,11 +840,11 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>Family Finance</t>
+          <t>Wikimedia Commons</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
@@ -859,31 +859,38 @@
       </c>
       <c r="E11" s="1" t="inlineStr">
         <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F11" s="1" t="inlineStr">
         <is>
-          <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
-Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
-Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the Parent Categories tab, the page is blank.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G11" s="1" t="inlineStr">
         <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
+2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
+3. Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;
+4. Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;
+5. Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;
+6. Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;
+7. Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;
+8. Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;
+9. Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;
+10. Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;
+11. Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;
+12. Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;
+13. Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;
+14. Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;
+15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="H11" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
       <c r="I11" s="1" t="inlineStr">
@@ -893,7 +900,7 @@
       </c>
       <c r="J11" s="1" t="inlineStr">
         <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
       <c r="K11" s="1" t="inlineStr">
@@ -902,11 +909,11 @@
         </is>
       </c>
       <c r="L11" s="1">
-        <f>IFERROR(COUNTIF(K11:K19,"CS")/COUNTA(K11:K19),"")</f>
+        <f>IFERROR(COUNTIF(K11:K25,"CS")/COUNTA(K11:K25),"")</f>
         <v/>
       </c>
       <c r="M11" s="1">
-        <f>COUNTIF(K11:K19,"CS")/8</f>
+        <f>COUNTIF(K11:K25,"CS")/15</f>
         <v/>
       </c>
       <c r="N11" s="1">
@@ -914,7 +921,7 @@
         <v/>
       </c>
       <c r="O11" s="1" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
     </row>
     <row r="12">
@@ -927,7 +934,7 @@
       <c r="G12" s="1" t="inlineStr"/>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Swipe left on the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
@@ -937,7 +944,7 @@
       </c>
       <c r="J12" s="1" t="inlineStr">
         <is>
-          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K12" s="1" t="inlineStr">
@@ -960,7 +967,7 @@
       <c r="G13" s="1" t="inlineStr"/>
       <c r="H13" s="1" t="inlineStr">
         <is>
-          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I13" s="1" t="inlineStr">
@@ -970,7 +977,7 @@
       </c>
       <c r="J13" s="1" t="inlineStr">
         <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K13" s="1" t="inlineStr">
@@ -993,7 +1000,7 @@
       <c r="G14" s="1" t="inlineStr"/>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>Open the Incomes by Articles tab. &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I14" s="1" t="inlineStr">
@@ -1003,7 +1010,7 @@
       </c>
       <c r="J14" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K14" s="1" t="inlineStr">
@@ -1026,7 +1033,7 @@
       <c r="G15" s="1" t="inlineStr"/>
       <c r="H15" s="1" t="inlineStr">
         <is>
-          <t>Tap Display. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I15" s="1" t="inlineStr">
@@ -1036,7 +1043,7 @@
       </c>
       <c r="J15" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K15" s="1" t="inlineStr">
@@ -1059,7 +1066,7 @@
       <c r="G16" s="1" t="inlineStr"/>
       <c r="H16" s="1" t="inlineStr">
         <is>
-          <t>Check View values. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Tap "YES!" on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I16" s="1" t="inlineStr">
@@ -1069,7 +1076,7 @@
       </c>
       <c r="J16" s="1" t="inlineStr">
         <is>
-          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="K16" s="1" t="inlineStr">
@@ -1092,7 +1099,7 @@
       <c r="G17" s="1" t="inlineStr"/>
       <c r="H17" s="1" t="inlineStr">
         <is>
-          <t>Check Use percent values. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I17" s="1" t="inlineStr">
@@ -1102,7 +1109,7 @@
       </c>
       <c r="J17" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="K17" s="1" t="inlineStr">
@@ -1125,7 +1132,7 @@
       <c r="G18" s="1" t="inlineStr"/>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>Tap OK. &lt;ef26a526444b0c0827ef99ce6360670c18cb2ac563b206cf97bd84c9479fa5f6&gt;</t>
+          <t>Tap "YES" on the skip login confirmation dialog. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I18" s="1" t="inlineStr">
@@ -1135,7 +1142,7 @@
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="K18" s="1" t="inlineStr">
@@ -1158,24 +1165,582 @@
       <c r="G19" s="1" t="inlineStr"/>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>If a crash dialog appears, tap OK. &lt;6aa06c426f17d83ac768c98cc6d31a987166d855462845d0b306e83f26fa76f9&gt;</t>
+          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="I19" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J19" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
       <c r="K19" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L19" s="1" t="inlineStr"/>
       <c r="M19" s="1" t="inlineStr"/>
       <c r="N19" s="1" t="inlineStr"/>
       <c r="O19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="1" t="inlineStr"/>
+      <c r="C20" s="1" t="inlineStr"/>
+      <c r="D20" s="1" t="inlineStr"/>
+      <c r="E20" s="1" t="inlineStr"/>
+      <c r="F20" s="1" t="inlineStr"/>
+      <c r="G20" s="1" t="inlineStr"/>
+      <c r="H20" s="1" t="inlineStr">
+        <is>
+          <t>Select "Explore" from the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+        </is>
+      </c>
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="inlineStr">
+        <is>
+          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+        </is>
+      </c>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L20" s="1" t="inlineStr"/>
+      <c r="M20" s="1" t="inlineStr"/>
+      <c r="N20" s="1" t="inlineStr"/>
+      <c r="O20" s="1" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="1" t="inlineStr"/>
+      <c r="B21" s="1" t="inlineStr"/>
+      <c r="C21" s="1" t="inlineStr"/>
+      <c r="D21" s="1" t="inlineStr"/>
+      <c r="E21" s="1" t="inlineStr"/>
+      <c r="F21" s="1" t="inlineStr"/>
+      <c r="G21" s="1" t="inlineStr"/>
+      <c r="H21" s="1" t="inlineStr">
+        <is>
+          <t>Tap a picture in the Explore grid to open its media details. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="I21" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J21" s="1" t="inlineStr">
+        <is>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="K21" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L21" s="1" t="inlineStr"/>
+      <c r="M21" s="1" t="inlineStr"/>
+      <c r="N21" s="1" t="inlineStr"/>
+      <c r="O21" s="1" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr"/>
+      <c r="B22" s="1" t="inlineStr"/>
+      <c r="C22" s="1" t="inlineStr"/>
+      <c r="D22" s="1" t="inlineStr"/>
+      <c r="E22" s="1" t="inlineStr"/>
+      <c r="F22" s="1" t="inlineStr"/>
+      <c r="G22" s="1" t="inlineStr"/>
+      <c r="H22" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="I22" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J22" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="K22" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L22" s="1" t="inlineStr"/>
+      <c r="M22" s="1" t="inlineStr"/>
+      <c r="N22" s="1" t="inlineStr"/>
+      <c r="O22" s="1" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr"/>
+      <c r="B23" s="1" t="inlineStr"/>
+      <c r="C23" s="1" t="inlineStr"/>
+      <c r="D23" s="1" t="inlineStr"/>
+      <c r="E23" s="1" t="inlineStr"/>
+      <c r="F23" s="1" t="inlineStr"/>
+      <c r="G23" s="1" t="inlineStr"/>
+      <c r="H23" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="I23" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="K23" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L23" s="1" t="inlineStr"/>
+      <c r="M23" s="1" t="inlineStr"/>
+      <c r="N23" s="1" t="inlineStr"/>
+      <c r="O23" s="1" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="inlineStr"/>
+      <c r="B24" s="1" t="inlineStr"/>
+      <c r="C24" s="1" t="inlineStr"/>
+      <c r="D24" s="1" t="inlineStr"/>
+      <c r="E24" s="1" t="inlineStr"/>
+      <c r="F24" s="1" t="inlineStr"/>
+      <c r="G24" s="1" t="inlineStr"/>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Tap a category from the media details categories list. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr">
+        <is>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L24" s="1" t="inlineStr"/>
+      <c r="M24" s="1" t="inlineStr"/>
+      <c r="N24" s="1" t="inlineStr"/>
+      <c r="O24" s="1" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="inlineStr"/>
+      <c r="B25" s="1" t="inlineStr"/>
+      <c r="C25" s="1" t="inlineStr"/>
+      <c r="D25" s="1" t="inlineStr"/>
+      <c r="E25" s="1" t="inlineStr"/>
+      <c r="F25" s="1" t="inlineStr"/>
+      <c r="G25" s="1" t="inlineStr"/>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L25" s="1" t="inlineStr"/>
+      <c r="M25" s="1" t="inlineStr"/>
+      <c r="N25" s="1" t="inlineStr"/>
+      <c r="O25" s="1" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B27" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C27" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>HC_HP</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr">
+        <is>
+          <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
+Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
+Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
+      <c r="G27" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H27" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J27" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K27" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L27" s="1">
+        <f>IFERROR(COUNTIF(K27:K35,"CS")/COUNTA(K27:K35),"")</f>
+        <v/>
+      </c>
+      <c r="M27" s="1">
+        <f>COUNTIF(K27:K35,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N27" s="1">
+        <f>IFERROR(2*(L27*M27)/(L27+M27),"")</f>
+        <v/>
+      </c>
+      <c r="O27" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="inlineStr"/>
+      <c r="B28" s="1" t="inlineStr"/>
+      <c r="C28" s="1" t="inlineStr"/>
+      <c r="D28" s="1" t="inlineStr"/>
+      <c r="E28" s="1" t="inlineStr"/>
+      <c r="F28" s="1" t="inlineStr"/>
+      <c r="G28" s="1" t="inlineStr"/>
+      <c r="H28" s="1" t="inlineStr">
+        <is>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="I28" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="K28" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L28" s="1" t="inlineStr"/>
+      <c r="M28" s="1" t="inlineStr"/>
+      <c r="N28" s="1" t="inlineStr"/>
+      <c r="O28" s="1" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr"/>
+      <c r="B29" s="1" t="inlineStr"/>
+      <c r="C29" s="1" t="inlineStr"/>
+      <c r="D29" s="1" t="inlineStr"/>
+      <c r="E29" s="1" t="inlineStr"/>
+      <c r="F29" s="1" t="inlineStr"/>
+      <c r="G29" s="1" t="inlineStr"/>
+      <c r="H29" s="1" t="inlineStr">
+        <is>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I29" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J29" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K29" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L29" s="1" t="inlineStr"/>
+      <c r="M29" s="1" t="inlineStr"/>
+      <c r="N29" s="1" t="inlineStr"/>
+      <c r="O29" s="1" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="1" t="inlineStr"/>
+      <c r="B30" s="1" t="inlineStr"/>
+      <c r="C30" s="1" t="inlineStr"/>
+      <c r="D30" s="1" t="inlineStr"/>
+      <c r="E30" s="1" t="inlineStr"/>
+      <c r="F30" s="1" t="inlineStr"/>
+      <c r="G30" s="1" t="inlineStr"/>
+      <c r="H30" s="1" t="inlineStr">
+        <is>
+          <t>Open the Incomes by Articles tab. &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="I30" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J30" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K30" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L30" s="1" t="inlineStr"/>
+      <c r="M30" s="1" t="inlineStr"/>
+      <c r="N30" s="1" t="inlineStr"/>
+      <c r="O30" s="1" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr"/>
+      <c r="B31" s="1" t="inlineStr"/>
+      <c r="C31" s="1" t="inlineStr"/>
+      <c r="D31" s="1" t="inlineStr"/>
+      <c r="E31" s="1" t="inlineStr"/>
+      <c r="F31" s="1" t="inlineStr"/>
+      <c r="G31" s="1" t="inlineStr"/>
+      <c r="H31" s="1" t="inlineStr">
+        <is>
+          <t>Tap Display. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I31" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K31" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L31" s="1" t="inlineStr"/>
+      <c r="M31" s="1" t="inlineStr"/>
+      <c r="N31" s="1" t="inlineStr"/>
+      <c r="O31" s="1" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="1" t="inlineStr"/>
+      <c r="B32" s="1" t="inlineStr"/>
+      <c r="C32" s="1" t="inlineStr"/>
+      <c r="D32" s="1" t="inlineStr"/>
+      <c r="E32" s="1" t="inlineStr"/>
+      <c r="F32" s="1" t="inlineStr"/>
+      <c r="G32" s="1" t="inlineStr"/>
+      <c r="H32" s="1" t="inlineStr">
+        <is>
+          <t>Check View values. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="I32" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J32" s="1" t="inlineStr">
+        <is>
+          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="K32" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L32" s="1" t="inlineStr"/>
+      <c r="M32" s="1" t="inlineStr"/>
+      <c r="N32" s="1" t="inlineStr"/>
+      <c r="O32" s="1" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="1" t="inlineStr"/>
+      <c r="B33" s="1" t="inlineStr"/>
+      <c r="C33" s="1" t="inlineStr"/>
+      <c r="D33" s="1" t="inlineStr"/>
+      <c r="E33" s="1" t="inlineStr"/>
+      <c r="F33" s="1" t="inlineStr"/>
+      <c r="G33" s="1" t="inlineStr"/>
+      <c r="H33" s="1" t="inlineStr">
+        <is>
+          <t>Check Use percent values. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I33" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K33" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L33" s="1" t="inlineStr"/>
+      <c r="M33" s="1" t="inlineStr"/>
+      <c r="N33" s="1" t="inlineStr"/>
+      <c r="O33" s="1" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="inlineStr"/>
+      <c r="B34" s="1" t="inlineStr"/>
+      <c r="C34" s="1" t="inlineStr"/>
+      <c r="D34" s="1" t="inlineStr"/>
+      <c r="E34" s="1" t="inlineStr"/>
+      <c r="F34" s="1" t="inlineStr"/>
+      <c r="G34" s="1" t="inlineStr"/>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>Tap OK. &lt;ef26a526444b0c0827ef99ce6360670c18cb2ac563b206cf97bd84c9479fa5f6&gt;</t>
+        </is>
+      </c>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L34" s="1" t="inlineStr"/>
+      <c r="M34" s="1" t="inlineStr"/>
+      <c r="N34" s="1" t="inlineStr"/>
+      <c r="O34" s="1" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr"/>
+      <c r="B35" s="1" t="inlineStr"/>
+      <c r="C35" s="1" t="inlineStr"/>
+      <c r="D35" s="1" t="inlineStr"/>
+      <c r="E35" s="1" t="inlineStr"/>
+      <c r="F35" s="1" t="inlineStr"/>
+      <c r="G35" s="1" t="inlineStr"/>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>If a crash dialog appears, tap OK. &lt;6aa06c426f17d83ac768c98cc6d31a987166d855462845d0b306e83f26fa76f9&gt;</t>
+        </is>
+      </c>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="inlineStr"/>
+      <c r="K35" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L35" s="1" t="inlineStr"/>
+      <c r="M35" s="1" t="inlineStr"/>
+      <c r="N35" s="1" t="inlineStr"/>
+      <c r="O35" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1188,7 +1753,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1351,36 +1916,118 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>HC_HP</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the Parent Categories tab, the page is blank.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
+        </is>
+      </c>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the page is blank
+Triggering GUI Interactions: taps the Parent Categories tab
+Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="inlineStr">
+      <c r="B6" s="1" t="inlineStr">
         <is>
           <t>Family Finance</t>
         </is>
       </c>
-      <c r="C4" s="1" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D4" s="1" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>HC_HP</t>
         </is>
       </c>
-      <c r="E4" s="1" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
         </is>
       </c>
-      <c r="F4" s="1" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
 Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
 Expected Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
-      <c r="G4" s="1" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
 Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
@@ -1388,7 +2035,7 @@
 Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
         </is>
       </c>
-      <c r="H4" s="1" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
 Triggering GUI Interactions: checks the View values checkbox, checks the Use percent values checkbox, and taps OK
@@ -1396,22 +2043,22 @@
 Correct Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
-      <c r="I4" s="1" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="J4" s="1" t="inlineStr">
+      <c r="J6" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="K4" s="1" t="inlineStr">
+      <c r="K6" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="L4" s="1" t="inlineStr">
+      <c r="L6" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -1576,13 +2223,13 @@
         <v/>
       </c>
       <c r="M2" t="n">
-        <v>155648</v>
+        <v>118778.6666666667</v>
       </c>
       <c r="N2" t="n">
-        <v>204.5602267084996</v>
+        <v>149.7703270973331</v>
       </c>
       <c r="O2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding results from most recent diminished dev set run
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O35"/>
+  <dimension ref="A1:O68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -537,19 +537,19 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>LC_LP</t>
+          <t>HC_LP</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>It restarts on its own.</t>
+          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Title: FTP server restarts on its own after being toggled and the app is dismissed from Recents
-Observed Behavior: On the FTP server screen, if the user turns the FTP server on, turns it off, presses Back to leave the app, and dismisses the Files app from the Recents screen, the FTP server restarts on its own.
-Expected Behavior: The FTP server should not restart on its own.</t>
+          <t>Title: FTP server restarts automatically after being stopped and the app is closed
+Observed Behavior: On the FTP server screen, if the user turns off the FTP server switch and then closes the app, the FTP server restarts automatically after stopping it and closing the app.
+Expected Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Open the Files app.</t>
+          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
@@ -583,11 +583,11 @@
         </is>
       </c>
       <c r="L2" s="1">
-        <f>IFERROR(COUNTIF(K2:K9,"CS")/COUNTA(K2:K9),"")</f>
+        <f>IFERROR(COUNTIF(K2:K7,"CS")/COUNTA(K2:K7),"")</f>
         <v/>
       </c>
       <c r="M2" s="1">
-        <f>COUNTIF(K2:K9,"CS")/6</f>
+        <f>COUNTIF(K2:K7,"CS")/6</f>
         <v/>
       </c>
       <c r="N2" s="1">
@@ -608,7 +608,7 @@
       <c r="G3" s="1" t="inlineStr"/>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>On the permission dialog, tap Allow.</t>
+          <t>Grant the storage permission by tapping Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
         </is>
       </c>
       <c r="I3" s="1" t="inlineStr">
@@ -641,7 +641,7 @@
       <c r="G4" s="1" t="inlineStr"/>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Tap the Navigate up button.</t>
+          <t>Open the navigation drawer from the main Files screen. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -674,7 +674,7 @@
       <c r="G5" s="1" t="inlineStr"/>
       <c r="H5" s="1" t="inlineStr">
         <is>
-          <t>Tap FTP server.</t>
+          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="I5" s="1" t="inlineStr">
@@ -707,7 +707,7 @@
       <c r="G6" s="1" t="inlineStr"/>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>On the FTP server screen, tap the switch to turn the FTP server on.</t>
+          <t>On the FTP server screen, tap the ON switch to stop the FTP server. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -740,22 +740,18 @@
       <c r="G7" s="1" t="inlineStr"/>
       <c r="H7" s="1" t="inlineStr">
         <is>
-          <t>Tap the switch to turn the FTP server off.</t>
+          <t>Close the app by pressing Back from the FTP server screen. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
         </is>
       </c>
       <c r="I7" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J7" s="1" t="inlineStr">
-        <is>
-          <t>Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr"/>
       <c r="K7" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L7" s="1" t="inlineStr"/>
@@ -764,112 +760,429 @@
       <c r="O7" s="1" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr"/>
-      <c r="B8" s="1" t="inlineStr"/>
-      <c r="C8" s="1" t="inlineStr"/>
-      <c r="D8" s="1" t="inlineStr"/>
-      <c r="E8" s="1" t="inlineStr"/>
-      <c r="F8" s="1" t="inlineStr"/>
-      <c r="G8" s="1" t="inlineStr"/>
-      <c r="H8" s="1" t="inlineStr">
-        <is>
-          <t>Press Back to leave the app.</t>
-        </is>
-      </c>
-      <c r="I8" s="1" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B9" s="1" t="inlineStr">
+        <is>
+          <t>Material Files</t>
+        </is>
+      </c>
+      <c r="C9" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="inlineStr">
+        <is>
+          <t>LC_LP</t>
+        </is>
+      </c>
+      <c r="E9" s="1" t="inlineStr">
+        <is>
+          <t>It restarts on its own.</t>
+        </is>
+      </c>
+      <c r="F9" s="1" t="inlineStr">
+        <is>
+          <t>Title: FTP server restarts automatically after being turned off and leaving the FTP server screen
+Observed Behavior: On the FTP server screen, if the user turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents, the FTP server is restarting on its own.
+Expected Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
+        </is>
+      </c>
+      <c r="G9" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
+2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
+3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
+4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
+5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
+6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L9" s="1">
+        <f>IFERROR(COUNTIF(K9:K18,"CS")/COUNTA(K9:K18),"")</f>
+        <v/>
+      </c>
+      <c r="M9" s="1">
+        <f>COUNTIF(K9:K18,"CS")/6</f>
+        <v/>
+      </c>
+      <c r="N9" s="1">
+        <f>IFERROR(2*(L9*M9)/(L9+M9),"")</f>
+        <v/>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr"/>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>On the permission dialog, tap Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr">
+        <is>
+          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+        </is>
+      </c>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="inlineStr"/>
+      <c r="M10" s="1" t="inlineStr"/>
+      <c r="N10" s="1" t="inlineStr"/>
+      <c r="O10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr"/>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>Open the navigation menu by tapping Navigate up. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
+        </is>
+      </c>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L11" s="1" t="inlineStr"/>
+      <c r="M11" s="1" t="inlineStr"/>
+      <c r="N11" s="1" t="inlineStr"/>
+      <c r="O11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr"/>
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="1" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr"/>
+      <c r="F12" s="1" t="inlineStr"/>
+      <c r="G12" s="1" t="inlineStr"/>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="inlineStr"/>
+      <c r="M12" s="1" t="inlineStr"/>
+      <c r="N12" s="1" t="inlineStr"/>
+      <c r="O12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr"/>
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr"/>
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>Tap the FTP server status switch while it is OFF to turn it ON. &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L13" s="1" t="inlineStr"/>
+      <c r="M13" s="1" t="inlineStr"/>
+      <c r="N13" s="1" t="inlineStr"/>
+      <c r="O13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr"/>
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr"/>
+      <c r="E14" s="1" t="inlineStr"/>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Tap the FTP server status switch while it is ON to turn it OFF. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="inlineStr"/>
+      <c r="M14" s="1" t="inlineStr"/>
+      <c r="N14" s="1" t="inlineStr"/>
+      <c r="O14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr"/>
+      <c r="B15" s="1" t="inlineStr"/>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr"/>
+      <c r="E15" s="1" t="inlineStr"/>
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>Leave the FTP server screen by tapping Navigate up. &lt;f5deb5a7a067fcecd183ba802aa26e2dfb3c5e38306d9407fd3b178866210afb&gt;</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="J8" s="1" t="inlineStr"/>
-      <c r="K8" s="1" t="inlineStr">
+      <c r="J15" s="1" t="inlineStr"/>
+      <c r="K15" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="L8" s="1" t="inlineStr"/>
-      <c r="M8" s="1" t="inlineStr"/>
-      <c r="N8" s="1" t="inlineStr"/>
-      <c r="O8" s="1" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr"/>
-      <c r="B9" s="1" t="inlineStr"/>
-      <c r="C9" s="1" t="inlineStr"/>
-      <c r="D9" s="1" t="inlineStr"/>
-      <c r="E9" s="1" t="inlineStr"/>
-      <c r="F9" s="1" t="inlineStr"/>
-      <c r="G9" s="1" t="inlineStr"/>
-      <c r="H9" s="1" t="inlineStr">
-        <is>
-          <t>In the Recents screen, dismiss the Files app.</t>
-        </is>
-      </c>
-      <c r="I9" s="1" t="inlineStr">
+      <c r="L15" s="1" t="inlineStr"/>
+      <c r="M15" s="1" t="inlineStr"/>
+      <c r="N15" s="1" t="inlineStr"/>
+      <c r="O15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr"/>
+      <c r="E16" s="1" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Tap the list item to return to the FTP server screen path context. &lt;6766d1c12b54808176b7d8e110b78ee25e2843492f806acedcc0d8e1da70972c&gt;</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="J9" s="1" t="inlineStr"/>
-      <c r="K9" s="1" t="inlineStr">
+      <c r="J16" s="1" t="inlineStr"/>
+      <c r="K16" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="L9" s="1" t="inlineStr"/>
-      <c r="M9" s="1" t="inlineStr"/>
-      <c r="N9" s="1" t="inlineStr"/>
-      <c r="O9" s="1" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr"/>
-      <c r="B10" s="2" t="inlineStr"/>
-      <c r="C10" s="2" t="inlineStr"/>
-      <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
-      <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
-      <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
-      <c r="L10" s="2" t="inlineStr"/>
-      <c r="M10" s="2" t="inlineStr"/>
-      <c r="N10" s="2" t="inlineStr"/>
-      <c r="O10" s="2" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="n">
+      <c r="L16" s="1" t="inlineStr"/>
+      <c r="M16" s="1" t="inlineStr"/>
+      <c r="N16" s="1" t="inlineStr"/>
+      <c r="O16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr"/>
+      <c r="B17" s="1" t="inlineStr"/>
+      <c r="C17" s="1" t="inlineStr"/>
+      <c r="D17" s="1" t="inlineStr"/>
+      <c r="E17" s="1" t="inlineStr"/>
+      <c r="F17" s="1" t="inlineStr"/>
+      <c r="G17" s="1" t="inlineStr"/>
+      <c r="H17" s="1" t="inlineStr">
+        <is>
+          <t>Open Recents using the system Back/Recents control. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
+        </is>
+      </c>
+      <c r="I17" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J17" s="1" t="inlineStr"/>
+      <c r="K17" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L17" s="1" t="inlineStr"/>
+      <c r="M17" s="1" t="inlineStr"/>
+      <c r="N17" s="1" t="inlineStr"/>
+      <c r="O17" s="1" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr"/>
+      <c r="B18" s="1" t="inlineStr"/>
+      <c r="C18" s="1" t="inlineStr"/>
+      <c r="D18" s="1" t="inlineStr"/>
+      <c r="E18" s="1" t="inlineStr"/>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr"/>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>Dismiss the Files app task from Recents. &lt;b05234dc13810ef197b494fe9ce3b3d6e6927d53c722ad904f3dc53e425da84c&gt;</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr"/>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L18" s="1" t="inlineStr"/>
+      <c r="M18" s="1" t="inlineStr"/>
+      <c r="N18" s="1" t="inlineStr"/>
+      <c r="O18" s="1" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr"/>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="B11" s="1" t="inlineStr">
+      <c r="B20" s="1" t="inlineStr">
         <is>
           <t>Wikimedia Commons</t>
         </is>
       </c>
-      <c r="C11" s="1" t="inlineStr">
+      <c r="C20" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D11" s="1" t="inlineStr">
-        <is>
-          <t>HC_HP</t>
-        </is>
-      </c>
-      <c r="E11" s="1" t="inlineStr">
-        <is>
-          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F11" s="1" t="inlineStr">
-        <is>
-          <t>Title: Parent Categories tab opens a blank page on the category details screen
-Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the Parent Categories tab, the page is blank.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="G11" s="1" t="inlineStr">
+      <c r="D20" s="1" t="inlineStr">
+        <is>
+          <t>LC_HP</t>
+        </is>
+      </c>
+      <c r="E20" s="1" t="inlineStr">
+        <is>
+          <t>The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F20" s="1" t="inlineStr">
+        <is>
+          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
+Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
+Expected Behavior: The parent categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
 2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
@@ -888,338 +1201,41 @@
 15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
-      <c r="H11" s="1" t="inlineStr">
+      <c r="H20" s="1" t="inlineStr">
         <is>
           <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="I11" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J11" s="1" t="inlineStr">
+      <c r="I20" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J20" s="1" t="inlineStr">
         <is>
           <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="K11" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L11" s="1">
-        <f>IFERROR(COUNTIF(K11:K25,"CS")/COUNTA(K11:K25),"")</f>
+      <c r="K20" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L20" s="1">
+        <f>IFERROR(COUNTIF(K20:K34,"CS")/COUNTA(K20:K34),"")</f>
         <v/>
       </c>
-      <c r="M11" s="1">
-        <f>COUNTIF(K11:K25,"CS")/15</f>
+      <c r="M20" s="1">
+        <f>COUNTIF(K20:K34,"CS")/15</f>
         <v/>
       </c>
-      <c r="N11" s="1">
-        <f>IFERROR(2*(L11*M11)/(L11+M11),"")</f>
+      <c r="N20" s="1">
+        <f>IFERROR(2*(L20*M20)/(L20+M20),"")</f>
         <v/>
       </c>
-      <c r="O11" s="1" t="n">
+      <c r="O20" s="1" t="n">
         <v>15</v>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr"/>
-      <c r="B12" s="1" t="inlineStr"/>
-      <c r="C12" s="1" t="inlineStr"/>
-      <c r="D12" s="1" t="inlineStr"/>
-      <c r="E12" s="1" t="inlineStr"/>
-      <c r="F12" s="1" t="inlineStr"/>
-      <c r="G12" s="1" t="inlineStr"/>
-      <c r="H12" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="I12" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="K12" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L12" s="1" t="inlineStr"/>
-      <c r="M12" s="1" t="inlineStr"/>
-      <c r="N12" s="1" t="inlineStr"/>
-      <c r="O12" s="1" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr"/>
-      <c r="B13" s="1" t="inlineStr"/>
-      <c r="C13" s="1" t="inlineStr"/>
-      <c r="D13" s="1" t="inlineStr"/>
-      <c r="E13" s="1" t="inlineStr"/>
-      <c r="F13" s="1" t="inlineStr"/>
-      <c r="G13" s="1" t="inlineStr"/>
-      <c r="H13" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="I13" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J13" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="K13" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L13" s="1" t="inlineStr"/>
-      <c r="M13" s="1" t="inlineStr"/>
-      <c r="N13" s="1" t="inlineStr"/>
-      <c r="O13" s="1" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr"/>
-      <c r="B14" s="1" t="inlineStr"/>
-      <c r="C14" s="1" t="inlineStr"/>
-      <c r="D14" s="1" t="inlineStr"/>
-      <c r="E14" s="1" t="inlineStr"/>
-      <c r="F14" s="1" t="inlineStr"/>
-      <c r="G14" s="1" t="inlineStr"/>
-      <c r="H14" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="I14" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J14" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="K14" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L14" s="1" t="inlineStr"/>
-      <c r="M14" s="1" t="inlineStr"/>
-      <c r="N14" s="1" t="inlineStr"/>
-      <c r="O14" s="1" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr"/>
-      <c r="B15" s="1" t="inlineStr"/>
-      <c r="C15" s="1" t="inlineStr"/>
-      <c r="D15" s="1" t="inlineStr"/>
-      <c r="E15" s="1" t="inlineStr"/>
-      <c r="F15" s="1" t="inlineStr"/>
-      <c r="G15" s="1" t="inlineStr"/>
-      <c r="H15" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="I15" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J15" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="K15" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L15" s="1" t="inlineStr"/>
-      <c r="M15" s="1" t="inlineStr"/>
-      <c r="N15" s="1" t="inlineStr"/>
-      <c r="O15" s="1" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr"/>
-      <c r="B16" s="1" t="inlineStr"/>
-      <c r="C16" s="1" t="inlineStr"/>
-      <c r="D16" s="1" t="inlineStr"/>
-      <c r="E16" s="1" t="inlineStr"/>
-      <c r="F16" s="1" t="inlineStr"/>
-      <c r="G16" s="1" t="inlineStr"/>
-      <c r="H16" s="1" t="inlineStr">
-        <is>
-          <t>Tap "YES!" on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="I16" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="K16" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L16" s="1" t="inlineStr"/>
-      <c r="M16" s="1" t="inlineStr"/>
-      <c r="N16" s="1" t="inlineStr"/>
-      <c r="O16" s="1" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr"/>
-      <c r="B17" s="1" t="inlineStr"/>
-      <c r="C17" s="1" t="inlineStr"/>
-      <c r="D17" s="1" t="inlineStr"/>
-      <c r="E17" s="1" t="inlineStr"/>
-      <c r="F17" s="1" t="inlineStr"/>
-      <c r="G17" s="1" t="inlineStr"/>
-      <c r="H17" s="1" t="inlineStr">
-        <is>
-          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="I17" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J17" s="1" t="inlineStr">
-        <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="K17" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L17" s="1" t="inlineStr"/>
-      <c r="M17" s="1" t="inlineStr"/>
-      <c r="N17" s="1" t="inlineStr"/>
-      <c r="O17" s="1" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr"/>
-      <c r="B18" s="1" t="inlineStr"/>
-      <c r="C18" s="1" t="inlineStr"/>
-      <c r="D18" s="1" t="inlineStr"/>
-      <c r="E18" s="1" t="inlineStr"/>
-      <c r="F18" s="1" t="inlineStr"/>
-      <c r="G18" s="1" t="inlineStr"/>
-      <c r="H18" s="1" t="inlineStr">
-        <is>
-          <t>Tap "YES" on the skip login confirmation dialog. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="I18" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J18" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="K18" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L18" s="1" t="inlineStr"/>
-      <c r="M18" s="1" t="inlineStr"/>
-      <c r="N18" s="1" t="inlineStr"/>
-      <c r="O18" s="1" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr"/>
-      <c r="B19" s="1" t="inlineStr"/>
-      <c r="C19" s="1" t="inlineStr"/>
-      <c r="D19" s="1" t="inlineStr"/>
-      <c r="E19" s="1" t="inlineStr"/>
-      <c r="F19" s="1" t="inlineStr"/>
-      <c r="G19" s="1" t="inlineStr"/>
-      <c r="H19" s="1" t="inlineStr">
-        <is>
-          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
-        </is>
-      </c>
-      <c r="I19" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J19" s="1" t="inlineStr">
-        <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
-        </is>
-      </c>
-      <c r="K19" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L19" s="1" t="inlineStr"/>
-      <c r="M19" s="1" t="inlineStr"/>
-      <c r="N19" s="1" t="inlineStr"/>
-      <c r="O19" s="1" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="inlineStr"/>
-      <c r="B20" s="1" t="inlineStr"/>
-      <c r="C20" s="1" t="inlineStr"/>
-      <c r="D20" s="1" t="inlineStr"/>
-      <c r="E20" s="1" t="inlineStr"/>
-      <c r="F20" s="1" t="inlineStr"/>
-      <c r="G20" s="1" t="inlineStr"/>
-      <c r="H20" s="1" t="inlineStr">
-        <is>
-          <t>Select "Explore" from the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
-        </is>
-      </c>
-      <c r="I20" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J20" s="1" t="inlineStr">
-        <is>
-          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
-        </is>
-      </c>
-      <c r="K20" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L20" s="1" t="inlineStr"/>
-      <c r="M20" s="1" t="inlineStr"/>
-      <c r="N20" s="1" t="inlineStr"/>
-      <c r="O20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr"/>
@@ -1231,7 +1247,7 @@
       <c r="G21" s="1" t="inlineStr"/>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>Tap a picture in the Explore grid to open its media details. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I21" s="1" t="inlineStr">
@@ -1241,7 +1257,7 @@
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K21" s="1" t="inlineStr">
@@ -1264,7 +1280,7 @@
       <c r="G22" s="1" t="inlineStr"/>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I22" s="1" t="inlineStr">
@@ -1274,7 +1290,7 @@
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
@@ -1297,7 +1313,7 @@
       <c r="G23" s="1" t="inlineStr"/>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
@@ -1307,7 +1323,7 @@
       </c>
       <c r="J23" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K23" s="1" t="inlineStr">
@@ -1330,7 +1346,7 @@
       <c r="G24" s="1" t="inlineStr"/>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>Tap a category from the media details categories list. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I24" s="1" t="inlineStr">
@@ -1340,7 +1356,7 @@
       </c>
       <c r="J24" s="1" t="inlineStr">
         <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K24" s="1" t="inlineStr">
@@ -1363,7 +1379,7 @@
       <c r="G25" s="1" t="inlineStr"/>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I25" s="1" t="inlineStr">
@@ -1373,7 +1389,7 @@
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
@@ -1387,68 +1403,49 @@
       <c r="O25" s="1" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-      <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr"/>
+      <c r="A26" s="1" t="inlineStr"/>
+      <c r="B26" s="1" t="inlineStr"/>
+      <c r="C26" s="1" t="inlineStr"/>
+      <c r="D26" s="1" t="inlineStr"/>
+      <c r="E26" s="1" t="inlineStr"/>
+      <c r="F26" s="1" t="inlineStr"/>
+      <c r="G26" s="1" t="inlineStr"/>
+      <c r="H26" s="1" t="inlineStr">
+        <is>
+          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="I26" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J26" s="1" t="inlineStr">
+        <is>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="K26" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L26" s="1" t="inlineStr"/>
+      <c r="M26" s="1" t="inlineStr"/>
+      <c r="N26" s="1" t="inlineStr"/>
+      <c r="O26" s="1" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B27" s="1" t="inlineStr">
-        <is>
-          <t>Family Finance</t>
-        </is>
-      </c>
-      <c r="C27" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D27" s="1" t="inlineStr">
-        <is>
-          <t>HC_HP</t>
-        </is>
-      </c>
-      <c r="E27" s="1" t="inlineStr">
-        <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
-        </is>
-      </c>
-      <c r="F27" s="1" t="inlineStr">
-        <is>
-          <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
-Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
-Expected Behavior: The appearance of the report should be changed to use percent values.</t>
-        </is>
-      </c>
-      <c r="G27" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
+      <c r="A27" s="1" t="inlineStr"/>
+      <c r="B27" s="1" t="inlineStr"/>
+      <c r="C27" s="1" t="inlineStr"/>
+      <c r="D27" s="1" t="inlineStr"/>
+      <c r="E27" s="1" t="inlineStr"/>
+      <c r="F27" s="1" t="inlineStr"/>
+      <c r="G27" s="1" t="inlineStr"/>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
@@ -1458,7 +1455,7 @@
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="K27" s="1" t="inlineStr">
@@ -1466,21 +1463,10 @@
           <t>CS</t>
         </is>
       </c>
-      <c r="L27" s="1">
-        <f>IFERROR(COUNTIF(K27:K35,"CS")/COUNTA(K27:K35),"")</f>
-        <v/>
-      </c>
-      <c r="M27" s="1">
-        <f>COUNTIF(K27:K35,"CS")/8</f>
-        <v/>
-      </c>
-      <c r="N27" s="1">
-        <f>IFERROR(2*(L27*M27)/(L27+M27),"")</f>
-        <v/>
-      </c>
-      <c r="O27" s="1" t="n">
-        <v>8</v>
-      </c>
+      <c r="L27" s="1" t="inlineStr"/>
+      <c r="M27" s="1" t="inlineStr"/>
+      <c r="N27" s="1" t="inlineStr"/>
+      <c r="O27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr"/>
@@ -1492,22 +1478,18 @@
       <c r="G28" s="1" t="inlineStr"/>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
         </is>
       </c>
       <c r="I28" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J28" s="1" t="inlineStr">
-        <is>
-          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr"/>
       <c r="K28" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L28" s="1" t="inlineStr"/>
@@ -1525,7 +1507,7 @@
       <c r="G29" s="1" t="inlineStr"/>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -1535,7 +1517,7 @@
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="K29" s="1" t="inlineStr">
@@ -1558,7 +1540,7 @@
       <c r="G30" s="1" t="inlineStr"/>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>Open the Incomes by Articles tab. &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I30" s="1" t="inlineStr">
@@ -1568,7 +1550,7 @@
       </c>
       <c r="J30" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="K30" s="1" t="inlineStr">
@@ -1591,7 +1573,7 @@
       <c r="G31" s="1" t="inlineStr"/>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>Tap Display. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I31" s="1" t="inlineStr">
@@ -1601,7 +1583,7 @@
       </c>
       <c r="J31" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="K31" s="1" t="inlineStr">
@@ -1624,7 +1606,7 @@
       <c r="G32" s="1" t="inlineStr"/>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>Check View values. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I32" s="1" t="inlineStr">
@@ -1634,7 +1616,7 @@
       </c>
       <c r="J32" s="1" t="inlineStr">
         <is>
-          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="K32" s="1" t="inlineStr">
@@ -1657,7 +1639,7 @@
       <c r="G33" s="1" t="inlineStr"/>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>Check Use percent values. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="I33" s="1" t="inlineStr">
@@ -1667,7 +1649,7 @@
       </c>
       <c r="J33" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="K33" s="1" t="inlineStr">
@@ -1690,22 +1672,18 @@
       <c r="G34" s="1" t="inlineStr"/>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>Tap OK. &lt;ef26a526444b0c0827ef99ce6360670c18cb2ac563b206cf97bd84c9479fa5f6&gt;</t>
+          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
         </is>
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J34" s="1" t="inlineStr">
-        <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr"/>
       <c r="K34" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L34" s="1" t="inlineStr"/>
@@ -1714,33 +1692,1211 @@
       <c r="O34" s="1" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr"/>
-      <c r="B35" s="1" t="inlineStr"/>
-      <c r="C35" s="1" t="inlineStr"/>
-      <c r="D35" s="1" t="inlineStr"/>
-      <c r="E35" s="1" t="inlineStr"/>
-      <c r="F35" s="1" t="inlineStr"/>
-      <c r="G35" s="1" t="inlineStr"/>
-      <c r="H35" s="1" t="inlineStr">
-        <is>
-          <t>If a crash dialog appears, tap OK. &lt;6aa06c426f17d83ac768c98cc6d31a987166d855462845d0b306e83f26fa76f9&gt;</t>
-        </is>
-      </c>
-      <c r="I35" s="1" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr"/>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr"/>
+      <c r="J35" s="2" t="inlineStr"/>
+      <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr"/>
+      <c r="M35" s="2" t="inlineStr"/>
+      <c r="N35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B36" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C36" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D36" s="1" t="inlineStr">
+        <is>
+          <t>MC_HP</t>
+        </is>
+      </c>
+      <c r="E36" s="1" t="inlineStr">
+        <is>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F36" s="1" t="inlineStr">
+        <is>
+          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
+Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="G36" s="1" t="inlineStr">
+        <is>
+          <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
+2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
+3. Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;
+4. Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;
+5. Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;
+6. Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;
+7. Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;
+8. Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;
+9. Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;
+10. Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;
+11. Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;
+12. Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;
+13. Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;
+14. Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;
+15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="inlineStr">
+        <is>
+          <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L36" s="1">
+        <f>IFERROR(COUNTIF(K36:K51,"CS")/COUNTA(K36:K51),"")</f>
+        <v/>
+      </c>
+      <c r="M36" s="1">
+        <f>COUNTIF(K36:K51,"CS")/15</f>
+        <v/>
+      </c>
+      <c r="N36" s="1">
+        <f>IFERROR(2*(L36*M36)/(L36+M36),"")</f>
+        <v/>
+      </c>
+      <c r="O36" s="1" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr"/>
+      <c r="B37" s="1" t="inlineStr"/>
+      <c r="C37" s="1" t="inlineStr"/>
+      <c r="D37" s="1" t="inlineStr"/>
+      <c r="E37" s="1" t="inlineStr"/>
+      <c r="F37" s="1" t="inlineStr"/>
+      <c r="G37" s="1" t="inlineStr"/>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+        </is>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L37" s="1" t="inlineStr"/>
+      <c r="M37" s="1" t="inlineStr"/>
+      <c r="N37" s="1" t="inlineStr"/>
+      <c r="O37" s="1" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr"/>
+      <c r="B38" s="1" t="inlineStr"/>
+      <c r="C38" s="1" t="inlineStr"/>
+      <c r="D38" s="1" t="inlineStr"/>
+      <c r="E38" s="1" t="inlineStr"/>
+      <c r="F38" s="1" t="inlineStr"/>
+      <c r="G38" s="1" t="inlineStr"/>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L38" s="1" t="inlineStr"/>
+      <c r="M38" s="1" t="inlineStr"/>
+      <c r="N38" s="1" t="inlineStr"/>
+      <c r="O38" s="1" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr"/>
+      <c r="B39" s="1" t="inlineStr"/>
+      <c r="C39" s="1" t="inlineStr"/>
+      <c r="D39" s="1" t="inlineStr"/>
+      <c r="E39" s="1" t="inlineStr"/>
+      <c r="F39" s="1" t="inlineStr"/>
+      <c r="G39" s="1" t="inlineStr"/>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L39" s="1" t="inlineStr"/>
+      <c r="M39" s="1" t="inlineStr"/>
+      <c r="N39" s="1" t="inlineStr"/>
+      <c r="O39" s="1" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr"/>
+      <c r="B40" s="1" t="inlineStr"/>
+      <c r="C40" s="1" t="inlineStr"/>
+      <c r="D40" s="1" t="inlineStr"/>
+      <c r="E40" s="1" t="inlineStr"/>
+      <c r="F40" s="1" t="inlineStr"/>
+      <c r="G40" s="1" t="inlineStr"/>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+        </is>
+      </c>
+      <c r="K40" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L40" s="1" t="inlineStr"/>
+      <c r="M40" s="1" t="inlineStr"/>
+      <c r="N40" s="1" t="inlineStr"/>
+      <c r="O40" s="1" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr"/>
+      <c r="B41" s="1" t="inlineStr"/>
+      <c r="C41" s="1" t="inlineStr"/>
+      <c r="D41" s="1" t="inlineStr"/>
+      <c r="E41" s="1" t="inlineStr"/>
+      <c r="F41" s="1" t="inlineStr"/>
+      <c r="G41" s="1" t="inlineStr"/>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+        </is>
+      </c>
+      <c r="K41" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L41" s="1" t="inlineStr"/>
+      <c r="M41" s="1" t="inlineStr"/>
+      <c r="N41" s="1" t="inlineStr"/>
+      <c r="O41" s="1" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr"/>
+      <c r="B42" s="1" t="inlineStr"/>
+      <c r="C42" s="1" t="inlineStr"/>
+      <c r="D42" s="1" t="inlineStr"/>
+      <c r="E42" s="1" t="inlineStr"/>
+      <c r="F42" s="1" t="inlineStr"/>
+      <c r="G42" s="1" t="inlineStr"/>
+      <c r="H42" s="1" t="inlineStr">
+        <is>
+          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
+        </is>
+      </c>
+      <c r="I42" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
+      <c r="K42" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L42" s="1" t="inlineStr"/>
+      <c r="M42" s="1" t="inlineStr"/>
+      <c r="N42" s="1" t="inlineStr"/>
+      <c r="O42" s="1" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr"/>
+      <c r="B43" s="1" t="inlineStr"/>
+      <c r="C43" s="1" t="inlineStr"/>
+      <c r="D43" s="1" t="inlineStr"/>
+      <c r="E43" s="1" t="inlineStr"/>
+      <c r="F43" s="1" t="inlineStr"/>
+      <c r="G43" s="1" t="inlineStr"/>
+      <c r="H43" s="1" t="inlineStr">
+        <is>
+          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
+        </is>
+      </c>
+      <c r="I43" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="J35" s="1" t="inlineStr"/>
-      <c r="K35" s="1" t="inlineStr">
+      <c r="J43" s="1" t="inlineStr"/>
+      <c r="K43" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="L35" s="1" t="inlineStr"/>
-      <c r="M35" s="1" t="inlineStr"/>
-      <c r="N35" s="1" t="inlineStr"/>
-      <c r="O35" s="1" t="inlineStr"/>
+      <c r="L43" s="1" t="inlineStr"/>
+      <c r="M43" s="1" t="inlineStr"/>
+      <c r="N43" s="1" t="inlineStr"/>
+      <c r="O43" s="1" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="1" t="inlineStr"/>
+      <c r="B44" s="1" t="inlineStr"/>
+      <c r="C44" s="1" t="inlineStr"/>
+      <c r="D44" s="1" t="inlineStr"/>
+      <c r="E44" s="1" t="inlineStr"/>
+      <c r="F44" s="1" t="inlineStr"/>
+      <c r="G44" s="1" t="inlineStr"/>
+      <c r="H44" s="1" t="inlineStr">
+        <is>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="I44" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr">
+        <is>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="K44" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L44" s="1" t="inlineStr"/>
+      <c r="M44" s="1" t="inlineStr"/>
+      <c r="N44" s="1" t="inlineStr"/>
+      <c r="O44" s="1" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="inlineStr"/>
+      <c r="B45" s="1" t="inlineStr"/>
+      <c r="C45" s="1" t="inlineStr"/>
+      <c r="D45" s="1" t="inlineStr"/>
+      <c r="E45" s="1" t="inlineStr"/>
+      <c r="F45" s="1" t="inlineStr"/>
+      <c r="G45" s="1" t="inlineStr"/>
+      <c r="H45" s="1" t="inlineStr">
+        <is>
+          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="K45" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L45" s="1" t="inlineStr"/>
+      <c r="M45" s="1" t="inlineStr"/>
+      <c r="N45" s="1" t="inlineStr"/>
+      <c r="O45" s="1" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="1" t="inlineStr"/>
+      <c r="B46" s="1" t="inlineStr"/>
+      <c r="C46" s="1" t="inlineStr"/>
+      <c r="D46" s="1" t="inlineStr"/>
+      <c r="E46" s="1" t="inlineStr"/>
+      <c r="F46" s="1" t="inlineStr"/>
+      <c r="G46" s="1" t="inlineStr"/>
+      <c r="H46" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+        </is>
+      </c>
+      <c r="I46" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="inlineStr"/>
+      <c r="K46" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L46" s="1" t="inlineStr"/>
+      <c r="M46" s="1" t="inlineStr"/>
+      <c r="N46" s="1" t="inlineStr"/>
+      <c r="O46" s="1" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="1" t="inlineStr"/>
+      <c r="B47" s="1" t="inlineStr"/>
+      <c r="C47" s="1" t="inlineStr"/>
+      <c r="D47" s="1" t="inlineStr"/>
+      <c r="E47" s="1" t="inlineStr"/>
+      <c r="F47" s="1" t="inlineStr"/>
+      <c r="G47" s="1" t="inlineStr"/>
+      <c r="H47" s="1" t="inlineStr">
+        <is>
+          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="I47" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J47" s="1" t="inlineStr">
+        <is>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="K47" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L47" s="1" t="inlineStr"/>
+      <c r="M47" s="1" t="inlineStr"/>
+      <c r="N47" s="1" t="inlineStr"/>
+      <c r="O47" s="1" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="1" t="inlineStr"/>
+      <c r="B48" s="1" t="inlineStr"/>
+      <c r="C48" s="1" t="inlineStr"/>
+      <c r="D48" s="1" t="inlineStr"/>
+      <c r="E48" s="1" t="inlineStr"/>
+      <c r="F48" s="1" t="inlineStr"/>
+      <c r="G48" s="1" t="inlineStr"/>
+      <c r="H48" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="I48" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J48" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="K48" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L48" s="1" t="inlineStr"/>
+      <c r="M48" s="1" t="inlineStr"/>
+      <c r="N48" s="1" t="inlineStr"/>
+      <c r="O48" s="1" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="1" t="inlineStr"/>
+      <c r="B49" s="1" t="inlineStr"/>
+      <c r="C49" s="1" t="inlineStr"/>
+      <c r="D49" s="1" t="inlineStr"/>
+      <c r="E49" s="1" t="inlineStr"/>
+      <c r="F49" s="1" t="inlineStr"/>
+      <c r="G49" s="1" t="inlineStr"/>
+      <c r="H49" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="I49" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J49" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="K49" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L49" s="1" t="inlineStr"/>
+      <c r="M49" s="1" t="inlineStr"/>
+      <c r="N49" s="1" t="inlineStr"/>
+      <c r="O49" s="1" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="1" t="inlineStr"/>
+      <c r="B50" s="1" t="inlineStr"/>
+      <c r="C50" s="1" t="inlineStr"/>
+      <c r="D50" s="1" t="inlineStr"/>
+      <c r="E50" s="1" t="inlineStr"/>
+      <c r="F50" s="1" t="inlineStr"/>
+      <c r="G50" s="1" t="inlineStr"/>
+      <c r="H50" s="1" t="inlineStr">
+        <is>
+          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="I50" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="K50" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L50" s="1" t="inlineStr"/>
+      <c r="M50" s="1" t="inlineStr"/>
+      <c r="N50" s="1" t="inlineStr"/>
+      <c r="O50" s="1" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="1" t="inlineStr"/>
+      <c r="B51" s="1" t="inlineStr"/>
+      <c r="C51" s="1" t="inlineStr"/>
+      <c r="D51" s="1" t="inlineStr"/>
+      <c r="E51" s="1" t="inlineStr"/>
+      <c r="F51" s="1" t="inlineStr"/>
+      <c r="G51" s="1" t="inlineStr"/>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="inlineStr"/>
+      <c r="M51" s="1" t="inlineStr"/>
+      <c r="N51" s="1" t="inlineStr"/>
+      <c r="O51" s="1" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr"/>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr"/>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr"/>
+      <c r="M52" s="2" t="inlineStr"/>
+      <c r="N52" s="2" t="inlineStr"/>
+      <c r="O52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B53" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D53" s="1" t="inlineStr">
+        <is>
+          <t>HC_HP</t>
+        </is>
+      </c>
+      <c r="E53" s="1" t="inlineStr">
+        <is>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F53" s="1" t="inlineStr">
+        <is>
+          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
+Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
+Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
+      <c r="G53" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L53" s="1">
+        <f>IFERROR(COUNTIF(K53:K60,"CS")/COUNTA(K53:K60),"")</f>
+        <v/>
+      </c>
+      <c r="M53" s="1">
+        <f>COUNTIF(K53:K60,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N53" s="1">
+        <f>IFERROR(2*(L53*M53)/(L53+M53),"")</f>
+        <v/>
+      </c>
+      <c r="O53" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="inlineStr"/>
+      <c r="B54" s="1" t="inlineStr"/>
+      <c r="C54" s="1" t="inlineStr"/>
+      <c r="D54" s="1" t="inlineStr"/>
+      <c r="E54" s="1" t="inlineStr"/>
+      <c r="F54" s="1" t="inlineStr"/>
+      <c r="G54" s="1" t="inlineStr"/>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="inlineStr"/>
+      <c r="M54" s="1" t="inlineStr"/>
+      <c r="N54" s="1" t="inlineStr"/>
+      <c r="O54" s="1" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr"/>
+      <c r="B55" s="1" t="inlineStr"/>
+      <c r="C55" s="1" t="inlineStr"/>
+      <c r="D55" s="1" t="inlineStr"/>
+      <c r="E55" s="1" t="inlineStr"/>
+      <c r="F55" s="1" t="inlineStr"/>
+      <c r="G55" s="1" t="inlineStr"/>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="inlineStr"/>
+      <c r="M55" s="1" t="inlineStr"/>
+      <c r="N55" s="1" t="inlineStr"/>
+      <c r="O55" s="1" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr"/>
+      <c r="B56" s="1" t="inlineStr"/>
+      <c r="C56" s="1" t="inlineStr"/>
+      <c r="D56" s="1" t="inlineStr"/>
+      <c r="E56" s="1" t="inlineStr"/>
+      <c r="F56" s="1" t="inlineStr"/>
+      <c r="G56" s="1" t="inlineStr"/>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J56" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L56" s="1" t="inlineStr"/>
+      <c r="M56" s="1" t="inlineStr"/>
+      <c r="N56" s="1" t="inlineStr"/>
+      <c r="O56" s="1" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr"/>
+      <c r="B57" s="1" t="inlineStr"/>
+      <c r="C57" s="1" t="inlineStr"/>
+      <c r="D57" s="1" t="inlineStr"/>
+      <c r="E57" s="1" t="inlineStr"/>
+      <c r="F57" s="1" t="inlineStr"/>
+      <c r="G57" s="1" t="inlineStr"/>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J57" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L57" s="1" t="inlineStr"/>
+      <c r="M57" s="1" t="inlineStr"/>
+      <c r="N57" s="1" t="inlineStr"/>
+      <c r="O57" s="1" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr"/>
+      <c r="B58" s="1" t="inlineStr"/>
+      <c r="C58" s="1" t="inlineStr"/>
+      <c r="D58" s="1" t="inlineStr"/>
+      <c r="E58" s="1" t="inlineStr"/>
+      <c r="F58" s="1" t="inlineStr"/>
+      <c r="G58" s="1" t="inlineStr"/>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J58" s="1" t="inlineStr">
+        <is>
+          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L58" s="1" t="inlineStr"/>
+      <c r="M58" s="1" t="inlineStr"/>
+      <c r="N58" s="1" t="inlineStr"/>
+      <c r="O58" s="1" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr"/>
+      <c r="B59" s="1" t="inlineStr"/>
+      <c r="C59" s="1" t="inlineStr"/>
+      <c r="D59" s="1" t="inlineStr"/>
+      <c r="E59" s="1" t="inlineStr"/>
+      <c r="F59" s="1" t="inlineStr"/>
+      <c r="G59" s="1" t="inlineStr"/>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J59" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L59" s="1" t="inlineStr"/>
+      <c r="M59" s="1" t="inlineStr"/>
+      <c r="N59" s="1" t="inlineStr"/>
+      <c r="O59" s="1" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr"/>
+      <c r="B60" s="1" t="inlineStr"/>
+      <c r="C60" s="1" t="inlineStr"/>
+      <c r="D60" s="1" t="inlineStr"/>
+      <c r="E60" s="1" t="inlineStr"/>
+      <c r="F60" s="1" t="inlineStr"/>
+      <c r="G60" s="1" t="inlineStr"/>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I60" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J60" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L60" s="1" t="inlineStr"/>
+      <c r="M60" s="1" t="inlineStr"/>
+      <c r="N60" s="1" t="inlineStr"/>
+      <c r="O60" s="1" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="inlineStr"/>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr"/>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr"/>
+      <c r="M61" s="2" t="inlineStr"/>
+      <c r="N61" s="2" t="inlineStr"/>
+      <c r="O61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B62" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C62" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D62" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E62" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F62" s="1" t="inlineStr">
+        <is>
+          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
+Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
+Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
+        </is>
+      </c>
+      <c r="G62" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H62" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+        </is>
+      </c>
+      <c r="I62" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J62" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K62" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L62" s="1">
+        <f>IFERROR(COUNTIF(K62:K68,"CS")/COUNTA(K62:K68),"")</f>
+        <v/>
+      </c>
+      <c r="M62" s="1">
+        <f>COUNTIF(K62:K68,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N62" s="1">
+        <f>IFERROR(2*(L62*M62)/(L62+M62),"")</f>
+        <v/>
+      </c>
+      <c r="O62" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="inlineStr"/>
+      <c r="B63" s="1" t="inlineStr"/>
+      <c r="C63" s="1" t="inlineStr"/>
+      <c r="D63" s="1" t="inlineStr"/>
+      <c r="E63" s="1" t="inlineStr"/>
+      <c r="F63" s="1" t="inlineStr"/>
+      <c r="G63" s="1" t="inlineStr"/>
+      <c r="H63" s="1" t="inlineStr">
+        <is>
+          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+        </is>
+      </c>
+      <c r="I63" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="inlineStr"/>
+      <c r="K63" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L63" s="1" t="inlineStr"/>
+      <c r="M63" s="1" t="inlineStr"/>
+      <c r="N63" s="1" t="inlineStr"/>
+      <c r="O63" s="1" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="1" t="inlineStr"/>
+      <c r="B64" s="1" t="inlineStr"/>
+      <c r="C64" s="1" t="inlineStr"/>
+      <c r="D64" s="1" t="inlineStr"/>
+      <c r="E64" s="1" t="inlineStr"/>
+      <c r="F64" s="1" t="inlineStr"/>
+      <c r="G64" s="1" t="inlineStr"/>
+      <c r="H64" s="1" t="inlineStr">
+        <is>
+          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I64" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J64" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K64" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L64" s="1" t="inlineStr"/>
+      <c r="M64" s="1" t="inlineStr"/>
+      <c r="N64" s="1" t="inlineStr"/>
+      <c r="O64" s="1" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="1" t="inlineStr"/>
+      <c r="B65" s="1" t="inlineStr"/>
+      <c r="C65" s="1" t="inlineStr"/>
+      <c r="D65" s="1" t="inlineStr"/>
+      <c r="E65" s="1" t="inlineStr"/>
+      <c r="F65" s="1" t="inlineStr"/>
+      <c r="G65" s="1" t="inlineStr"/>
+      <c r="H65" s="1" t="inlineStr">
+        <is>
+          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="I65" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J65" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K65" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L65" s="1" t="inlineStr"/>
+      <c r="M65" s="1" t="inlineStr"/>
+      <c r="N65" s="1" t="inlineStr"/>
+      <c r="O65" s="1" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="1" t="inlineStr"/>
+      <c r="B66" s="1" t="inlineStr"/>
+      <c r="C66" s="1" t="inlineStr"/>
+      <c r="D66" s="1" t="inlineStr"/>
+      <c r="E66" s="1" t="inlineStr"/>
+      <c r="F66" s="1" t="inlineStr"/>
+      <c r="G66" s="1" t="inlineStr"/>
+      <c r="H66" s="1" t="inlineStr">
+        <is>
+          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I66" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J66" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K66" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L66" s="1" t="inlineStr"/>
+      <c r="M66" s="1" t="inlineStr"/>
+      <c r="N66" s="1" t="inlineStr"/>
+      <c r="O66" s="1" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="1" t="inlineStr"/>
+      <c r="B67" s="1" t="inlineStr"/>
+      <c r="C67" s="1" t="inlineStr"/>
+      <c r="D67" s="1" t="inlineStr"/>
+      <c r="E67" s="1" t="inlineStr"/>
+      <c r="F67" s="1" t="inlineStr"/>
+      <c r="G67" s="1" t="inlineStr"/>
+      <c r="H67" s="1" t="inlineStr">
+        <is>
+          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I67" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J67" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K67" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L67" s="1" t="inlineStr"/>
+      <c r="M67" s="1" t="inlineStr"/>
+      <c r="N67" s="1" t="inlineStr"/>
+      <c r="O67" s="1" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="1" t="inlineStr"/>
+      <c r="B68" s="1" t="inlineStr"/>
+      <c r="C68" s="1" t="inlineStr"/>
+      <c r="D68" s="1" t="inlineStr"/>
+      <c r="E68" s="1" t="inlineStr"/>
+      <c r="F68" s="1" t="inlineStr"/>
+      <c r="G68" s="1" t="inlineStr"/>
+      <c r="H68" s="1" t="inlineStr">
+        <is>
+          <t>Tap "OK" to confirm the change. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I68" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J68" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K68" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L68" s="1" t="inlineStr"/>
+      <c r="M68" s="1" t="inlineStr"/>
+      <c r="N68" s="1" t="inlineStr"/>
+      <c r="O68" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1753,7 +2909,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1848,19 +3004,19 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>LC_LP</t>
+          <t>HC_LP</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>It restarts on its own.</t>
+          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Title: FTP server restarts on its own after being toggled and the app is dismissed from Recents
-Observed Behavior: On the FTP server screen, if the user turns the FTP server on, turns it off, presses Back to leave the app, and dismisses the Files app from the Recents screen, the FTP server restarts on its own.
-Expected Behavior: The FTP server should not restart on its own.</t>
+          <t>Title: FTP server restarts automatically after being stopped and the app is closed
+Observed Behavior: On the FTP server screen, if the user turns off the FTP server switch and then closes the app, the FTP server restarts automatically after stopping it and closing the app.
+Expected Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
@@ -1873,10 +3029,10 @@
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the FTP server restarts on its own
-Triggering GUI Interactions: turns the FTP server on, turns it off, presses Back to leave the app, and dismisses the Files app from the Recents screen
+          <t>Buggy Behavior: the FTP server restarts automatically after stopping it and closing the app
+Triggering GUI Interactions: the user turns off the FTP server switch and then closes the app
 Triggering Screen Reference: On the FTP server screen
-Correct Behavior: The FTP server should not restart on its own.</t>
+Correct Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
@@ -1886,7 +3042,7 @@
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Incorrect</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
@@ -1916,11 +3072,11 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>135</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Wikimedia Commons</t>
+          <t>Material Files</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -1930,35 +3086,35 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>HC_HP</t>
+          <t>LC_LP</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+          <t>It restarts on its own.</t>
         </is>
       </c>
       <c r="F4" s="1" t="inlineStr">
         <is>
-          <t>Title: Parent Categories tab opens a blank page on the category details screen
-Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the Parent Categories tab, the page is blank.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Title: FTP server restarts automatically after being turned off and leaving the FTP server screen
+Observed Behavior: On the FTP server screen, if the user turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents, the FTP server is restarting on its own.
+Expected Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
         </is>
       </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: see a blank page
-Triggering GUI Interaction: clicks the Parent Categories tab
-Triggering Screen Reference: Category screen, Parent Categories tab
-Correct Behavior: The Parent Categories of the current category should be displayed</t>
+          <t>Buggy Behavior: the server restarts automatically
+Triggering GUI Interaction: stops the FTP server and then closes the app
+Triggering Screen Reference: FTP server screen
+Correct Behavior: The FTP server should remain stopped</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the page is blank
-Triggering GUI Interactions: taps the Parent Categories tab
-Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
-Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: the FTP server is restarting on its own
+Triggering GUI Interactions: turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents
+Triggering Screen Reference: On the FTP server screen
+Correct Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -1998,36 +3154,200 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B6" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C6" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D6" s="1" t="inlineStr">
+        <is>
+          <t>LC_HP</t>
+        </is>
+      </c>
+      <c r="E6" s="1" t="inlineStr">
+        <is>
+          <t>The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr">
+        <is>
+          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
+Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
+Expected Behavior: The parent categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="G6" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
+        </is>
+      </c>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the parent categories of the current category are not displayed
+Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
+Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
+Correct Behavior: The parent categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B8" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C8" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="inlineStr">
+        <is>
+          <t>MC_HP</t>
+        </is>
+      </c>
+      <c r="E8" s="1" t="inlineStr">
+        <is>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr">
+        <is>
+          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
+Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="G8" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
+        </is>
+      </c>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the app results in a blank page
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>Incomplete</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="1" t="inlineStr">
+      <c r="B10" s="1" t="inlineStr">
         <is>
           <t>Family Finance</t>
         </is>
       </c>
-      <c r="C6" s="1" t="inlineStr">
+      <c r="C10" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D6" s="1" t="inlineStr">
+      <c r="D10" s="1" t="inlineStr">
         <is>
           <t>HC_HP</t>
         </is>
       </c>
-      <c r="E6" s="1" t="inlineStr">
+      <c r="E10" s="1" t="inlineStr">
         <is>
           <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
         </is>
       </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>Title: App crashes when enabling View values and Use percent values for the Incomes by Articles report and tapping OK
-Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks the View values checkbox, checks the Use percent values checkbox, and taps OK, the application crashes.
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
+Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
 Expected Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
-      <c r="G6" s="1" t="inlineStr">
+      <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
 Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
@@ -2035,30 +3355,112 @@
 Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
         </is>
       </c>
-      <c r="H6" s="1" t="inlineStr">
+      <c r="H10" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
-Triggering GUI Interactions: checks the View values checkbox, checks the Use percent values checkbox, and taps OK
-Triggering Screen Reference: On the Display of Incomes by Articles pop-up of the Reports screen
+Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
+Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
 Correct Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
-      <c r="I6" s="1" t="inlineStr">
+      <c r="I10" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="J6" s="1" t="inlineStr">
+      <c r="J10" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="K6" s="1" t="inlineStr">
+      <c r="K10" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="L6" s="1" t="inlineStr">
+      <c r="L10" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C12" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D12" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E12" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr">
+        <is>
+          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
+Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
+Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
+        </is>
+      </c>
+      <c r="G12" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
+Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
+Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+        </is>
+      </c>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interactions: the user taps the "Use percent values" checkbox
+Triggering Screen Reference: On the Display of Incomes by Articles dialog
+Correct Behavior: The application should change the report appearance to use percent values without crashing.</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -2223,13 +3625,13 @@
         <v/>
       </c>
       <c r="M2" t="n">
-        <v>118778.6666666667</v>
+        <v>82577.16666666667</v>
       </c>
       <c r="N2" t="n">
-        <v>149.7703270973331</v>
+        <v>70.47254125000002</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cleaned up burt.py and graph_utils.py documentation and code quality
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O68"/>
+  <dimension ref="A1:O84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1167,19 +1167,19 @@
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>LC_HP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr">
         <is>
-          <t>The Parent Categories of the current category should be displayed.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F20" s="1" t="inlineStr">
         <is>
-          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
-Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
-Expected Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Title: Parent Categories tab shows a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G20" s="1" t="inlineStr">
@@ -1280,7 +1280,7 @@
       <c r="G22" s="1" t="inlineStr"/>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+          <t>Swipe left through the second onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I22" s="1" t="inlineStr">
@@ -1313,7 +1313,7 @@
       <c r="G23" s="1" t="inlineStr"/>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+          <t>Swipe left through the third onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
@@ -1346,7 +1346,7 @@
       <c r="G24" s="1" t="inlineStr"/>
       <c r="H24" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+          <t>Swipe left through the fourth onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I24" s="1" t="inlineStr">
@@ -1379,7 +1379,7 @@
       <c r="G25" s="1" t="inlineStr"/>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Tap YES! on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I25" s="1" t="inlineStr">
@@ -1412,7 +1412,7 @@
       <c r="G26" s="1" t="inlineStr"/>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I26" s="1" t="inlineStr">
@@ -1445,7 +1445,7 @@
       <c r="G27" s="1" t="inlineStr"/>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
@@ -1478,18 +1478,22 @@
       <c r="G28" s="1" t="inlineStr"/>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="I28" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J28" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J28" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
       <c r="K28" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L28" s="1" t="inlineStr"/>
@@ -1507,7 +1511,7 @@
       <c r="G29" s="1" t="inlineStr"/>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Select Explore from the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -1517,7 +1521,7 @@
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
         </is>
       </c>
       <c r="K29" s="1" t="inlineStr">
@@ -1540,7 +1544,7 @@
       <c r="G30" s="1" t="inlineStr"/>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Tap a picture in the Explore grid to open its media details. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I30" s="1" t="inlineStr">
@@ -1550,7 +1554,7 @@
       </c>
       <c r="J30" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="K30" s="1" t="inlineStr">
@@ -1573,7 +1577,7 @@
       <c r="G31" s="1" t="inlineStr"/>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I31" s="1" t="inlineStr">
@@ -1583,7 +1587,7 @@
       </c>
       <c r="J31" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="K31" s="1" t="inlineStr">
@@ -1606,7 +1610,7 @@
       <c r="G32" s="1" t="inlineStr"/>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I32" s="1" t="inlineStr">
@@ -1616,7 +1620,7 @@
       </c>
       <c r="J32" s="1" t="inlineStr">
         <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="K32" s="1" t="inlineStr">
@@ -1639,7 +1643,7 @@
       <c r="G33" s="1" t="inlineStr"/>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Tap a category in the media details screen to open category details. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I33" s="1" t="inlineStr">
@@ -1649,7 +1653,7 @@
       </c>
       <c r="J33" s="1" t="inlineStr">
         <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="K33" s="1" t="inlineStr">
@@ -1672,18 +1676,22 @@
       <c r="G34" s="1" t="inlineStr"/>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
+          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J34" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
       <c r="K34" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L34" s="1" t="inlineStr"/>
@@ -1724,19 +1732,19 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>MC_HP</t>
+          <t>LC_HP</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+          <t>The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
-Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
+Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
+Expected Behavior: The parent categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G36" s="1" t="inlineStr">
@@ -1779,11 +1787,11 @@
         </is>
       </c>
       <c r="L36" s="1">
-        <f>IFERROR(COUNTIF(K36:K51,"CS")/COUNTA(K36:K51),"")</f>
+        <f>IFERROR(COUNTIF(K36:K50,"CS")/COUNTA(K36:K50),"")</f>
         <v/>
       </c>
       <c r="M36" s="1">
-        <f>COUNTIF(K36:K51,"CS")/15</f>
+        <f>COUNTIF(K36:K50,"CS")/15</f>
         <v/>
       </c>
       <c r="N36" s="1">
@@ -1804,7 +1812,7 @@
       <c r="G37" s="1" t="inlineStr"/>
       <c r="H37" s="1" t="inlineStr">
         <is>
-          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I37" s="1" t="inlineStr">
@@ -1837,7 +1845,7 @@
       <c r="G38" s="1" t="inlineStr"/>
       <c r="H38" s="1" t="inlineStr">
         <is>
-          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I38" s="1" t="inlineStr">
@@ -1870,7 +1878,7 @@
       <c r="G39" s="1" t="inlineStr"/>
       <c r="H39" s="1" t="inlineStr">
         <is>
-          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I39" s="1" t="inlineStr">
@@ -1903,7 +1911,7 @@
       <c r="G40" s="1" t="inlineStr"/>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I40" s="1" t="inlineStr">
@@ -1936,7 +1944,7 @@
       <c r="G41" s="1" t="inlineStr"/>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I41" s="1" t="inlineStr">
@@ -1969,7 +1977,7 @@
       <c r="G42" s="1" t="inlineStr"/>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
+          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I42" s="1" t="inlineStr">
@@ -1979,7 +1987,7 @@
       </c>
       <c r="J42" s="1" t="inlineStr">
         <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="K42" s="1" t="inlineStr">
@@ -2002,18 +2010,22 @@
       <c r="G43" s="1" t="inlineStr"/>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
+          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I43" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J43" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
       <c r="K43" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L43" s="1" t="inlineStr"/>
@@ -2031,22 +2043,18 @@
       <c r="G44" s="1" t="inlineStr"/>
       <c r="H44" s="1" t="inlineStr">
         <is>
-          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
         </is>
       </c>
       <c r="I44" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J44" s="1" t="inlineStr">
-        <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr"/>
       <c r="K44" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L44" s="1" t="inlineStr"/>
@@ -2064,7 +2072,7 @@
       <c r="G45" s="1" t="inlineStr"/>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I45" s="1" t="inlineStr">
@@ -2074,7 +2082,7 @@
       </c>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
@@ -2097,18 +2105,22 @@
       <c r="G46" s="1" t="inlineStr"/>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I46" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J46" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J46" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
       <c r="K46" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L46" s="1" t="inlineStr"/>
@@ -2126,7 +2138,7 @@
       <c r="G47" s="1" t="inlineStr"/>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I47" s="1" t="inlineStr">
@@ -2136,7 +2148,7 @@
       </c>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -2159,7 +2171,7 @@
       <c r="G48" s="1" t="inlineStr"/>
       <c r="H48" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I48" s="1" t="inlineStr">
@@ -2169,7 +2181,7 @@
       </c>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -2192,7 +2204,7 @@
       <c r="G49" s="1" t="inlineStr"/>
       <c r="H49" s="1" t="inlineStr">
         <is>
-          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="I49" s="1" t="inlineStr">
@@ -2202,7 +2214,7 @@
       </c>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="K49" s="1" t="inlineStr">
@@ -2225,22 +2237,18 @@
       <c r="G50" s="1" t="inlineStr"/>
       <c r="H50" s="1" t="inlineStr">
         <is>
-          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
         </is>
       </c>
       <c r="I50" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J50" s="1" t="inlineStr">
-        <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr"/>
       <c r="K50" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L50" s="1" t="inlineStr"/>
@@ -2249,101 +2257,119 @@
       <c r="O50" s="1" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="1" t="inlineStr"/>
-      <c r="B51" s="1" t="inlineStr"/>
-      <c r="C51" s="1" t="inlineStr"/>
-      <c r="D51" s="1" t="inlineStr"/>
-      <c r="E51" s="1" t="inlineStr"/>
-      <c r="F51" s="1" t="inlineStr"/>
-      <c r="G51" s="1" t="inlineStr"/>
-      <c r="H51" s="1" t="inlineStr">
-        <is>
-          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
-        </is>
-      </c>
-      <c r="I51" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J51" s="1" t="inlineStr">
-        <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
-        </is>
-      </c>
-      <c r="K51" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L51" s="1" t="inlineStr"/>
-      <c r="M51" s="1" t="inlineStr"/>
-      <c r="N51" s="1" t="inlineStr"/>
-      <c r="O51" s="1" t="inlineStr"/>
+      <c r="A51" s="2" t="inlineStr"/>
+      <c r="B51" s="2" t="inlineStr"/>
+      <c r="C51" s="2" t="inlineStr"/>
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr"/>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr"/>
+      <c r="M51" s="2" t="inlineStr"/>
+      <c r="N51" s="2" t="inlineStr"/>
+      <c r="O51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="inlineStr"/>
-      <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
-      <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr"/>
-      <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr"/>
-      <c r="M52" s="2" t="inlineStr"/>
-      <c r="N52" s="2" t="inlineStr"/>
-      <c r="O52" s="2" t="inlineStr"/>
+      <c r="A52" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B52" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C52" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D52" s="1" t="inlineStr">
+        <is>
+          <t>MC_HP</t>
+        </is>
+      </c>
+      <c r="E52" s="1" t="inlineStr">
+        <is>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F52" s="1" t="inlineStr">
+        <is>
+          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
+Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="G52" s="1" t="inlineStr">
+        <is>
+          <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
+2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
+3. Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;
+4. Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;
+5. Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;
+6. Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;
+7. Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;
+8. Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;
+9. Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;
+10. Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;
+11. Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;
+12. Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;
+13. Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;
+14. Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;
+15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L52" s="1">
+        <f>IFERROR(COUNTIF(K52:K67,"CS")/COUNTA(K52:K67),"")</f>
+        <v/>
+      </c>
+      <c r="M52" s="1">
+        <f>COUNTIF(K52:K67,"CS")/15</f>
+        <v/>
+      </c>
+      <c r="N52" s="1">
+        <f>IFERROR(2*(L52*M52)/(L52+M52),"")</f>
+        <v/>
+      </c>
+      <c r="O52" s="1" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B53" s="1" t="inlineStr">
-        <is>
-          <t>Family Finance</t>
-        </is>
-      </c>
-      <c r="C53" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D53" s="1" t="inlineStr">
-        <is>
-          <t>HC_HP</t>
-        </is>
-      </c>
-      <c r="E53" s="1" t="inlineStr">
-        <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
-        </is>
-      </c>
-      <c r="F53" s="1" t="inlineStr">
-        <is>
-          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
-Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
-Expected Behavior: The appearance of the report should be changed to use percent values.</t>
-        </is>
-      </c>
-      <c r="G53" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
+      <c r="A53" s="1" t="inlineStr"/>
+      <c r="B53" s="1" t="inlineStr"/>
+      <c r="C53" s="1" t="inlineStr"/>
+      <c r="D53" s="1" t="inlineStr"/>
+      <c r="E53" s="1" t="inlineStr"/>
+      <c r="F53" s="1" t="inlineStr"/>
+      <c r="G53" s="1" t="inlineStr"/>
       <c r="H53" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I53" s="1" t="inlineStr">
@@ -2353,7 +2379,7 @@
       </c>
       <c r="J53" s="1" t="inlineStr">
         <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K53" s="1" t="inlineStr">
@@ -2361,21 +2387,10 @@
           <t>CS</t>
         </is>
       </c>
-      <c r="L53" s="1">
-        <f>IFERROR(COUNTIF(K53:K60,"CS")/COUNTA(K53:K60),"")</f>
-        <v/>
-      </c>
-      <c r="M53" s="1">
-        <f>COUNTIF(K53:K60,"CS")/8</f>
-        <v/>
-      </c>
-      <c r="N53" s="1">
-        <f>IFERROR(2*(L53*M53)/(L53+M53),"")</f>
-        <v/>
-      </c>
-      <c r="O53" s="1" t="n">
-        <v>8</v>
-      </c>
+      <c r="L53" s="1" t="inlineStr"/>
+      <c r="M53" s="1" t="inlineStr"/>
+      <c r="N53" s="1" t="inlineStr"/>
+      <c r="O53" s="1" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="1" t="inlineStr"/>
@@ -2387,7 +2402,7 @@
       <c r="G54" s="1" t="inlineStr"/>
       <c r="H54" s="1" t="inlineStr">
         <is>
-          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I54" s="1" t="inlineStr">
@@ -2397,7 +2412,7 @@
       </c>
       <c r="J54" s="1" t="inlineStr">
         <is>
-          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K54" s="1" t="inlineStr">
@@ -2420,7 +2435,7 @@
       <c r="G55" s="1" t="inlineStr"/>
       <c r="H55" s="1" t="inlineStr">
         <is>
-          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I55" s="1" t="inlineStr">
@@ -2430,7 +2445,7 @@
       </c>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K55" s="1" t="inlineStr">
@@ -2453,7 +2468,7 @@
       <c r="G56" s="1" t="inlineStr"/>
       <c r="H56" s="1" t="inlineStr">
         <is>
-          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
+          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I56" s="1" t="inlineStr">
@@ -2463,7 +2478,7 @@
       </c>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K56" s="1" t="inlineStr">
@@ -2486,7 +2501,7 @@
       <c r="G57" s="1" t="inlineStr"/>
       <c r="H57" s="1" t="inlineStr">
         <is>
-          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I57" s="1" t="inlineStr">
@@ -2496,7 +2511,7 @@
       </c>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -2519,7 +2534,7 @@
       <c r="G58" s="1" t="inlineStr"/>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
         </is>
       </c>
       <c r="I58" s="1" t="inlineStr">
@@ -2529,7 +2544,7 @@
       </c>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -2552,22 +2567,18 @@
       <c r="G59" s="1" t="inlineStr"/>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
         </is>
       </c>
       <c r="I59" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J59" s="1" t="inlineStr">
-        <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J59" s="1" t="inlineStr"/>
       <c r="K59" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L59" s="1" t="inlineStr"/>
@@ -2585,7 +2596,7 @@
       <c r="G60" s="1" t="inlineStr"/>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I60" s="1" t="inlineStr">
@@ -2595,7 +2606,7 @@
       </c>
       <c r="J60" s="1" t="inlineStr">
         <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="K60" s="1" t="inlineStr">
@@ -2609,100 +2620,66 @@
       <c r="O60" s="1" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="inlineStr"/>
-      <c r="B61" s="2" t="inlineStr"/>
-      <c r="C61" s="2" t="inlineStr"/>
-      <c r="D61" s="2" t="inlineStr"/>
-      <c r="E61" s="2" t="inlineStr"/>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
-      <c r="H61" s="2" t="inlineStr"/>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr"/>
-      <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr"/>
-      <c r="M61" s="2" t="inlineStr"/>
-      <c r="N61" s="2" t="inlineStr"/>
-      <c r="O61" s="2" t="inlineStr"/>
+      <c r="A61" s="1" t="inlineStr"/>
+      <c r="B61" s="1" t="inlineStr"/>
+      <c r="C61" s="1" t="inlineStr"/>
+      <c r="D61" s="1" t="inlineStr"/>
+      <c r="E61" s="1" t="inlineStr"/>
+      <c r="F61" s="1" t="inlineStr"/>
+      <c r="G61" s="1" t="inlineStr"/>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L61" s="1" t="inlineStr"/>
+      <c r="M61" s="1" t="inlineStr"/>
+      <c r="N61" s="1" t="inlineStr"/>
+      <c r="O61" s="1" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B62" s="1" t="inlineStr">
-        <is>
-          <t>Family Finance</t>
-        </is>
-      </c>
-      <c r="C62" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D62" s="1" t="inlineStr">
-        <is>
-          <t>MC_MP</t>
-        </is>
-      </c>
-      <c r="E62" s="1" t="inlineStr">
-        <is>
-          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
-        </is>
-      </c>
-      <c r="F62" s="1" t="inlineStr">
-        <is>
-          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
-Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
-Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
-        </is>
-      </c>
-      <c r="G62" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
+      <c r="A62" s="1" t="inlineStr"/>
+      <c r="B62" s="1" t="inlineStr"/>
+      <c r="C62" s="1" t="inlineStr"/>
+      <c r="D62" s="1" t="inlineStr"/>
+      <c r="E62" s="1" t="inlineStr"/>
+      <c r="F62" s="1" t="inlineStr"/>
+      <c r="G62" s="1" t="inlineStr"/>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
         </is>
       </c>
       <c r="I62" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J62" s="1" t="inlineStr">
-        <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J62" s="1" t="inlineStr"/>
       <c r="K62" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L62" s="1">
-        <f>IFERROR(COUNTIF(K62:K68,"CS")/COUNTA(K62:K68),"")</f>
-        <v/>
-      </c>
-      <c r="M62" s="1">
-        <f>COUNTIF(K62:K68,"CS")/8</f>
-        <v/>
-      </c>
-      <c r="N62" s="1">
-        <f>IFERROR(2*(L62*M62)/(L62+M62),"")</f>
-        <v/>
-      </c>
-      <c r="O62" s="1" t="n">
-        <v>8</v>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L62" s="1" t="inlineStr"/>
+      <c r="M62" s="1" t="inlineStr"/>
+      <c r="N62" s="1" t="inlineStr"/>
+      <c r="O62" s="1" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="1" t="inlineStr"/>
@@ -2714,18 +2691,22 @@
       <c r="G63" s="1" t="inlineStr"/>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I63" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J63" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="inlineStr">
+        <is>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
       <c r="K63" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L63" s="1" t="inlineStr"/>
@@ -2743,7 +2724,7 @@
       <c r="G64" s="1" t="inlineStr"/>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I64" s="1" t="inlineStr">
@@ -2753,7 +2734,7 @@
       </c>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
@@ -2776,7 +2757,7 @@
       <c r="G65" s="1" t="inlineStr"/>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I65" s="1" t="inlineStr">
@@ -2786,7 +2767,7 @@
       </c>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -2809,7 +2790,7 @@
       <c r="G66" s="1" t="inlineStr"/>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I66" s="1" t="inlineStr">
@@ -2819,7 +2800,7 @@
       </c>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
@@ -2842,7 +2823,7 @@
       <c r="G67" s="1" t="inlineStr"/>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="I67" s="1" t="inlineStr">
@@ -2852,7 +2833,7 @@
       </c>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
@@ -2866,37 +2847,621 @@
       <c r="O67" s="1" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="1" t="inlineStr"/>
-      <c r="B68" s="1" t="inlineStr"/>
-      <c r="C68" s="1" t="inlineStr"/>
-      <c r="D68" s="1" t="inlineStr"/>
-      <c r="E68" s="1" t="inlineStr"/>
-      <c r="F68" s="1" t="inlineStr"/>
-      <c r="G68" s="1" t="inlineStr"/>
-      <c r="H68" s="1" t="inlineStr">
+      <c r="A68" s="2" t="inlineStr"/>
+      <c r="B68" s="2" t="inlineStr"/>
+      <c r="C68" s="2" t="inlineStr"/>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr"/>
+      <c r="J68" s="2" t="inlineStr"/>
+      <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="2" t="inlineStr"/>
+      <c r="N68" s="2" t="inlineStr"/>
+      <c r="O68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B69" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C69" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D69" s="1" t="inlineStr">
+        <is>
+          <t>HC_HP</t>
+        </is>
+      </c>
+      <c r="E69" s="1" t="inlineStr">
+        <is>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F69" s="1" t="inlineStr">
+        <is>
+          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
+Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
+Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
+      <c r="G69" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H69" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="I69" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J69" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L69" s="1">
+        <f>IFERROR(COUNTIF(K69:K76,"CS")/COUNTA(K69:K76),"")</f>
+        <v/>
+      </c>
+      <c r="M69" s="1">
+        <f>COUNTIF(K69:K76,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N69" s="1">
+        <f>IFERROR(2*(L69*M69)/(L69+M69),"")</f>
+        <v/>
+      </c>
+      <c r="O69" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="inlineStr"/>
+      <c r="B70" s="1" t="inlineStr"/>
+      <c r="C70" s="1" t="inlineStr"/>
+      <c r="D70" s="1" t="inlineStr"/>
+      <c r="E70" s="1" t="inlineStr"/>
+      <c r="F70" s="1" t="inlineStr"/>
+      <c r="G70" s="1" t="inlineStr"/>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="I70" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J70" s="1" t="inlineStr">
+        <is>
+          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L70" s="1" t="inlineStr"/>
+      <c r="M70" s="1" t="inlineStr"/>
+      <c r="N70" s="1" t="inlineStr"/>
+      <c r="O70" s="1" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr"/>
+      <c r="B71" s="1" t="inlineStr"/>
+      <c r="C71" s="1" t="inlineStr"/>
+      <c r="D71" s="1" t="inlineStr"/>
+      <c r="E71" s="1" t="inlineStr"/>
+      <c r="F71" s="1" t="inlineStr"/>
+      <c r="G71" s="1" t="inlineStr"/>
+      <c r="H71" s="1" t="inlineStr">
+        <is>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I71" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J71" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K71" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L71" s="1" t="inlineStr"/>
+      <c r="M71" s="1" t="inlineStr"/>
+      <c r="N71" s="1" t="inlineStr"/>
+      <c r="O71" s="1" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr"/>
+      <c r="B72" s="1" t="inlineStr"/>
+      <c r="C72" s="1" t="inlineStr"/>
+      <c r="D72" s="1" t="inlineStr"/>
+      <c r="E72" s="1" t="inlineStr"/>
+      <c r="F72" s="1" t="inlineStr"/>
+      <c r="G72" s="1" t="inlineStr"/>
+      <c r="H72" s="1" t="inlineStr">
+        <is>
+          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
+        </is>
+      </c>
+      <c r="I72" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J72" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L72" s="1" t="inlineStr"/>
+      <c r="M72" s="1" t="inlineStr"/>
+      <c r="N72" s="1" t="inlineStr"/>
+      <c r="O72" s="1" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr"/>
+      <c r="B73" s="1" t="inlineStr"/>
+      <c r="C73" s="1" t="inlineStr"/>
+      <c r="D73" s="1" t="inlineStr"/>
+      <c r="E73" s="1" t="inlineStr"/>
+      <c r="F73" s="1" t="inlineStr"/>
+      <c r="G73" s="1" t="inlineStr"/>
+      <c r="H73" s="1" t="inlineStr">
+        <is>
+          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I73" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J73" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K73" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L73" s="1" t="inlineStr"/>
+      <c r="M73" s="1" t="inlineStr"/>
+      <c r="N73" s="1" t="inlineStr"/>
+      <c r="O73" s="1" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr"/>
+      <c r="B74" s="1" t="inlineStr"/>
+      <c r="C74" s="1" t="inlineStr"/>
+      <c r="D74" s="1" t="inlineStr"/>
+      <c r="E74" s="1" t="inlineStr"/>
+      <c r="F74" s="1" t="inlineStr"/>
+      <c r="G74" s="1" t="inlineStr"/>
+      <c r="H74" s="1" t="inlineStr">
+        <is>
+          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="I74" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J74" s="1" t="inlineStr">
+        <is>
+          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="K74" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L74" s="1" t="inlineStr"/>
+      <c r="M74" s="1" t="inlineStr"/>
+      <c r="N74" s="1" t="inlineStr"/>
+      <c r="O74" s="1" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr"/>
+      <c r="B75" s="1" t="inlineStr"/>
+      <c r="C75" s="1" t="inlineStr"/>
+      <c r="D75" s="1" t="inlineStr"/>
+      <c r="E75" s="1" t="inlineStr"/>
+      <c r="F75" s="1" t="inlineStr"/>
+      <c r="G75" s="1" t="inlineStr"/>
+      <c r="H75" s="1" t="inlineStr">
+        <is>
+          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I75" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J75" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K75" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L75" s="1" t="inlineStr"/>
+      <c r="M75" s="1" t="inlineStr"/>
+      <c r="N75" s="1" t="inlineStr"/>
+      <c r="O75" s="1" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr"/>
+      <c r="B76" s="1" t="inlineStr"/>
+      <c r="C76" s="1" t="inlineStr"/>
+      <c r="D76" s="1" t="inlineStr"/>
+      <c r="E76" s="1" t="inlineStr"/>
+      <c r="F76" s="1" t="inlineStr"/>
+      <c r="G76" s="1" t="inlineStr"/>
+      <c r="H76" s="1" t="inlineStr">
+        <is>
+          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I76" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J76" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K76" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L76" s="1" t="inlineStr"/>
+      <c r="M76" s="1" t="inlineStr"/>
+      <c r="N76" s="1" t="inlineStr"/>
+      <c r="O76" s="1" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr"/>
+      <c r="B77" s="2" t="inlineStr"/>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr"/>
+      <c r="I77" s="2" t="inlineStr"/>
+      <c r="J77" s="2" t="inlineStr"/>
+      <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr"/>
+      <c r="M77" s="2" t="inlineStr"/>
+      <c r="N77" s="2" t="inlineStr"/>
+      <c r="O77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B78" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C78" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D78" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E78" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F78" s="1" t="inlineStr">
+        <is>
+          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
+Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
+Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
+        </is>
+      </c>
+      <c r="G78" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H78" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+        </is>
+      </c>
+      <c r="I78" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J78" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K78" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L78" s="1">
+        <f>IFERROR(COUNTIF(K78:K84,"CS")/COUNTA(K78:K84),"")</f>
+        <v/>
+      </c>
+      <c r="M78" s="1">
+        <f>COUNTIF(K78:K84,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N78" s="1">
+        <f>IFERROR(2*(L78*M78)/(L78+M78),"")</f>
+        <v/>
+      </c>
+      <c r="O78" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="inlineStr"/>
+      <c r="B79" s="1" t="inlineStr"/>
+      <c r="C79" s="1" t="inlineStr"/>
+      <c r="D79" s="1" t="inlineStr"/>
+      <c r="E79" s="1" t="inlineStr"/>
+      <c r="F79" s="1" t="inlineStr"/>
+      <c r="G79" s="1" t="inlineStr"/>
+      <c r="H79" s="1" t="inlineStr">
+        <is>
+          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+        </is>
+      </c>
+      <c r="I79" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J79" s="1" t="inlineStr"/>
+      <c r="K79" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L79" s="1" t="inlineStr"/>
+      <c r="M79" s="1" t="inlineStr"/>
+      <c r="N79" s="1" t="inlineStr"/>
+      <c r="O79" s="1" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="1" t="inlineStr"/>
+      <c r="B80" s="1" t="inlineStr"/>
+      <c r="C80" s="1" t="inlineStr"/>
+      <c r="D80" s="1" t="inlineStr"/>
+      <c r="E80" s="1" t="inlineStr"/>
+      <c r="F80" s="1" t="inlineStr"/>
+      <c r="G80" s="1" t="inlineStr"/>
+      <c r="H80" s="1" t="inlineStr">
+        <is>
+          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I80" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K80" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L80" s="1" t="inlineStr"/>
+      <c r="M80" s="1" t="inlineStr"/>
+      <c r="N80" s="1" t="inlineStr"/>
+      <c r="O80" s="1" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="1" t="inlineStr"/>
+      <c r="B81" s="1" t="inlineStr"/>
+      <c r="C81" s="1" t="inlineStr"/>
+      <c r="D81" s="1" t="inlineStr"/>
+      <c r="E81" s="1" t="inlineStr"/>
+      <c r="F81" s="1" t="inlineStr"/>
+      <c r="G81" s="1" t="inlineStr"/>
+      <c r="H81" s="1" t="inlineStr">
+        <is>
+          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="I81" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J81" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K81" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L81" s="1" t="inlineStr"/>
+      <c r="M81" s="1" t="inlineStr"/>
+      <c r="N81" s="1" t="inlineStr"/>
+      <c r="O81" s="1" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="1" t="inlineStr"/>
+      <c r="B82" s="1" t="inlineStr"/>
+      <c r="C82" s="1" t="inlineStr"/>
+      <c r="D82" s="1" t="inlineStr"/>
+      <c r="E82" s="1" t="inlineStr"/>
+      <c r="F82" s="1" t="inlineStr"/>
+      <c r="G82" s="1" t="inlineStr"/>
+      <c r="H82" s="1" t="inlineStr">
+        <is>
+          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I82" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J82" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K82" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L82" s="1" t="inlineStr"/>
+      <c r="M82" s="1" t="inlineStr"/>
+      <c r="N82" s="1" t="inlineStr"/>
+      <c r="O82" s="1" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="1" t="inlineStr"/>
+      <c r="B83" s="1" t="inlineStr"/>
+      <c r="C83" s="1" t="inlineStr"/>
+      <c r="D83" s="1" t="inlineStr"/>
+      <c r="E83" s="1" t="inlineStr"/>
+      <c r="F83" s="1" t="inlineStr"/>
+      <c r="G83" s="1" t="inlineStr"/>
+      <c r="H83" s="1" t="inlineStr">
+        <is>
+          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I83" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J83" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K83" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L83" s="1" t="inlineStr"/>
+      <c r="M83" s="1" t="inlineStr"/>
+      <c r="N83" s="1" t="inlineStr"/>
+      <c r="O83" s="1" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="1" t="inlineStr"/>
+      <c r="B84" s="1" t="inlineStr"/>
+      <c r="C84" s="1" t="inlineStr"/>
+      <c r="D84" s="1" t="inlineStr"/>
+      <c r="E84" s="1" t="inlineStr"/>
+      <c r="F84" s="1" t="inlineStr"/>
+      <c r="G84" s="1" t="inlineStr"/>
+      <c r="H84" s="1" t="inlineStr">
         <is>
           <t>Tap "OK" to confirm the change. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
         </is>
       </c>
-      <c r="I68" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J68" s="1" t="inlineStr">
+      <c r="I84" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J84" s="1" t="inlineStr">
         <is>
           <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
         </is>
       </c>
-      <c r="K68" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L68" s="1" t="inlineStr"/>
-      <c r="M68" s="1" t="inlineStr"/>
-      <c r="N68" s="1" t="inlineStr"/>
-      <c r="O68" s="1" t="inlineStr"/>
+      <c r="K84" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L84" s="1" t="inlineStr"/>
+      <c r="M84" s="1" t="inlineStr"/>
+      <c r="N84" s="1" t="inlineStr"/>
+      <c r="O84" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2909,7 +3474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L12"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3168,19 +3733,19 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>LC_HP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>The Parent Categories of the current category should be displayed.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr">
         <is>
-          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
-Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
-Expected Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Title: Parent Categories tab shows a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G6" s="1" t="inlineStr">
@@ -3193,10 +3758,10 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the parent categories of the current category are not displayed
-Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
-Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
-Correct Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: a blank page is shown
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -3211,7 +3776,7 @@
       </c>
       <c r="K6" s="1" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="L6" s="1" t="inlineStr">
@@ -3250,19 +3815,19 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>MC_HP</t>
+          <t>LC_HP</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+          <t>The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
-Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
+Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
+Expected Behavior: The parent categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G8" s="1" t="inlineStr">
@@ -3275,10 +3840,10 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the app results in a blank page
-Triggering GUI Interactions: taps the PARENT CATEGORIES tab
-Triggering Screen Reference: On the Category Details screen
-Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: the parent categories of the current category are not displayed
+Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
+Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
+Correct Behavior: The parent categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">
@@ -3318,11 +3883,11 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>Family Finance</t>
+          <t>Wikimedia Commons</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
@@ -3332,35 +3897,35 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>HC_HP</t>
+          <t>MC_HP</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F10" s="1" t="inlineStr">
         <is>
-          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
-Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
-Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
+Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the application crashes
-Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
-Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
-Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
         </is>
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the application crashes
-Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
-Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
-Correct Behavior: The appearance of the report should be changed to use percent values.</t>
+          <t>Buggy Behavior: the app results in a blank page
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I10" s="1" t="inlineStr">
@@ -3375,7 +3940,7 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t>Correct</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="L10" s="1" t="inlineStr">
@@ -3414,19 +3979,19 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>MC_MP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr">
         <is>
-          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
-Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
-Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
+          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
+Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
+Expected Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
       <c r="G12" s="1" t="inlineStr">
@@ -3440,27 +4005,109 @@
       <c r="H12" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
+Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
+Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
+Correct Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr"/>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C14" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D14" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E14" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr">
+        <is>
+          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
+Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
+Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
+        </is>
+      </c>
+      <c r="G14" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
+Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
+Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+        </is>
+      </c>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
 Triggering GUI Interactions: the user taps the "Use percent values" checkbox
 Triggering Screen Reference: On the Display of Incomes by Articles dialog
 Correct Behavior: The application should change the report appearance to use percent values without crashing.</t>
         </is>
       </c>
-      <c r="I12" s="1" t="inlineStr">
+      <c r="I14" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="J12" s="1" t="inlineStr">
+      <c r="J14" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="K12" s="1" t="inlineStr">
+      <c r="K14" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="L12" s="1" t="inlineStr">
+      <c r="L14" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -3625,13 +4272,13 @@
         <v/>
       </c>
       <c r="M2" t="n">
-        <v>82577.16666666667</v>
+        <v>77215</v>
       </c>
       <c r="N2" t="n">
-        <v>70.47254125000002</v>
+        <v>65.56321271428571</v>
       </c>
       <c r="O2" t="n">
-        <v>1.5</v>
+        <v>1.428571428571429</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: evaluator container and cli output compatibility
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O84"/>
+  <dimension ref="A1:O102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -523,11 +523,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>10</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Material Files</t>
+          <t>Wikimedia Commons</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -537,652 +537,22 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>HC_LP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Title: FTP server restarts automatically after being stopped and the app is closed
-Observed Behavior: On the FTP server screen, if the user turns off the FTP server switch and then closes the app, the FTP server restarts automatically after stopping it and closing the app.
-Expected Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the category details screen, if the user taps the Parent Categories tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
-2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
-3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
-4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
-5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
-6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
-        </is>
-      </c>
-      <c r="H2" s="1" t="inlineStr">
-        <is>
-          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
-        </is>
-      </c>
-      <c r="I2" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J2" s="1" t="inlineStr">
-        <is>
-          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
-        </is>
-      </c>
-      <c r="K2" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L2" s="1">
-        <f>IFERROR(COUNTIF(K2:K7,"CS")/COUNTA(K2:K7),"")</f>
-        <v/>
-      </c>
-      <c r="M2" s="1">
-        <f>COUNTIF(K2:K7,"CS")/6</f>
-        <v/>
-      </c>
-      <c r="N2" s="1">
-        <f>IFERROR(2*(L2*M2)/(L2+M2),"")</f>
-        <v/>
-      </c>
-      <c r="O2" s="1" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="inlineStr"/>
-      <c r="B3" s="1" t="inlineStr"/>
-      <c r="C3" s="1" t="inlineStr"/>
-      <c r="D3" s="1" t="inlineStr"/>
-      <c r="E3" s="1" t="inlineStr"/>
-      <c r="F3" s="1" t="inlineStr"/>
-      <c r="G3" s="1" t="inlineStr"/>
-      <c r="H3" s="1" t="inlineStr">
-        <is>
-          <t>Grant the storage permission by tapping Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
-        </is>
-      </c>
-      <c r="I3" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J3" s="1" t="inlineStr">
-        <is>
-          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
-        </is>
-      </c>
-      <c r="K3" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L3" s="1" t="inlineStr"/>
-      <c r="M3" s="1" t="inlineStr"/>
-      <c r="N3" s="1" t="inlineStr"/>
-      <c r="O3" s="1" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="inlineStr"/>
-      <c r="B4" s="1" t="inlineStr"/>
-      <c r="C4" s="1" t="inlineStr"/>
-      <c r="D4" s="1" t="inlineStr"/>
-      <c r="E4" s="1" t="inlineStr"/>
-      <c r="F4" s="1" t="inlineStr"/>
-      <c r="G4" s="1" t="inlineStr"/>
-      <c r="H4" s="1" t="inlineStr">
-        <is>
-          <t>Open the navigation drawer from the main Files screen. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
-        </is>
-      </c>
-      <c r="I4" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J4" s="1" t="inlineStr">
-        <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
-        </is>
-      </c>
-      <c r="K4" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L4" s="1" t="inlineStr"/>
-      <c r="M4" s="1" t="inlineStr"/>
-      <c r="N4" s="1" t="inlineStr"/>
-      <c r="O4" s="1" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="inlineStr"/>
-      <c r="B5" s="1" t="inlineStr"/>
-      <c r="C5" s="1" t="inlineStr"/>
-      <c r="D5" s="1" t="inlineStr"/>
-      <c r="E5" s="1" t="inlineStr"/>
-      <c r="F5" s="1" t="inlineStr"/>
-      <c r="G5" s="1" t="inlineStr"/>
-      <c r="H5" s="1" t="inlineStr">
-        <is>
-          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
-        </is>
-      </c>
-      <c r="I5" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J5" s="1" t="inlineStr">
-        <is>
-          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
-        </is>
-      </c>
-      <c r="K5" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L5" s="1" t="inlineStr"/>
-      <c r="M5" s="1" t="inlineStr"/>
-      <c r="N5" s="1" t="inlineStr"/>
-      <c r="O5" s="1" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1" t="inlineStr"/>
-      <c r="B6" s="1" t="inlineStr"/>
-      <c r="C6" s="1" t="inlineStr"/>
-      <c r="D6" s="1" t="inlineStr"/>
-      <c r="E6" s="1" t="inlineStr"/>
-      <c r="F6" s="1" t="inlineStr"/>
-      <c r="G6" s="1" t="inlineStr"/>
-      <c r="H6" s="1" t="inlineStr">
-        <is>
-          <t>On the FTP server screen, tap the ON switch to stop the FTP server. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
-        </is>
-      </c>
-      <c r="I6" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J6" s="1" t="inlineStr">
-        <is>
-          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
-        </is>
-      </c>
-      <c r="K6" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L6" s="1" t="inlineStr"/>
-      <c r="M6" s="1" t="inlineStr"/>
-      <c r="N6" s="1" t="inlineStr"/>
-      <c r="O6" s="1" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="1" t="inlineStr"/>
-      <c r="C7" s="1" t="inlineStr"/>
-      <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr"/>
-      <c r="F7" s="1" t="inlineStr"/>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr">
-        <is>
-          <t>Close the app by pressing Back from the FTP server screen. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
-        </is>
-      </c>
-      <c r="I7" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J7" s="1" t="inlineStr"/>
-      <c r="K7" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L7" s="1" t="inlineStr"/>
-      <c r="M7" s="1" t="inlineStr"/>
-      <c r="N7" s="1" t="inlineStr"/>
-      <c r="O7" s="1" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr"/>
-      <c r="C8" s="2" t="inlineStr"/>
-      <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
-      <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
-      <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="2" t="inlineStr"/>
-      <c r="N8" s="2" t="inlineStr"/>
-      <c r="O8" s="2" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="inlineStr">
-        <is>
-          <t>Material Files</t>
-        </is>
-      </c>
-      <c r="C9" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D9" s="1" t="inlineStr">
-        <is>
-          <t>LC_LP</t>
-        </is>
-      </c>
-      <c r="E9" s="1" t="inlineStr">
-        <is>
-          <t>It restarts on its own.</t>
-        </is>
-      </c>
-      <c r="F9" s="1" t="inlineStr">
-        <is>
-          <t>Title: FTP server restarts automatically after being turned off and leaving the FTP server screen
-Observed Behavior: On the FTP server screen, if the user turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents, the FTP server is restarting on its own.
-Expected Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
-        </is>
-      </c>
-      <c r="G9" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
-2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
-3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
-4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
-5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
-6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
-        </is>
-      </c>
-      <c r="H9" s="1" t="inlineStr">
-        <is>
-          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
-        </is>
-      </c>
-      <c r="I9" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J9" s="1" t="inlineStr">
-        <is>
-          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
-        </is>
-      </c>
-      <c r="K9" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L9" s="1">
-        <f>IFERROR(COUNTIF(K9:K18,"CS")/COUNTA(K9:K18),"")</f>
-        <v/>
-      </c>
-      <c r="M9" s="1">
-        <f>COUNTIF(K9:K18,"CS")/6</f>
-        <v/>
-      </c>
-      <c r="N9" s="1">
-        <f>IFERROR(2*(L9*M9)/(L9+M9),"")</f>
-        <v/>
-      </c>
-      <c r="O9" s="1" t="n">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="inlineStr"/>
-      <c r="B10" s="1" t="inlineStr"/>
-      <c r="C10" s="1" t="inlineStr"/>
-      <c r="D10" s="1" t="inlineStr"/>
-      <c r="E10" s="1" t="inlineStr"/>
-      <c r="F10" s="1" t="inlineStr"/>
-      <c r="G10" s="1" t="inlineStr"/>
-      <c r="H10" s="1" t="inlineStr">
-        <is>
-          <t>On the permission dialog, tap Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
-        </is>
-      </c>
-      <c r="I10" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J10" s="1" t="inlineStr">
-        <is>
-          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
-        </is>
-      </c>
-      <c r="K10" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L10" s="1" t="inlineStr"/>
-      <c r="M10" s="1" t="inlineStr"/>
-      <c r="N10" s="1" t="inlineStr"/>
-      <c r="O10" s="1" t="inlineStr"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr"/>
-      <c r="B11" s="1" t="inlineStr"/>
-      <c r="C11" s="1" t="inlineStr"/>
-      <c r="D11" s="1" t="inlineStr"/>
-      <c r="E11" s="1" t="inlineStr"/>
-      <c r="F11" s="1" t="inlineStr"/>
-      <c r="G11" s="1" t="inlineStr"/>
-      <c r="H11" s="1" t="inlineStr">
-        <is>
-          <t>Open the navigation menu by tapping Navigate up. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
-        </is>
-      </c>
-      <c r="I11" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J11" s="1" t="inlineStr">
-        <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
-        </is>
-      </c>
-      <c r="K11" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L11" s="1" t="inlineStr"/>
-      <c r="M11" s="1" t="inlineStr"/>
-      <c r="N11" s="1" t="inlineStr"/>
-      <c r="O11" s="1" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr"/>
-      <c r="B12" s="1" t="inlineStr"/>
-      <c r="C12" s="1" t="inlineStr"/>
-      <c r="D12" s="1" t="inlineStr"/>
-      <c r="E12" s="1" t="inlineStr"/>
-      <c r="F12" s="1" t="inlineStr"/>
-      <c r="G12" s="1" t="inlineStr"/>
-      <c r="H12" s="1" t="inlineStr">
-        <is>
-          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
-        </is>
-      </c>
-      <c r="I12" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J12" s="1" t="inlineStr">
-        <is>
-          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
-        </is>
-      </c>
-      <c r="K12" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L12" s="1" t="inlineStr"/>
-      <c r="M12" s="1" t="inlineStr"/>
-      <c r="N12" s="1" t="inlineStr"/>
-      <c r="O12" s="1" t="inlineStr"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr"/>
-      <c r="B13" s="1" t="inlineStr"/>
-      <c r="C13" s="1" t="inlineStr"/>
-      <c r="D13" s="1" t="inlineStr"/>
-      <c r="E13" s="1" t="inlineStr"/>
-      <c r="F13" s="1" t="inlineStr"/>
-      <c r="G13" s="1" t="inlineStr"/>
-      <c r="H13" s="1" t="inlineStr">
-        <is>
-          <t>Tap the FTP server status switch while it is OFF to turn it ON. &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
-        </is>
-      </c>
-      <c r="I13" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J13" s="1" t="inlineStr">
-        <is>
-          <t>Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
-        </is>
-      </c>
-      <c r="K13" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L13" s="1" t="inlineStr"/>
-      <c r="M13" s="1" t="inlineStr"/>
-      <c r="N13" s="1" t="inlineStr"/>
-      <c r="O13" s="1" t="inlineStr"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="1" t="inlineStr"/>
-      <c r="B14" s="1" t="inlineStr"/>
-      <c r="C14" s="1" t="inlineStr"/>
-      <c r="D14" s="1" t="inlineStr"/>
-      <c r="E14" s="1" t="inlineStr"/>
-      <c r="F14" s="1" t="inlineStr"/>
-      <c r="G14" s="1" t="inlineStr"/>
-      <c r="H14" s="1" t="inlineStr">
-        <is>
-          <t>Tap the FTP server status switch while it is ON to turn it OFF. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
-        </is>
-      </c>
-      <c r="I14" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J14" s="1" t="inlineStr">
-        <is>
-          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
-        </is>
-      </c>
-      <c r="K14" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L14" s="1" t="inlineStr"/>
-      <c r="M14" s="1" t="inlineStr"/>
-      <c r="N14" s="1" t="inlineStr"/>
-      <c r="O14" s="1" t="inlineStr"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr"/>
-      <c r="B15" s="1" t="inlineStr"/>
-      <c r="C15" s="1" t="inlineStr"/>
-      <c r="D15" s="1" t="inlineStr"/>
-      <c r="E15" s="1" t="inlineStr"/>
-      <c r="F15" s="1" t="inlineStr"/>
-      <c r="G15" s="1" t="inlineStr"/>
-      <c r="H15" s="1" t="inlineStr">
-        <is>
-          <t>Leave the FTP server screen by tapping Navigate up. &lt;f5deb5a7a067fcecd183ba802aa26e2dfb3c5e38306d9407fd3b178866210afb&gt;</t>
-        </is>
-      </c>
-      <c r="I15" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J15" s="1" t="inlineStr"/>
-      <c r="K15" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L15" s="1" t="inlineStr"/>
-      <c r="M15" s="1" t="inlineStr"/>
-      <c r="N15" s="1" t="inlineStr"/>
-      <c r="O15" s="1" t="inlineStr"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="1" t="inlineStr"/>
-      <c r="B16" s="1" t="inlineStr"/>
-      <c r="C16" s="1" t="inlineStr"/>
-      <c r="D16" s="1" t="inlineStr"/>
-      <c r="E16" s="1" t="inlineStr"/>
-      <c r="F16" s="1" t="inlineStr"/>
-      <c r="G16" s="1" t="inlineStr"/>
-      <c r="H16" s="1" t="inlineStr">
-        <is>
-          <t>Tap the list item to return to the FTP server screen path context. &lt;6766d1c12b54808176b7d8e110b78ee25e2843492f806acedcc0d8e1da70972c&gt;</t>
-        </is>
-      </c>
-      <c r="I16" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J16" s="1" t="inlineStr"/>
-      <c r="K16" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L16" s="1" t="inlineStr"/>
-      <c r="M16" s="1" t="inlineStr"/>
-      <c r="N16" s="1" t="inlineStr"/>
-      <c r="O16" s="1" t="inlineStr"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="1" t="inlineStr"/>
-      <c r="B17" s="1" t="inlineStr"/>
-      <c r="C17" s="1" t="inlineStr"/>
-      <c r="D17" s="1" t="inlineStr"/>
-      <c r="E17" s="1" t="inlineStr"/>
-      <c r="F17" s="1" t="inlineStr"/>
-      <c r="G17" s="1" t="inlineStr"/>
-      <c r="H17" s="1" t="inlineStr">
-        <is>
-          <t>Open Recents using the system Back/Recents control. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
-        </is>
-      </c>
-      <c r="I17" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J17" s="1" t="inlineStr"/>
-      <c r="K17" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L17" s="1" t="inlineStr"/>
-      <c r="M17" s="1" t="inlineStr"/>
-      <c r="N17" s="1" t="inlineStr"/>
-      <c r="O17" s="1" t="inlineStr"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="1" t="inlineStr"/>
-      <c r="B18" s="1" t="inlineStr"/>
-      <c r="C18" s="1" t="inlineStr"/>
-      <c r="D18" s="1" t="inlineStr"/>
-      <c r="E18" s="1" t="inlineStr"/>
-      <c r="F18" s="1" t="inlineStr"/>
-      <c r="G18" s="1" t="inlineStr"/>
-      <c r="H18" s="1" t="inlineStr">
-        <is>
-          <t>Dismiss the Files app task from Recents. &lt;b05234dc13810ef197b494fe9ce3b3d6e6927d53c722ad904f3dc53e425da84c&gt;</t>
-        </is>
-      </c>
-      <c r="I18" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J18" s="1" t="inlineStr"/>
-      <c r="K18" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L18" s="1" t="inlineStr"/>
-      <c r="M18" s="1" t="inlineStr"/>
-      <c r="N18" s="1" t="inlineStr"/>
-      <c r="O18" s="1" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr"/>
-      <c r="B19" s="2" t="inlineStr"/>
-      <c r="C19" s="2" t="inlineStr"/>
-      <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
-      <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
-      <c r="H19" s="2" t="inlineStr"/>
-      <c r="I19" s="2" t="inlineStr"/>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
-      <c r="L19" s="2" t="inlineStr"/>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="1" t="n">
-        <v>135</v>
-      </c>
-      <c r="B20" s="1" t="inlineStr">
-        <is>
-          <t>Wikimedia Commons</t>
-        </is>
-      </c>
-      <c r="C20" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D20" s="1" t="inlineStr">
-        <is>
-          <t>HC_HP</t>
-        </is>
-      </c>
-      <c r="E20" s="1" t="inlineStr">
-        <is>
-          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F20" s="1" t="inlineStr">
-        <is>
-          <t>Title: Parent Categories tab shows a blank page on the category details screen
-Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="G20" s="1" t="inlineStr">
         <is>
           <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
 2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
@@ -1201,9 +571,636 @@
 15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
+      <c r="H2" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="I2" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="K2" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L2" s="1">
+        <f>IFERROR(COUNTIF(K2:K16,"CS")/COUNTA(K2:K16),"")</f>
+        <v/>
+      </c>
+      <c r="M2" s="1">
+        <f>COUNTIF(K2:K16,"CS")/15</f>
+        <v/>
+      </c>
+      <c r="N2" s="1">
+        <f>IFERROR(2*(L2*M2)/(L2+M2),"")</f>
+        <v/>
+      </c>
+      <c r="O2" s="1" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr"/>
+      <c r="B3" s="1" t="inlineStr"/>
+      <c r="C3" s="1" t="inlineStr"/>
+      <c r="D3" s="1" t="inlineStr"/>
+      <c r="E3" s="1" t="inlineStr"/>
+      <c r="F3" s="1" t="inlineStr"/>
+      <c r="G3" s="1" t="inlineStr"/>
+      <c r="H3" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left on the welcome/tutorial screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+        </is>
+      </c>
+      <c r="I3" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+        </is>
+      </c>
+      <c r="K3" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L3" s="1" t="inlineStr"/>
+      <c r="M3" s="1" t="inlineStr"/>
+      <c r="N3" s="1" t="inlineStr"/>
+      <c r="O3" s="1" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr"/>
+      <c r="B4" s="1" t="inlineStr"/>
+      <c r="C4" s="1" t="inlineStr"/>
+      <c r="D4" s="1" t="inlineStr"/>
+      <c r="E4" s="1" t="inlineStr"/>
+      <c r="F4" s="1" t="inlineStr"/>
+      <c r="G4" s="1" t="inlineStr"/>
+      <c r="H4" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left again on the welcome/tutorial screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+        </is>
+      </c>
+      <c r="I4" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+        </is>
+      </c>
+      <c r="K4" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L4" s="1" t="inlineStr"/>
+      <c r="M4" s="1" t="inlineStr"/>
+      <c r="N4" s="1" t="inlineStr"/>
+      <c r="O4" s="1" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr"/>
+      <c r="B5" s="1" t="inlineStr"/>
+      <c r="C5" s="1" t="inlineStr"/>
+      <c r="D5" s="1" t="inlineStr"/>
+      <c r="E5" s="1" t="inlineStr"/>
+      <c r="F5" s="1" t="inlineStr"/>
+      <c r="G5" s="1" t="inlineStr"/>
+      <c r="H5" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left a third time on the welcome/tutorial screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+        </is>
+      </c>
+      <c r="I5" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+        </is>
+      </c>
+      <c r="K5" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L5" s="1" t="inlineStr"/>
+      <c r="M5" s="1" t="inlineStr"/>
+      <c r="N5" s="1" t="inlineStr"/>
+      <c r="O5" s="1" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr"/>
+      <c r="B6" s="1" t="inlineStr"/>
+      <c r="C6" s="1" t="inlineStr"/>
+      <c r="D6" s="1" t="inlineStr"/>
+      <c r="E6" s="1" t="inlineStr"/>
+      <c r="F6" s="1" t="inlineStr"/>
+      <c r="G6" s="1" t="inlineStr"/>
+      <c r="H6" s="1" t="inlineStr">
+        <is>
+          <t>Swipe left a fourth time on the welcome/tutorial screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+        </is>
+      </c>
+      <c r="I6" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+        </is>
+      </c>
+      <c r="K6" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L6" s="1" t="inlineStr"/>
+      <c r="M6" s="1" t="inlineStr"/>
+      <c r="N6" s="1" t="inlineStr"/>
+      <c r="O6" s="1" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr"/>
+      <c r="B7" s="1" t="inlineStr"/>
+      <c r="C7" s="1" t="inlineStr"/>
+      <c r="D7" s="1" t="inlineStr"/>
+      <c r="E7" s="1" t="inlineStr"/>
+      <c r="F7" s="1" t="inlineStr"/>
+      <c r="G7" s="1" t="inlineStr"/>
+      <c r="H7" s="1" t="inlineStr">
+        <is>
+          <t>Tap "YES!" on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+        </is>
+      </c>
+      <c r="I7" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+        </is>
+      </c>
+      <c r="K7" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L7" s="1" t="inlineStr"/>
+      <c r="M7" s="1" t="inlineStr"/>
+      <c r="N7" s="1" t="inlineStr"/>
+      <c r="O7" s="1" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr"/>
+      <c r="B8" s="1" t="inlineStr"/>
+      <c r="C8" s="1" t="inlineStr"/>
+      <c r="D8" s="1" t="inlineStr"/>
+      <c r="E8" s="1" t="inlineStr"/>
+      <c r="F8" s="1" t="inlineStr"/>
+      <c r="G8" s="1" t="inlineStr"/>
+      <c r="H8" s="1" t="inlineStr">
+        <is>
+          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="I8" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="inlineStr">
+        <is>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="K8" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L8" s="1" t="inlineStr"/>
+      <c r="M8" s="1" t="inlineStr"/>
+      <c r="N8" s="1" t="inlineStr"/>
+      <c r="O8" s="1" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr"/>
+      <c r="B9" s="1" t="inlineStr"/>
+      <c r="C9" s="1" t="inlineStr"/>
+      <c r="D9" s="1" t="inlineStr"/>
+      <c r="E9" s="1" t="inlineStr"/>
+      <c r="F9" s="1" t="inlineStr"/>
+      <c r="G9" s="1" t="inlineStr"/>
+      <c r="H9" s="1" t="inlineStr">
+        <is>
+          <t>Confirm skipping login by tapping "YES". &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="I9" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="K9" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L9" s="1" t="inlineStr"/>
+      <c r="M9" s="1" t="inlineStr"/>
+      <c r="N9" s="1" t="inlineStr"/>
+      <c r="O9" s="1" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr"/>
+      <c r="B10" s="1" t="inlineStr"/>
+      <c r="C10" s="1" t="inlineStr"/>
+      <c r="D10" s="1" t="inlineStr"/>
+      <c r="E10" s="1" t="inlineStr"/>
+      <c r="F10" s="1" t="inlineStr"/>
+      <c r="G10" s="1" t="inlineStr"/>
+      <c r="H10" s="1" t="inlineStr">
+        <is>
+          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
+      <c r="I10" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
+      <c r="K10" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L10" s="1" t="inlineStr"/>
+      <c r="M10" s="1" t="inlineStr"/>
+      <c r="N10" s="1" t="inlineStr"/>
+      <c r="O10" s="1" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr"/>
+      <c r="B11" s="1" t="inlineStr"/>
+      <c r="C11" s="1" t="inlineStr"/>
+      <c r="D11" s="1" t="inlineStr"/>
+      <c r="E11" s="1" t="inlineStr"/>
+      <c r="F11" s="1" t="inlineStr"/>
+      <c r="G11" s="1" t="inlineStr"/>
+      <c r="H11" s="1" t="inlineStr">
+        <is>
+          <t>Select "Explore" from the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+        </is>
+      </c>
+      <c r="I11" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J11" s="1" t="inlineStr">
+        <is>
+          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+        </is>
+      </c>
+      <c r="K11" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L11" s="1" t="inlineStr"/>
+      <c r="M11" s="1" t="inlineStr"/>
+      <c r="N11" s="1" t="inlineStr"/>
+      <c r="O11" s="1" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr"/>
+      <c r="B12" s="1" t="inlineStr"/>
+      <c r="C12" s="1" t="inlineStr"/>
+      <c r="D12" s="1" t="inlineStr"/>
+      <c r="E12" s="1" t="inlineStr"/>
+      <c r="F12" s="1" t="inlineStr"/>
+      <c r="G12" s="1" t="inlineStr"/>
+      <c r="H12" s="1" t="inlineStr">
+        <is>
+          <t>Tap a picture in Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="I12" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J12" s="1" t="inlineStr">
+        <is>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="K12" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L12" s="1" t="inlineStr"/>
+      <c r="M12" s="1" t="inlineStr"/>
+      <c r="N12" s="1" t="inlineStr"/>
+      <c r="O12" s="1" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr"/>
+      <c r="B13" s="1" t="inlineStr"/>
+      <c r="C13" s="1" t="inlineStr"/>
+      <c r="D13" s="1" t="inlineStr"/>
+      <c r="E13" s="1" t="inlineStr"/>
+      <c r="F13" s="1" t="inlineStr"/>
+      <c r="G13" s="1" t="inlineStr"/>
+      <c r="H13" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="I13" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J13" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="K13" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L13" s="1" t="inlineStr"/>
+      <c r="M13" s="1" t="inlineStr"/>
+      <c r="N13" s="1" t="inlineStr"/>
+      <c r="O13" s="1" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr"/>
+      <c r="B14" s="1" t="inlineStr"/>
+      <c r="C14" s="1" t="inlineStr"/>
+      <c r="D14" s="1" t="inlineStr"/>
+      <c r="E14" s="1" t="inlineStr"/>
+      <c r="F14" s="1" t="inlineStr"/>
+      <c r="G14" s="1" t="inlineStr"/>
+      <c r="H14" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="inlineStr"/>
+      <c r="M14" s="1" t="inlineStr"/>
+      <c r="N14" s="1" t="inlineStr"/>
+      <c r="O14" s="1" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr"/>
+      <c r="B15" s="1" t="inlineStr"/>
+      <c r="C15" s="1" t="inlineStr"/>
+      <c r="D15" s="1" t="inlineStr"/>
+      <c r="E15" s="1" t="inlineStr"/>
+      <c r="F15" s="1" t="inlineStr"/>
+      <c r="G15" s="1" t="inlineStr"/>
+      <c r="H15" s="1" t="inlineStr">
+        <is>
+          <t>Tap a category from the media details categories list. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="I15" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J15" s="1" t="inlineStr">
+        <is>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="K15" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L15" s="1" t="inlineStr"/>
+      <c r="M15" s="1" t="inlineStr"/>
+      <c r="N15" s="1" t="inlineStr"/>
+      <c r="O15" s="1" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr"/>
+      <c r="B16" s="1" t="inlineStr"/>
+      <c r="C16" s="1" t="inlineStr"/>
+      <c r="D16" s="1" t="inlineStr"/>
+      <c r="E16" s="1" t="inlineStr"/>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr"/>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Tap the "PARENT CATEGORIES" tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K16" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L16" s="1" t="inlineStr"/>
+      <c r="M16" s="1" t="inlineStr"/>
+      <c r="N16" s="1" t="inlineStr"/>
+      <c r="O16" s="1" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Material Files</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>HC_LP</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
+2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
+3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
+4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
+5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
+6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+        </is>
+      </c>
+      <c r="I18" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J18" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+        </is>
+      </c>
+      <c r="K18" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L18" s="1">
+        <f>IFERROR(COUNTIF(K18:K23,"CS")/COUNTA(K18:K23),"")</f>
+        <v/>
+      </c>
+      <c r="M18" s="1">
+        <f>COUNTIF(K18:K23,"CS")/6</f>
+        <v/>
+      </c>
+      <c r="N18" s="1">
+        <f>IFERROR(2*(L18*M18)/(L18+M18),"")</f>
+        <v/>
+      </c>
+      <c r="O18" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr"/>
+      <c r="B19" s="1" t="inlineStr"/>
+      <c r="C19" s="1" t="inlineStr"/>
+      <c r="D19" s="1" t="inlineStr"/>
+      <c r="E19" s="1" t="inlineStr"/>
+      <c r="F19" s="1" t="inlineStr"/>
+      <c r="G19" s="1" t="inlineStr"/>
+      <c r="H19" s="1" t="inlineStr">
+        <is>
+          <t>Grant the storage permission by tapping Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+        </is>
+      </c>
+      <c r="I19" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J19" s="1" t="inlineStr">
+        <is>
+          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+        </is>
+      </c>
+      <c r="K19" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L19" s="1" t="inlineStr"/>
+      <c r="M19" s="1" t="inlineStr"/>
+      <c r="N19" s="1" t="inlineStr"/>
+      <c r="O19" s="1" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr"/>
+      <c r="B20" s="1" t="inlineStr"/>
+      <c r="C20" s="1" t="inlineStr"/>
+      <c r="D20" s="1" t="inlineStr"/>
+      <c r="E20" s="1" t="inlineStr"/>
+      <c r="F20" s="1" t="inlineStr"/>
+      <c r="G20" s="1" t="inlineStr"/>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+          <t>Open the navigation drawer from the main Files screen. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="I20" s="1" t="inlineStr">
@@ -1213,7 +1210,7 @@
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
@@ -1221,21 +1218,10 @@
           <t>CS</t>
         </is>
       </c>
-      <c r="L20" s="1">
-        <f>IFERROR(COUNTIF(K20:K34,"CS")/COUNTA(K20:K34),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="1">
-        <f>COUNTIF(K20:K34,"CS")/15</f>
-        <v/>
-      </c>
-      <c r="N20" s="1">
-        <f>IFERROR(2*(L20*M20)/(L20+M20),"")</f>
-        <v/>
-      </c>
-      <c r="O20" s="1" t="n">
-        <v>15</v>
-      </c>
+      <c r="L20" s="1" t="inlineStr"/>
+      <c r="M20" s="1" t="inlineStr"/>
+      <c r="N20" s="1" t="inlineStr"/>
+      <c r="O20" s="1" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="1" t="inlineStr"/>
@@ -1247,7 +1233,7 @@
       <c r="G21" s="1" t="inlineStr"/>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="I21" s="1" t="inlineStr">
@@ -1257,7 +1243,7 @@
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="K21" s="1" t="inlineStr">
@@ -1280,7 +1266,7 @@
       <c r="G22" s="1" t="inlineStr"/>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the second onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+          <t>On the FTP server screen, tap the ON switch to stop the FTP server. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
         </is>
       </c>
       <c r="I22" s="1" t="inlineStr">
@@ -1290,7 +1276,7 @@
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
@@ -1313,22 +1299,18 @@
       <c r="G23" s="1" t="inlineStr"/>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the third onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+          <t>Close the app by pressing Back from the FTP server screen. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J23" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr"/>
       <c r="K23" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L23" s="1" t="inlineStr"/>
@@ -1337,49 +1319,60 @@
       <c r="O23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="1" t="inlineStr"/>
-      <c r="B24" s="1" t="inlineStr"/>
-      <c r="C24" s="1" t="inlineStr"/>
-      <c r="D24" s="1" t="inlineStr"/>
-      <c r="E24" s="1" t="inlineStr"/>
-      <c r="F24" s="1" t="inlineStr"/>
-      <c r="G24" s="1" t="inlineStr"/>
-      <c r="H24" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left through the fourth onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="I24" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J24" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="K24" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L24" s="1" t="inlineStr"/>
-      <c r="M24" s="1" t="inlineStr"/>
-      <c r="N24" s="1" t="inlineStr"/>
-      <c r="O24" s="1" t="inlineStr"/>
+      <c r="A24" s="2" t="inlineStr"/>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="2" t="inlineStr"/>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
+      <c r="N24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="inlineStr"/>
-      <c r="B25" s="1" t="inlineStr"/>
-      <c r="C25" s="1" t="inlineStr"/>
-      <c r="D25" s="1" t="inlineStr"/>
-      <c r="E25" s="1" t="inlineStr"/>
+      <c r="A25" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B25" s="1" t="inlineStr">
+        <is>
+          <t>Material Files</t>
+        </is>
+      </c>
+      <c r="C25" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D25" s="1" t="inlineStr">
+        <is>
+          <t>LC_LP</t>
+        </is>
+      </c>
+      <c r="E25" s="1" t="inlineStr">
+        <is>
+          <t>It restarts on its own.</t>
+        </is>
+      </c>
       <c r="F25" s="1" t="inlineStr"/>
-      <c r="G25" s="1" t="inlineStr"/>
+      <c r="G25" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
+2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
+3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
+4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
+5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
+6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
       <c r="H25" s="1" t="inlineStr">
         <is>
-          <t>Tap YES! on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
         </is>
       </c>
       <c r="I25" s="1" t="inlineStr">
@@ -1389,7 +1382,7 @@
       </c>
       <c r="J25" s="1" t="inlineStr">
         <is>
-          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
         </is>
       </c>
       <c r="K25" s="1" t="inlineStr">
@@ -1397,10 +1390,21 @@
           <t>CS</t>
         </is>
       </c>
-      <c r="L25" s="1" t="inlineStr"/>
-      <c r="M25" s="1" t="inlineStr"/>
-      <c r="N25" s="1" t="inlineStr"/>
-      <c r="O25" s="1" t="inlineStr"/>
+      <c r="L25" s="1">
+        <f>IFERROR(COUNTIF(K25:K34,"CS")/COUNTA(K25:K34),"")</f>
+        <v/>
+      </c>
+      <c r="M25" s="1">
+        <f>COUNTIF(K25:K34,"CS")/6</f>
+        <v/>
+      </c>
+      <c r="N25" s="1">
+        <f>IFERROR(2*(L25*M25)/(L25+M25),"")</f>
+        <v/>
+      </c>
+      <c r="O25" s="1" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr"/>
@@ -1412,7 +1416,7 @@
       <c r="G26" s="1" t="inlineStr"/>
       <c r="H26" s="1" t="inlineStr">
         <is>
-          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+          <t>On the permission dialog, tap Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
         </is>
       </c>
       <c r="I26" s="1" t="inlineStr">
@@ -1422,7 +1426,7 @@
       </c>
       <c r="J26" s="1" t="inlineStr">
         <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
         </is>
       </c>
       <c r="K26" s="1" t="inlineStr">
@@ -1445,7 +1449,7 @@
       <c r="G27" s="1" t="inlineStr"/>
       <c r="H27" s="1" t="inlineStr">
         <is>
-          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Open the navigation menu by tapping Navigate up. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="I27" s="1" t="inlineStr">
@@ -1455,7 +1459,7 @@
       </c>
       <c r="J27" s="1" t="inlineStr">
         <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="K27" s="1" t="inlineStr">
@@ -1478,7 +1482,7 @@
       <c r="G28" s="1" t="inlineStr"/>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="I28" s="1" t="inlineStr">
@@ -1488,7 +1492,7 @@
       </c>
       <c r="J28" s="1" t="inlineStr">
         <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="K28" s="1" t="inlineStr">
@@ -1511,7 +1515,7 @@
       <c r="G29" s="1" t="inlineStr"/>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>Select Explore from the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+          <t>Tap the FTP server status switch while it is OFF to turn it ON. &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -1521,7 +1525,7 @@
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
-          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+          <t>Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
         </is>
       </c>
       <c r="K29" s="1" t="inlineStr">
@@ -1544,7 +1548,7 @@
       <c r="G30" s="1" t="inlineStr"/>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>Tap a picture in the Explore grid to open its media details. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Tap the FTP server status switch while it is ON to turn it OFF. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
         </is>
       </c>
       <c r="I30" s="1" t="inlineStr">
@@ -1554,7 +1558,7 @@
       </c>
       <c r="J30" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
         </is>
       </c>
       <c r="K30" s="1" t="inlineStr">
@@ -1577,22 +1581,18 @@
       <c r="G31" s="1" t="inlineStr"/>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Leave the FTP server screen by tapping Navigate up. &lt;f5deb5a7a067fcecd183ba802aa26e2dfb3c5e38306d9407fd3b178866210afb&gt;</t>
         </is>
       </c>
       <c r="I31" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J31" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="inlineStr"/>
       <c r="K31" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L31" s="1" t="inlineStr"/>
@@ -1610,22 +1610,18 @@
       <c r="G32" s="1" t="inlineStr"/>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Tap the list item to return to the FTP server screen path context. &lt;6766d1c12b54808176b7d8e110b78ee25e2843492f806acedcc0d8e1da70972c&gt;</t>
         </is>
       </c>
       <c r="I32" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J32" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J32" s="1" t="inlineStr"/>
       <c r="K32" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L32" s="1" t="inlineStr"/>
@@ -1643,22 +1639,18 @@
       <c r="G33" s="1" t="inlineStr"/>
       <c r="H33" s="1" t="inlineStr">
         <is>
-          <t>Tap a category in the media details screen to open category details. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Open Recents using the system Back/Recents control. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
         </is>
       </c>
       <c r="I33" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J33" s="1" t="inlineStr">
-        <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J33" s="1" t="inlineStr"/>
       <c r="K33" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L33" s="1" t="inlineStr"/>
@@ -1676,22 +1668,18 @@
       <c r="G34" s="1" t="inlineStr"/>
       <c r="H34" s="1" t="inlineStr">
         <is>
-          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Dismiss the Files app task from Recents. &lt;b05234dc13810ef197b494fe9ce3b3d6e6927d53c722ad904f3dc53e425da84c&gt;</t>
         </is>
       </c>
       <c r="I34" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J34" s="1" t="inlineStr">
-        <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr"/>
       <c r="K34" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L34" s="1" t="inlineStr"/>
@@ -1732,19 +1720,19 @@
       </c>
       <c r="D36" s="1" t="inlineStr">
         <is>
-          <t>LC_HP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E36" s="1" t="inlineStr">
         <is>
-          <t>The Parent Categories of the current category should be displayed.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F36" s="1" t="inlineStr">
         <is>
-          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
-Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
-Expected Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G36" s="1" t="inlineStr">
@@ -1787,11 +1775,11 @@
         </is>
       </c>
       <c r="L36" s="1">
-        <f>IFERROR(COUNTIF(K36:K50,"CS")/COUNTA(K36:K50),"")</f>
+        <f>IFERROR(COUNTIF(K36:K52,"CS")/COUNTA(K36:K52),"")</f>
         <v/>
       </c>
       <c r="M36" s="1">
-        <f>COUNTIF(K36:K50,"CS")/15</f>
+        <f>COUNTIF(K36:K52,"CS")/15</f>
         <v/>
       </c>
       <c r="N36" s="1">
@@ -1812,7 +1800,7 @@
       <c r="G37" s="1" t="inlineStr"/>
       <c r="H37" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+          <t>Swipe left on the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I37" s="1" t="inlineStr">
@@ -1845,7 +1833,7 @@
       <c r="G38" s="1" t="inlineStr"/>
       <c r="H38" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I38" s="1" t="inlineStr">
@@ -1878,7 +1866,7 @@
       <c r="G39" s="1" t="inlineStr"/>
       <c r="H39" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I39" s="1" t="inlineStr">
@@ -1911,7 +1899,7 @@
       <c r="G40" s="1" t="inlineStr"/>
       <c r="H40" s="1" t="inlineStr">
         <is>
-          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I40" s="1" t="inlineStr">
@@ -1944,7 +1932,7 @@
       <c r="G41" s="1" t="inlineStr"/>
       <c r="H41" s="1" t="inlineStr">
         <is>
-          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Tap YES! on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I41" s="1" t="inlineStr">
@@ -1977,22 +1965,18 @@
       <c r="G42" s="1" t="inlineStr"/>
       <c r="H42" s="1" t="inlineStr">
         <is>
-          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
         </is>
       </c>
       <c r="I42" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J42" s="1" t="inlineStr">
-        <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J42" s="1" t="inlineStr"/>
       <c r="K42" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L42" s="1" t="inlineStr"/>
@@ -2010,22 +1994,18 @@
       <c r="G43" s="1" t="inlineStr"/>
       <c r="H43" s="1" t="inlineStr">
         <is>
-          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
         </is>
       </c>
       <c r="I43" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J43" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J43" s="1" t="inlineStr"/>
       <c r="K43" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L43" s="1" t="inlineStr"/>
@@ -2043,18 +2023,22 @@
       <c r="G44" s="1" t="inlineStr"/>
       <c r="H44" s="1" t="inlineStr">
         <is>
-          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I44" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J44" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J44" s="1" t="inlineStr">
+        <is>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
       <c r="K44" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L44" s="1" t="inlineStr"/>
@@ -2072,7 +2056,7 @@
       <c r="G45" s="1" t="inlineStr"/>
       <c r="H45" s="1" t="inlineStr">
         <is>
-          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Tap YES on the skip-login confirmation dialog. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I45" s="1" t="inlineStr">
@@ -2082,7 +2066,7 @@
       </c>
       <c r="J45" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="K45" s="1" t="inlineStr">
@@ -2105,7 +2089,7 @@
       <c r="G46" s="1" t="inlineStr"/>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="I46" s="1" t="inlineStr">
@@ -2115,7 +2099,7 @@
       </c>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -2138,7 +2122,7 @@
       <c r="G47" s="1" t="inlineStr"/>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Tap Explore in the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
         </is>
       </c>
       <c r="I47" s="1" t="inlineStr">
@@ -2148,7 +2132,7 @@
       </c>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -2171,7 +2155,7 @@
       <c r="G48" s="1" t="inlineStr"/>
       <c r="H48" s="1" t="inlineStr">
         <is>
-          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Tap a picture from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I48" s="1" t="inlineStr">
@@ -2181,7 +2165,7 @@
       </c>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -2204,7 +2188,7 @@
       <c r="G49" s="1" t="inlineStr"/>
       <c r="H49" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I49" s="1" t="inlineStr">
@@ -2214,7 +2198,7 @@
       </c>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="K49" s="1" t="inlineStr">
@@ -2237,18 +2221,22 @@
       <c r="G50" s="1" t="inlineStr"/>
       <c r="H50" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
+          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I50" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J50" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J50" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
       <c r="K50" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L50" s="1" t="inlineStr"/>
@@ -2257,54 +2245,114 @@
       <c r="O50" s="1" t="inlineStr"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="inlineStr"/>
-      <c r="B51" s="2" t="inlineStr"/>
-      <c r="C51" s="2" t="inlineStr"/>
-      <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
-      <c r="H51" s="2" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr"/>
-      <c r="K51" s="2" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr"/>
-      <c r="M51" s="2" t="inlineStr"/>
-      <c r="N51" s="2" t="inlineStr"/>
-      <c r="O51" s="2" t="inlineStr"/>
+      <c r="A51" s="1" t="inlineStr"/>
+      <c r="B51" s="1" t="inlineStr"/>
+      <c r="C51" s="1" t="inlineStr"/>
+      <c r="D51" s="1" t="inlineStr"/>
+      <c r="E51" s="1" t="inlineStr"/>
+      <c r="F51" s="1" t="inlineStr"/>
+      <c r="G51" s="1" t="inlineStr"/>
+      <c r="H51" s="1" t="inlineStr">
+        <is>
+          <t>Tap a category in the media details metadata list. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="I51" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr">
+        <is>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="K51" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L51" s="1" t="inlineStr"/>
+      <c r="M51" s="1" t="inlineStr"/>
+      <c r="N51" s="1" t="inlineStr"/>
+      <c r="O51" s="1" t="inlineStr"/>
     </row>
     <row r="52">
-      <c r="A52" s="1" t="n">
+      <c r="A52" s="1" t="inlineStr"/>
+      <c r="B52" s="1" t="inlineStr"/>
+      <c r="C52" s="1" t="inlineStr"/>
+      <c r="D52" s="1" t="inlineStr"/>
+      <c r="E52" s="1" t="inlineStr"/>
+      <c r="F52" s="1" t="inlineStr"/>
+      <c r="G52" s="1" t="inlineStr"/>
+      <c r="H52" s="1" t="inlineStr">
+        <is>
+          <t>Tap the PARENT CATEGORIES tab on the category details screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I52" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K52" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L52" s="1" t="inlineStr"/>
+      <c r="M52" s="1" t="inlineStr"/>
+      <c r="N52" s="1" t="inlineStr"/>
+      <c r="O52" s="1" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="inlineStr"/>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr"/>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr"/>
+      <c r="M53" s="2" t="inlineStr"/>
+      <c r="N53" s="2" t="inlineStr"/>
+      <c r="O53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="B52" s="1" t="inlineStr">
+      <c r="B54" s="1" t="inlineStr">
         <is>
           <t>Wikimedia Commons</t>
         </is>
       </c>
-      <c r="C52" s="1" t="inlineStr">
+      <c r="C54" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D52" s="1" t="inlineStr">
-        <is>
-          <t>MC_HP</t>
-        </is>
-      </c>
-      <c r="E52" s="1" t="inlineStr">
-        <is>
-          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F52" s="1" t="inlineStr">
-        <is>
-          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
-Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="G52" s="1" t="inlineStr">
+      <c r="D54" s="1" t="inlineStr">
+        <is>
+          <t>LC_HP</t>
+        </is>
+      </c>
+      <c r="E54" s="1" t="inlineStr">
+        <is>
+          <t>The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F54" s="1" t="inlineStr"/>
+      <c r="G54" s="1" t="inlineStr">
         <is>
           <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
 2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
@@ -2323,107 +2371,41 @@
 15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
-      <c r="H52" s="1" t="inlineStr">
+      <c r="H54" s="1" t="inlineStr">
         <is>
           <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="I52" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J52" s="1" t="inlineStr">
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
         <is>
           <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="K52" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L52" s="1">
-        <f>IFERROR(COUNTIF(K52:K67,"CS")/COUNTA(K52:K67),"")</f>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L54" s="1">
+        <f>IFERROR(COUNTIF(K54:K68,"CS")/COUNTA(K54:K68),"")</f>
         <v/>
       </c>
-      <c r="M52" s="1">
-        <f>COUNTIF(K52:K67,"CS")/15</f>
+      <c r="M54" s="1">
+        <f>COUNTIF(K54:K68,"CS")/15</f>
         <v/>
       </c>
-      <c r="N52" s="1">
-        <f>IFERROR(2*(L52*M52)/(L52+M52),"")</f>
+      <c r="N54" s="1">
+        <f>IFERROR(2*(L54*M54)/(L54+M54),"")</f>
         <v/>
       </c>
-      <c r="O52" s="1" t="n">
+      <c r="O54" s="1" t="n">
         <v>15</v>
       </c>
-    </row>
-    <row r="53">
-      <c r="A53" s="1" t="inlineStr"/>
-      <c r="B53" s="1" t="inlineStr"/>
-      <c r="C53" s="1" t="inlineStr"/>
-      <c r="D53" s="1" t="inlineStr"/>
-      <c r="E53" s="1" t="inlineStr"/>
-      <c r="F53" s="1" t="inlineStr"/>
-      <c r="G53" s="1" t="inlineStr"/>
-      <c r="H53" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="I53" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J53" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="K53" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L53" s="1" t="inlineStr"/>
-      <c r="M53" s="1" t="inlineStr"/>
-      <c r="N53" s="1" t="inlineStr"/>
-      <c r="O53" s="1" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="1" t="inlineStr"/>
-      <c r="B54" s="1" t="inlineStr"/>
-      <c r="C54" s="1" t="inlineStr"/>
-      <c r="D54" s="1" t="inlineStr"/>
-      <c r="E54" s="1" t="inlineStr"/>
-      <c r="F54" s="1" t="inlineStr"/>
-      <c r="G54" s="1" t="inlineStr"/>
-      <c r="H54" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="I54" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J54" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="K54" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L54" s="1" t="inlineStr"/>
-      <c r="M54" s="1" t="inlineStr"/>
-      <c r="N54" s="1" t="inlineStr"/>
-      <c r="O54" s="1" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="1" t="inlineStr"/>
@@ -2435,7 +2417,7 @@
       <c r="G55" s="1" t="inlineStr"/>
       <c r="H55" s="1" t="inlineStr">
         <is>
-          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I55" s="1" t="inlineStr">
@@ -2445,7 +2427,7 @@
       </c>
       <c r="J55" s="1" t="inlineStr">
         <is>
-          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K55" s="1" t="inlineStr">
@@ -2468,7 +2450,7 @@
       <c r="G56" s="1" t="inlineStr"/>
       <c r="H56" s="1" t="inlineStr">
         <is>
-          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I56" s="1" t="inlineStr">
@@ -2478,7 +2460,7 @@
       </c>
       <c r="J56" s="1" t="inlineStr">
         <is>
-          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K56" s="1" t="inlineStr">
@@ -2501,7 +2483,7 @@
       <c r="G57" s="1" t="inlineStr"/>
       <c r="H57" s="1" t="inlineStr">
         <is>
-          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I57" s="1" t="inlineStr">
@@ -2511,7 +2493,7 @@
       </c>
       <c r="J57" s="1" t="inlineStr">
         <is>
-          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K57" s="1" t="inlineStr">
@@ -2534,7 +2516,7 @@
       <c r="G58" s="1" t="inlineStr"/>
       <c r="H58" s="1" t="inlineStr">
         <is>
-          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I58" s="1" t="inlineStr">
@@ -2544,7 +2526,7 @@
       </c>
       <c r="J58" s="1" t="inlineStr">
         <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K58" s="1" t="inlineStr">
@@ -2567,18 +2549,22 @@
       <c r="G59" s="1" t="inlineStr"/>
       <c r="H59" s="1" t="inlineStr">
         <is>
-          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
+          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I59" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J59" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J59" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+        </is>
+      </c>
       <c r="K59" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L59" s="1" t="inlineStr"/>
@@ -2596,7 +2582,7 @@
       <c r="G60" s="1" t="inlineStr"/>
       <c r="H60" s="1" t="inlineStr">
         <is>
-          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I60" s="1" t="inlineStr">
@@ -2629,7 +2615,7 @@
       <c r="G61" s="1" t="inlineStr"/>
       <c r="H61" s="1" t="inlineStr">
         <is>
-          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I61" s="1" t="inlineStr">
@@ -2662,7 +2648,7 @@
       <c r="G62" s="1" t="inlineStr"/>
       <c r="H62" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
         </is>
       </c>
       <c r="I62" s="1" t="inlineStr">
@@ -2691,7 +2677,7 @@
       <c r="G63" s="1" t="inlineStr"/>
       <c r="H63" s="1" t="inlineStr">
         <is>
-          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I63" s="1" t="inlineStr">
@@ -2724,7 +2710,7 @@
       <c r="G64" s="1" t="inlineStr"/>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I64" s="1" t="inlineStr">
@@ -2757,7 +2743,7 @@
       <c r="G65" s="1" t="inlineStr"/>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I65" s="1" t="inlineStr">
@@ -2790,7 +2776,7 @@
       <c r="G66" s="1" t="inlineStr"/>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I66" s="1" t="inlineStr">
@@ -2823,7 +2809,7 @@
       <c r="G67" s="1" t="inlineStr"/>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="I67" s="1" t="inlineStr">
@@ -2847,133 +2833,130 @@
       <c r="O67" s="1" t="inlineStr"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="inlineStr"/>
-      <c r="B68" s="2" t="inlineStr"/>
-      <c r="C68" s="2" t="inlineStr"/>
-      <c r="D68" s="2" t="inlineStr"/>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
-      <c r="H68" s="2" t="inlineStr"/>
-      <c r="I68" s="2" t="inlineStr"/>
-      <c r="J68" s="2" t="inlineStr"/>
-      <c r="K68" s="2" t="inlineStr"/>
-      <c r="L68" s="2" t="inlineStr"/>
-      <c r="M68" s="2" t="inlineStr"/>
-      <c r="N68" s="2" t="inlineStr"/>
-      <c r="O68" s="2" t="inlineStr"/>
+      <c r="A68" s="1" t="inlineStr"/>
+      <c r="B68" s="1" t="inlineStr"/>
+      <c r="C68" s="1" t="inlineStr"/>
+      <c r="D68" s="1" t="inlineStr"/>
+      <c r="E68" s="1" t="inlineStr"/>
+      <c r="F68" s="1" t="inlineStr"/>
+      <c r="G68" s="1" t="inlineStr"/>
+      <c r="H68" s="1" t="inlineStr">
+        <is>
+          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
+        </is>
+      </c>
+      <c r="I68" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J68" s="1" t="inlineStr"/>
+      <c r="K68" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L68" s="1" t="inlineStr"/>
+      <c r="M68" s="1" t="inlineStr"/>
+      <c r="N68" s="1" t="inlineStr"/>
+      <c r="O68" s="1" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B69" s="1" t="inlineStr">
-        <is>
-          <t>Family Finance</t>
-        </is>
-      </c>
-      <c r="C69" s="1" t="inlineStr">
+      <c r="A69" s="2" t="inlineStr"/>
+      <c r="B69" s="2" t="inlineStr"/>
+      <c r="C69" s="2" t="inlineStr"/>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr"/>
+      <c r="J69" s="2" t="inlineStr"/>
+      <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr"/>
+      <c r="M69" s="2" t="inlineStr"/>
+      <c r="N69" s="2" t="inlineStr"/>
+      <c r="O69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="1" t="n">
+        <v>135</v>
+      </c>
+      <c r="B70" s="1" t="inlineStr">
+        <is>
+          <t>Wikimedia Commons</t>
+        </is>
+      </c>
+      <c r="C70" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D69" s="1" t="inlineStr">
-        <is>
-          <t>HC_HP</t>
-        </is>
-      </c>
-      <c r="E69" s="1" t="inlineStr">
-        <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
-        </is>
-      </c>
-      <c r="F69" s="1" t="inlineStr">
-        <is>
-          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
-Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
-Expected Behavior: The appearance of the report should be changed to use percent values.</t>
-        </is>
-      </c>
-      <c r="G69" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
-      <c r="H69" s="1" t="inlineStr">
-        <is>
-          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
-        </is>
-      </c>
-      <c r="I69" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J69" s="1" t="inlineStr">
-        <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
-        </is>
-      </c>
-      <c r="K69" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L69" s="1">
-        <f>IFERROR(COUNTIF(K69:K76,"CS")/COUNTA(K69:K76),"")</f>
+      <c r="D70" s="1" t="inlineStr">
+        <is>
+          <t>MC_HP</t>
+        </is>
+      </c>
+      <c r="E70" s="1" t="inlineStr">
+        <is>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F70" s="1" t="inlineStr"/>
+      <c r="G70" s="1" t="inlineStr">
+        <is>
+          <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
+2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
+3. Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;
+4. Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;
+5. Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;
+6. Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;
+7. Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;
+8. Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;
+9. Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;
+10. Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;
+11. Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;
+12. Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;
+13. Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;
+14. Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;
+15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="I70" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J70" s="1" t="inlineStr">
+        <is>
+          <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L70" s="1">
+        <f>IFERROR(COUNTIF(K70:K85,"CS")/COUNTA(K70:K85),"")</f>
         <v/>
       </c>
-      <c r="M69" s="1">
-        <f>COUNTIF(K69:K76,"CS")/8</f>
+      <c r="M70" s="1">
+        <f>COUNTIF(K70:K85,"CS")/15</f>
         <v/>
       </c>
-      <c r="N69" s="1">
-        <f>IFERROR(2*(L69*M69)/(L69+M69),"")</f>
+      <c r="N70" s="1">
+        <f>IFERROR(2*(L70*M70)/(L70+M70),"")</f>
         <v/>
       </c>
-      <c r="O69" s="1" t="n">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="1" t="inlineStr"/>
-      <c r="B70" s="1" t="inlineStr"/>
-      <c r="C70" s="1" t="inlineStr"/>
-      <c r="D70" s="1" t="inlineStr"/>
-      <c r="E70" s="1" t="inlineStr"/>
-      <c r="F70" s="1" t="inlineStr"/>
-      <c r="G70" s="1" t="inlineStr"/>
-      <c r="H70" s="1" t="inlineStr">
-        <is>
-          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
-        </is>
-      </c>
-      <c r="I70" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J70" s="1" t="inlineStr">
-        <is>
-          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
-        </is>
-      </c>
-      <c r="K70" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L70" s="1" t="inlineStr"/>
-      <c r="M70" s="1" t="inlineStr"/>
-      <c r="N70" s="1" t="inlineStr"/>
-      <c r="O70" s="1" t="inlineStr"/>
+      <c r="O70" s="1" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="1" t="inlineStr"/>
@@ -2985,7 +2968,7 @@
       <c r="G71" s="1" t="inlineStr"/>
       <c r="H71" s="1" t="inlineStr">
         <is>
-          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I71" s="1" t="inlineStr">
@@ -2995,7 +2978,7 @@
       </c>
       <c r="J71" s="1" t="inlineStr">
         <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K71" s="1" t="inlineStr">
@@ -3018,7 +3001,7 @@
       <c r="G72" s="1" t="inlineStr"/>
       <c r="H72" s="1" t="inlineStr">
         <is>
-          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
+          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I72" s="1" t="inlineStr">
@@ -3028,7 +3011,7 @@
       </c>
       <c r="J72" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K72" s="1" t="inlineStr">
@@ -3051,7 +3034,7 @@
       <c r="G73" s="1" t="inlineStr"/>
       <c r="H73" s="1" t="inlineStr">
         <is>
-          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I73" s="1" t="inlineStr">
@@ -3061,7 +3044,7 @@
       </c>
       <c r="J73" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K73" s="1" t="inlineStr">
@@ -3084,7 +3067,7 @@
       <c r="G74" s="1" t="inlineStr"/>
       <c r="H74" s="1" t="inlineStr">
         <is>
-          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I74" s="1" t="inlineStr">
@@ -3094,7 +3077,7 @@
       </c>
       <c r="J74" s="1" t="inlineStr">
         <is>
-          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K74" s="1" t="inlineStr">
@@ -3117,7 +3100,7 @@
       <c r="G75" s="1" t="inlineStr"/>
       <c r="H75" s="1" t="inlineStr">
         <is>
-          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I75" s="1" t="inlineStr">
@@ -3127,7 +3110,7 @@
       </c>
       <c r="J75" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="K75" s="1" t="inlineStr">
@@ -3150,7 +3133,7 @@
       <c r="G76" s="1" t="inlineStr"/>
       <c r="H76" s="1" t="inlineStr">
         <is>
-          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
         </is>
       </c>
       <c r="I76" s="1" t="inlineStr">
@@ -3160,7 +3143,7 @@
       </c>
       <c r="J76" s="1" t="inlineStr">
         <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="K76" s="1" t="inlineStr">
@@ -3174,68 +3157,45 @@
       <c r="O76" s="1" t="inlineStr"/>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr"/>
-      <c r="B77" s="2" t="inlineStr"/>
-      <c r="C77" s="2" t="inlineStr"/>
-      <c r="D77" s="2" t="inlineStr"/>
-      <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr"/>
-      <c r="H77" s="2" t="inlineStr"/>
-      <c r="I77" s="2" t="inlineStr"/>
-      <c r="J77" s="2" t="inlineStr"/>
-      <c r="K77" s="2" t="inlineStr"/>
-      <c r="L77" s="2" t="inlineStr"/>
-      <c r="M77" s="2" t="inlineStr"/>
-      <c r="N77" s="2" t="inlineStr"/>
-      <c r="O77" s="2" t="inlineStr"/>
+      <c r="A77" s="1" t="inlineStr"/>
+      <c r="B77" s="1" t="inlineStr"/>
+      <c r="C77" s="1" t="inlineStr"/>
+      <c r="D77" s="1" t="inlineStr"/>
+      <c r="E77" s="1" t="inlineStr"/>
+      <c r="F77" s="1" t="inlineStr"/>
+      <c r="G77" s="1" t="inlineStr"/>
+      <c r="H77" s="1" t="inlineStr">
+        <is>
+          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
+        </is>
+      </c>
+      <c r="I77" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J77" s="1" t="inlineStr"/>
+      <c r="K77" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L77" s="1" t="inlineStr"/>
+      <c r="M77" s="1" t="inlineStr"/>
+      <c r="N77" s="1" t="inlineStr"/>
+      <c r="O77" s="1" t="inlineStr"/>
     </row>
     <row r="78">
-      <c r="A78" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B78" s="1" t="inlineStr">
-        <is>
-          <t>Family Finance</t>
-        </is>
-      </c>
-      <c r="C78" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D78" s="1" t="inlineStr">
-        <is>
-          <t>MC_MP</t>
-        </is>
-      </c>
-      <c r="E78" s="1" t="inlineStr">
-        <is>
-          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
-        </is>
-      </c>
-      <c r="F78" s="1" t="inlineStr">
-        <is>
-          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
-Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
-Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
-        </is>
-      </c>
-      <c r="G78" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
+      <c r="A78" s="1" t="inlineStr"/>
+      <c r="B78" s="1" t="inlineStr"/>
+      <c r="C78" s="1" t="inlineStr"/>
+      <c r="D78" s="1" t="inlineStr"/>
+      <c r="E78" s="1" t="inlineStr"/>
+      <c r="F78" s="1" t="inlineStr"/>
+      <c r="G78" s="1" t="inlineStr"/>
       <c r="H78" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I78" s="1" t="inlineStr">
@@ -3245,7 +3205,7 @@
       </c>
       <c r="J78" s="1" t="inlineStr">
         <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="K78" s="1" t="inlineStr">
@@ -3253,21 +3213,10 @@
           <t>CS</t>
         </is>
       </c>
-      <c r="L78" s="1">
-        <f>IFERROR(COUNTIF(K78:K84,"CS")/COUNTA(K78:K84),"")</f>
-        <v/>
-      </c>
-      <c r="M78" s="1">
-        <f>COUNTIF(K78:K84,"CS")/8</f>
-        <v/>
-      </c>
-      <c r="N78" s="1">
-        <f>IFERROR(2*(L78*M78)/(L78+M78),"")</f>
-        <v/>
-      </c>
-      <c r="O78" s="1" t="n">
-        <v>8</v>
-      </c>
+      <c r="L78" s="1" t="inlineStr"/>
+      <c r="M78" s="1" t="inlineStr"/>
+      <c r="N78" s="1" t="inlineStr"/>
+      <c r="O78" s="1" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="1" t="inlineStr"/>
@@ -3279,18 +3228,22 @@
       <c r="G79" s="1" t="inlineStr"/>
       <c r="H79" s="1" t="inlineStr">
         <is>
-          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I79" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J79" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J79" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
       <c r="K79" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L79" s="1" t="inlineStr"/>
@@ -3308,22 +3261,18 @@
       <c r="G80" s="1" t="inlineStr"/>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
         </is>
       </c>
       <c r="I80" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="inlineStr">
-        <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="inlineStr"/>
       <c r="K80" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L80" s="1" t="inlineStr"/>
@@ -3341,7 +3290,7 @@
       <c r="G81" s="1" t="inlineStr"/>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I81" s="1" t="inlineStr">
@@ -3351,7 +3300,7 @@
       </c>
       <c r="J81" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="K81" s="1" t="inlineStr">
@@ -3374,7 +3323,7 @@
       <c r="G82" s="1" t="inlineStr"/>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I82" s="1" t="inlineStr">
@@ -3384,7 +3333,7 @@
       </c>
       <c r="J82" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="K82" s="1" t="inlineStr">
@@ -3407,7 +3356,7 @@
       <c r="G83" s="1" t="inlineStr"/>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I83" s="1" t="inlineStr">
@@ -3417,7 +3366,7 @@
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="K83" s="1" t="inlineStr">
@@ -3440,7 +3389,7 @@
       <c r="G84" s="1" t="inlineStr"/>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>Tap "OK" to confirm the change. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I84" s="1" t="inlineStr">
@@ -3450,7 +3399,7 @@
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="K84" s="1" t="inlineStr">
@@ -3462,6 +3411,644 @@
       <c r="M84" s="1" t="inlineStr"/>
       <c r="N84" s="1" t="inlineStr"/>
       <c r="O84" s="1" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="1" t="inlineStr"/>
+      <c r="B85" s="1" t="inlineStr"/>
+      <c r="C85" s="1" t="inlineStr"/>
+      <c r="D85" s="1" t="inlineStr"/>
+      <c r="E85" s="1" t="inlineStr"/>
+      <c r="F85" s="1" t="inlineStr"/>
+      <c r="G85" s="1" t="inlineStr"/>
+      <c r="H85" s="1" t="inlineStr">
+        <is>
+          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I85" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J85" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K85" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L85" s="1" t="inlineStr"/>
+      <c r="M85" s="1" t="inlineStr"/>
+      <c r="N85" s="1" t="inlineStr"/>
+      <c r="O85" s="1" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr"/>
+      <c r="B86" s="2" t="inlineStr"/>
+      <c r="C86" s="2" t="inlineStr"/>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+      <c r="I86" s="2" t="inlineStr"/>
+      <c r="J86" s="2" t="inlineStr"/>
+      <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr"/>
+      <c r="M86" s="2" t="inlineStr"/>
+      <c r="N86" s="2" t="inlineStr"/>
+      <c r="O86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B87" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C87" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D87" s="1" t="inlineStr">
+        <is>
+          <t>HC_HP</t>
+        </is>
+      </c>
+      <c r="E87" s="1" t="inlineStr">
+        <is>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F87" s="1" t="inlineStr"/>
+      <c r="G87" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H87" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="I87" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J87" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K87" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L87" s="1">
+        <f>IFERROR(COUNTIF(K87:K94,"CS")/COUNTA(K87:K94),"")</f>
+        <v/>
+      </c>
+      <c r="M87" s="1">
+        <f>COUNTIF(K87:K94,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N87" s="1">
+        <f>IFERROR(2*(L87*M87)/(L87+M87),"")</f>
+        <v/>
+      </c>
+      <c r="O87" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="1" t="inlineStr"/>
+      <c r="B88" s="1" t="inlineStr"/>
+      <c r="C88" s="1" t="inlineStr"/>
+      <c r="D88" s="1" t="inlineStr"/>
+      <c r="E88" s="1" t="inlineStr"/>
+      <c r="F88" s="1" t="inlineStr"/>
+      <c r="G88" s="1" t="inlineStr"/>
+      <c r="H88" s="1" t="inlineStr">
+        <is>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="I88" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J88" s="1" t="inlineStr">
+        <is>
+          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
+      <c r="K88" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L88" s="1" t="inlineStr"/>
+      <c r="M88" s="1" t="inlineStr"/>
+      <c r="N88" s="1" t="inlineStr"/>
+      <c r="O88" s="1" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="1" t="inlineStr"/>
+      <c r="B89" s="1" t="inlineStr"/>
+      <c r="C89" s="1" t="inlineStr"/>
+      <c r="D89" s="1" t="inlineStr"/>
+      <c r="E89" s="1" t="inlineStr"/>
+      <c r="F89" s="1" t="inlineStr"/>
+      <c r="G89" s="1" t="inlineStr"/>
+      <c r="H89" s="1" t="inlineStr">
+        <is>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I89" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J89" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K89" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L89" s="1" t="inlineStr"/>
+      <c r="M89" s="1" t="inlineStr"/>
+      <c r="N89" s="1" t="inlineStr"/>
+      <c r="O89" s="1" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="1" t="inlineStr"/>
+      <c r="B90" s="1" t="inlineStr"/>
+      <c r="C90" s="1" t="inlineStr"/>
+      <c r="D90" s="1" t="inlineStr"/>
+      <c r="E90" s="1" t="inlineStr"/>
+      <c r="F90" s="1" t="inlineStr"/>
+      <c r="G90" s="1" t="inlineStr"/>
+      <c r="H90" s="1" t="inlineStr">
+        <is>
+          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
+        </is>
+      </c>
+      <c r="I90" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J90" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K90" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L90" s="1" t="inlineStr"/>
+      <c r="M90" s="1" t="inlineStr"/>
+      <c r="N90" s="1" t="inlineStr"/>
+      <c r="O90" s="1" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="1" t="inlineStr"/>
+      <c r="B91" s="1" t="inlineStr"/>
+      <c r="C91" s="1" t="inlineStr"/>
+      <c r="D91" s="1" t="inlineStr"/>
+      <c r="E91" s="1" t="inlineStr"/>
+      <c r="F91" s="1" t="inlineStr"/>
+      <c r="G91" s="1" t="inlineStr"/>
+      <c r="H91" s="1" t="inlineStr">
+        <is>
+          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I91" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J91" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K91" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L91" s="1" t="inlineStr"/>
+      <c r="M91" s="1" t="inlineStr"/>
+      <c r="N91" s="1" t="inlineStr"/>
+      <c r="O91" s="1" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="1" t="inlineStr"/>
+      <c r="B92" s="1" t="inlineStr"/>
+      <c r="C92" s="1" t="inlineStr"/>
+      <c r="D92" s="1" t="inlineStr"/>
+      <c r="E92" s="1" t="inlineStr"/>
+      <c r="F92" s="1" t="inlineStr"/>
+      <c r="G92" s="1" t="inlineStr"/>
+      <c r="H92" s="1" t="inlineStr">
+        <is>
+          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="I92" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J92" s="1" t="inlineStr">
+        <is>
+          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
+      <c r="K92" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L92" s="1" t="inlineStr"/>
+      <c r="M92" s="1" t="inlineStr"/>
+      <c r="N92" s="1" t="inlineStr"/>
+      <c r="O92" s="1" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="1" t="inlineStr"/>
+      <c r="B93" s="1" t="inlineStr"/>
+      <c r="C93" s="1" t="inlineStr"/>
+      <c r="D93" s="1" t="inlineStr"/>
+      <c r="E93" s="1" t="inlineStr"/>
+      <c r="F93" s="1" t="inlineStr"/>
+      <c r="G93" s="1" t="inlineStr"/>
+      <c r="H93" s="1" t="inlineStr">
+        <is>
+          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I93" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J93" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K93" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L93" s="1" t="inlineStr"/>
+      <c r="M93" s="1" t="inlineStr"/>
+      <c r="N93" s="1" t="inlineStr"/>
+      <c r="O93" s="1" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="1" t="inlineStr"/>
+      <c r="B94" s="1" t="inlineStr"/>
+      <c r="C94" s="1" t="inlineStr"/>
+      <c r="D94" s="1" t="inlineStr"/>
+      <c r="E94" s="1" t="inlineStr"/>
+      <c r="F94" s="1" t="inlineStr"/>
+      <c r="G94" s="1" t="inlineStr"/>
+      <c r="H94" s="1" t="inlineStr">
+        <is>
+          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I94" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J94" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K94" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L94" s="1" t="inlineStr"/>
+      <c r="M94" s="1" t="inlineStr"/>
+      <c r="N94" s="1" t="inlineStr"/>
+      <c r="O94" s="1" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr"/>
+      <c r="B95" s="2" t="inlineStr"/>
+      <c r="C95" s="2" t="inlineStr"/>
+      <c r="D95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+      <c r="H95" s="2" t="inlineStr"/>
+      <c r="I95" s="2" t="inlineStr"/>
+      <c r="J95" s="2" t="inlineStr"/>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr"/>
+      <c r="M95" s="2" t="inlineStr"/>
+      <c r="N95" s="2" t="inlineStr"/>
+      <c r="O95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B96" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C96" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D96" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E96" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F96" s="1" t="inlineStr"/>
+      <c r="G96" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H96" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+        </is>
+      </c>
+      <c r="I96" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J96" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K96" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L96" s="1">
+        <f>IFERROR(COUNTIF(K96:K102,"CS")/COUNTA(K96:K102),"")</f>
+        <v/>
+      </c>
+      <c r="M96" s="1">
+        <f>COUNTIF(K96:K102,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N96" s="1">
+        <f>IFERROR(2*(L96*M96)/(L96+M96),"")</f>
+        <v/>
+      </c>
+      <c r="O96" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="1" t="inlineStr"/>
+      <c r="B97" s="1" t="inlineStr"/>
+      <c r="C97" s="1" t="inlineStr"/>
+      <c r="D97" s="1" t="inlineStr"/>
+      <c r="E97" s="1" t="inlineStr"/>
+      <c r="F97" s="1" t="inlineStr"/>
+      <c r="G97" s="1" t="inlineStr"/>
+      <c r="H97" s="1" t="inlineStr">
+        <is>
+          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+        </is>
+      </c>
+      <c r="I97" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J97" s="1" t="inlineStr"/>
+      <c r="K97" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L97" s="1" t="inlineStr"/>
+      <c r="M97" s="1" t="inlineStr"/>
+      <c r="N97" s="1" t="inlineStr"/>
+      <c r="O97" s="1" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="1" t="inlineStr"/>
+      <c r="B98" s="1" t="inlineStr"/>
+      <c r="C98" s="1" t="inlineStr"/>
+      <c r="D98" s="1" t="inlineStr"/>
+      <c r="E98" s="1" t="inlineStr"/>
+      <c r="F98" s="1" t="inlineStr"/>
+      <c r="G98" s="1" t="inlineStr"/>
+      <c r="H98" s="1" t="inlineStr">
+        <is>
+          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I98" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J98" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K98" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L98" s="1" t="inlineStr"/>
+      <c r="M98" s="1" t="inlineStr"/>
+      <c r="N98" s="1" t="inlineStr"/>
+      <c r="O98" s="1" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="1" t="inlineStr"/>
+      <c r="B99" s="1" t="inlineStr"/>
+      <c r="C99" s="1" t="inlineStr"/>
+      <c r="D99" s="1" t="inlineStr"/>
+      <c r="E99" s="1" t="inlineStr"/>
+      <c r="F99" s="1" t="inlineStr"/>
+      <c r="G99" s="1" t="inlineStr"/>
+      <c r="H99" s="1" t="inlineStr">
+        <is>
+          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="I99" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J99" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K99" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L99" s="1" t="inlineStr"/>
+      <c r="M99" s="1" t="inlineStr"/>
+      <c r="N99" s="1" t="inlineStr"/>
+      <c r="O99" s="1" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="1" t="inlineStr"/>
+      <c r="B100" s="1" t="inlineStr"/>
+      <c r="C100" s="1" t="inlineStr"/>
+      <c r="D100" s="1" t="inlineStr"/>
+      <c r="E100" s="1" t="inlineStr"/>
+      <c r="F100" s="1" t="inlineStr"/>
+      <c r="G100" s="1" t="inlineStr"/>
+      <c r="H100" s="1" t="inlineStr">
+        <is>
+          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I100" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J100" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K100" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L100" s="1" t="inlineStr"/>
+      <c r="M100" s="1" t="inlineStr"/>
+      <c r="N100" s="1" t="inlineStr"/>
+      <c r="O100" s="1" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="1" t="inlineStr"/>
+      <c r="B101" s="1" t="inlineStr"/>
+      <c r="C101" s="1" t="inlineStr"/>
+      <c r="D101" s="1" t="inlineStr"/>
+      <c r="E101" s="1" t="inlineStr"/>
+      <c r="F101" s="1" t="inlineStr"/>
+      <c r="G101" s="1" t="inlineStr"/>
+      <c r="H101" s="1" t="inlineStr">
+        <is>
+          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I101" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J101" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K101" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L101" s="1" t="inlineStr"/>
+      <c r="M101" s="1" t="inlineStr"/>
+      <c r="N101" s="1" t="inlineStr"/>
+      <c r="O101" s="1" t="inlineStr"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="1" t="inlineStr"/>
+      <c r="B102" s="1" t="inlineStr"/>
+      <c r="C102" s="1" t="inlineStr"/>
+      <c r="D102" s="1" t="inlineStr"/>
+      <c r="E102" s="1" t="inlineStr"/>
+      <c r="F102" s="1" t="inlineStr"/>
+      <c r="G102" s="1" t="inlineStr"/>
+      <c r="H102" s="1" t="inlineStr">
+        <is>
+          <t>Tap "OK" to confirm the change. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I102" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J102" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K102" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L102" s="1" t="inlineStr"/>
+      <c r="M102" s="1" t="inlineStr"/>
+      <c r="N102" s="1" t="inlineStr"/>
+      <c r="O102" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3474,7 +4061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:L16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3555,11 +4142,11 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>10</v>
+        <v>135</v>
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>Material Files</t>
+          <t>Wikimedia Commons</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
@@ -3569,35 +4156,35 @@
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>HC_LP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr">
         <is>
-          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F2" s="1" t="inlineStr">
         <is>
-          <t>Title: FTP server restarts automatically after being stopped and the app is closed
-Observed Behavior: On the FTP server screen, if the user turns off the FTP server switch and then closes the app, the FTP server restarts automatically after stopping it and closing the app.
-Expected Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the category details screen, if the user taps the Parent Categories tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G2" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the server restarts automatically
-Triggering GUI Interaction: stops the FTP server and then closes the app
-Triggering Screen Reference: FTP server screen
-Correct Behavior: The FTP server should remain stopped</t>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
         </is>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the FTP server restarts automatically after stopping it and closing the app
-Triggering GUI Interactions: the user turns off the FTP server switch and then closes the app
-Triggering Screen Reference: On the FTP server screen
-Correct Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
+          <t>Buggy Behavior: a blank page is shown
+Triggering GUI Interactions: taps the Parent Categories tab
+Triggering Screen Reference: On the category details screen
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I2" s="1" t="inlineStr">
@@ -3612,7 +4199,7 @@
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>Correct</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="L2" s="1" t="inlineStr">
@@ -3651,21 +4238,15 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>LC_LP</t>
+          <t>HC_LP</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>It restarts on its own.</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr">
-        <is>
-          <t>Title: FTP server restarts automatically after being turned off and leaving the FTP server screen
-Observed Behavior: On the FTP server screen, if the user turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents, the FTP server is restarting on its own.
-Expected Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
-        </is>
-      </c>
+          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr"/>
       <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the server restarts automatically
@@ -3676,10 +4257,10 @@
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the FTP server is restarting on its own
-Triggering GUI Interactions: turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents
+          <t>Buggy Behavior: the FTP server restarts automatically after stopping it and closing the app
+Triggering GUI Interactions: the user turns off the FTP server switch and then closes the app
 Triggering Screen Reference: On the FTP server screen
-Correct Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
+Correct Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -3719,11 +4300,11 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>135</v>
+        <v>10</v>
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>Wikimedia Commons</t>
+          <t>Material Files</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
@@ -3733,35 +4314,29 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>HC_HP</t>
+          <t>LC_LP</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F6" s="1" t="inlineStr">
-        <is>
-          <t>Title: Parent Categories tab shows a blank page on the category details screen
-Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
+          <t>It restarts on its own.</t>
+        </is>
+      </c>
+      <c r="F6" s="1" t="inlineStr"/>
       <c r="G6" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: see a blank page
-Triggering GUI Interaction: clicks the Parent Categories tab
-Triggering Screen Reference: Category screen, Parent Categories tab
-Correct Behavior: The Parent Categories of the current category should be displayed</t>
+          <t>Buggy Behavior: the server restarts automatically
+Triggering GUI Interaction: stops the FTP server and then closes the app
+Triggering Screen Reference: FTP server screen
+Correct Behavior: The FTP server should remain stopped</t>
         </is>
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: a blank page is shown
-Triggering GUI Interactions: taps the PARENT CATEGORIES tab
-Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
-Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: the FTP server is restarting on its own
+Triggering GUI Interactions: turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents
+Triggering Screen Reference: On the FTP server screen
+Correct Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -3815,19 +4390,19 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>LC_HP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>The Parent Categories of the current category should be displayed.</t>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F8" s="1" t="inlineStr">
         <is>
-          <t>Title: Parent categories are not shown after selecting the PARENT CATEGORIES tab on a category details screen
-Observed Behavior: On the category details screen for "Focus stacking images of insects," if the user taps the "PARENT CATEGORIES" tab, the parent categories of the current category are not displayed.
-Expected Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="G8" s="1" t="inlineStr">
@@ -3840,10 +4415,10 @@
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the parent categories of the current category are not displayed
-Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
-Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
-Correct Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: a blank page is shown
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">
@@ -3858,7 +4433,7 @@
       </c>
       <c r="K8" s="1" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="L8" s="1" t="inlineStr">
@@ -3897,21 +4472,15 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>MC_HP</t>
+          <t>LC_HP</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr">
-        <is>
-          <t>Title: Tapping the Parent Categories tab on a category details screen opens a blank page
-Observed Behavior: On the Category Details screen, if the user taps the PARENT CATEGORIES tab, the app results in a blank page.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
+          <t>The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr"/>
       <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: see a blank page
@@ -3922,10 +4491,10 @@
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the app results in a blank page
-Triggering GUI Interactions: taps the PARENT CATEGORIES tab
-Triggering Screen Reference: On the Category Details screen
-Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: the parent categories of the current category are not displayed
+Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
+Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
+Correct Behavior: The parent categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I10" s="1" t="inlineStr">
@@ -3965,11 +4534,11 @@
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>Family Finance</t>
+          <t>Wikimedia Commons</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
@@ -3979,35 +4548,29 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>HC_HP</t>
+          <t>MC_HP</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
-        </is>
-      </c>
-      <c r="F12" s="1" t="inlineStr">
-        <is>
-          <t>Title: App crashes when applying both View values and Use percent values in the Incomes by Articles report display dialog
-Observed Behavior: On the Display of Incomes by Articles dialog of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
-Expected Behavior: The appearance of the report should be changed to use percent values.</t>
-        </is>
-      </c>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F12" s="1" t="inlineStr"/>
       <c r="G12" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the application crashes
-Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
-Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
-Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
         </is>
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the application crashes
-Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
-Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
-Correct Behavior: The appearance of the report should be changed to use percent values.</t>
+          <t>Buggy Behavior: the app results in a blank page
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
@@ -4022,7 +4585,7 @@
       </c>
       <c r="K12" s="1" t="inlineStr">
         <is>
-          <t>Correct</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="L12" s="1" t="inlineStr">
@@ -4061,21 +4624,15 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>MC_MP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
-        </is>
-      </c>
-      <c r="F14" s="1" t="inlineStr">
-        <is>
-          <t>Title: Selecting "Use percent values" for the Incomes by Articles report causes the app to crash
-Observed Behavior: On the Display of Incomes by Articles dialog, if the user taps the "Use percent values" checkbox, the application crashes.
-Expected Behavior: The application should change the report appearance to use percent values without crashing.</t>
-        </is>
-      </c>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F14" s="1" t="inlineStr"/>
       <c r="G14" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
@@ -4087,27 +4644,103 @@
       <c r="H14" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
+Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
+Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
+Correct Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
+      <c r="I14" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J14" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K14" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="L14" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr"/>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C16" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D16" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E16" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F16" s="1" t="inlineStr"/>
+      <c r="G16" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
+Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
+Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+        </is>
+      </c>
+      <c r="H16" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
 Triggering GUI Interactions: the user taps the "Use percent values" checkbox
 Triggering Screen Reference: On the Display of Incomes by Articles dialog
 Correct Behavior: The application should change the report appearance to use percent values without crashing.</t>
         </is>
       </c>
-      <c r="I14" s="1" t="inlineStr">
+      <c r="I16" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="J14" s="1" t="inlineStr">
+      <c r="J16" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="K14" s="1" t="inlineStr">
+      <c r="K16" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="L14" s="1" t="inlineStr">
+      <c r="L16" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -4124,7 +4757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4141,7 +4774,8 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="34" customWidth="1" min="13" max="13"/>
     <col width="32" customWidth="1" min="14" max="14"/>
-    <col width="26" customWidth="1" min="15" max="15"/>
+    <col width="34" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4212,10 +4846,15 @@
       </c>
       <c r="N1" t="inlineStr">
         <is>
-          <t>average_conversation_time_in_seconds</t>
+          <t>average_wall_clock_seconds_per_conv</t>
         </is>
       </c>
       <c r="O1" t="inlineStr">
+        <is>
+          <t>average_turn_processing_seconds_per_conv</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>average_conversation_turns</t>
         </is>
@@ -4272,13 +4911,16 @@
         <v/>
       </c>
       <c r="M2" t="n">
-        <v>77215</v>
+        <v>73273.75</v>
       </c>
       <c r="N2" t="n">
-        <v>65.56321271428571</v>
+        <v>32.391268</v>
       </c>
       <c r="O2" t="n">
-        <v>1.428571428571429</v>
+        <v>32.391268</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1.375</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor: dynamic gt_and_test_data consumption
</commit_message>
<xml_diff>
--- a/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
+++ b/Results/bugscribe_mutli-candidate_transitions_and_screen_descriptions/manual_review.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O102"/>
+  <dimension ref="A1:O111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1088,11 +1088,11 @@
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>Material Files</t>
+          <t>Family Finance</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
@@ -1102,28 +1102,36 @@
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>HC_LP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr">
         <is>
-          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
-        </is>
-      </c>
-      <c r="F18" s="1" t="inlineStr"/>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr">
+        <is>
+          <t>Title: App crashes when applying both View values and Use percent values in the Display of Incomes by Articles dialog
+Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
+Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
       <c r="G18" s="1" t="inlineStr">
         <is>
-          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
-2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
-3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
-4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
-5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
-6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
         </is>
       </c>
       <c r="H18" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
         </is>
       </c>
       <c r="I18" s="1" t="inlineStr">
@@ -1133,7 +1141,7 @@
       </c>
       <c r="J18" s="1" t="inlineStr">
         <is>
-          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
         </is>
       </c>
       <c r="K18" s="1" t="inlineStr">
@@ -1142,11 +1150,11 @@
         </is>
       </c>
       <c r="L18" s="1">
-        <f>IFERROR(COUNTIF(K18:K23,"CS")/COUNTA(K18:K23),"")</f>
+        <f>IFERROR(COUNTIF(K18:K25,"CS")/COUNTA(K18:K25),"")</f>
         <v/>
       </c>
       <c r="M18" s="1">
-        <f>COUNTIF(K18:K23,"CS")/6</f>
+        <f>COUNTIF(K18:K25,"CS")/8</f>
         <v/>
       </c>
       <c r="N18" s="1">
@@ -1154,7 +1162,7 @@
         <v/>
       </c>
       <c r="O18" s="1" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="19">
@@ -1167,7 +1175,7 @@
       <c r="G19" s="1" t="inlineStr"/>
       <c r="H19" s="1" t="inlineStr">
         <is>
-          <t>Grant the storage permission by tapping Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
         </is>
       </c>
       <c r="I19" s="1" t="inlineStr">
@@ -1177,7 +1185,7 @@
       </c>
       <c r="J19" s="1" t="inlineStr">
         <is>
-          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
         </is>
       </c>
       <c r="K19" s="1" t="inlineStr">
@@ -1200,7 +1208,7 @@
       <c r="G20" s="1" t="inlineStr"/>
       <c r="H20" s="1" t="inlineStr">
         <is>
-          <t>Open the navigation drawer from the main Files screen. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
         </is>
       </c>
       <c r="I20" s="1" t="inlineStr">
@@ -1210,7 +1218,7 @@
       </c>
       <c r="J20" s="1" t="inlineStr">
         <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
         </is>
       </c>
       <c r="K20" s="1" t="inlineStr">
@@ -1233,7 +1241,7 @@
       <c r="G21" s="1" t="inlineStr"/>
       <c r="H21" s="1" t="inlineStr">
         <is>
-          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+          <t>Select Incomes by Articles. &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
         </is>
       </c>
       <c r="I21" s="1" t="inlineStr">
@@ -1243,7 +1251,7 @@
       </c>
       <c r="J21" s="1" t="inlineStr">
         <is>
-          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
         </is>
       </c>
       <c r="K21" s="1" t="inlineStr">
@@ -1266,7 +1274,7 @@
       <c r="G22" s="1" t="inlineStr"/>
       <c r="H22" s="1" t="inlineStr">
         <is>
-          <t>On the FTP server screen, tap the ON switch to stop the FTP server. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
+          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
         </is>
       </c>
       <c r="I22" s="1" t="inlineStr">
@@ -1276,7 +1284,7 @@
       </c>
       <c r="J22" s="1" t="inlineStr">
         <is>
-          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
         </is>
       </c>
       <c r="K22" s="1" t="inlineStr">
@@ -1299,18 +1307,22 @@
       <c r="G23" s="1" t="inlineStr"/>
       <c r="H23" s="1" t="inlineStr">
         <is>
-          <t>Close the app by pressing Back from the FTP server screen. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
+          <t>Check View values. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
         </is>
       </c>
       <c r="I23" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J23" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J23" s="1" t="inlineStr">
+        <is>
+          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+        </is>
+      </c>
       <c r="K23" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L23" s="1" t="inlineStr"/>
@@ -1319,48 +1331,114 @@
       <c r="O23" s="1" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr"/>
-      <c r="B24" s="2" t="inlineStr"/>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-      <c r="H24" s="2" t="inlineStr"/>
-      <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
-      <c r="L24" s="2" t="inlineStr"/>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
+      <c r="A24" s="1" t="inlineStr"/>
+      <c r="B24" s="1" t="inlineStr"/>
+      <c r="C24" s="1" t="inlineStr"/>
+      <c r="D24" s="1" t="inlineStr"/>
+      <c r="E24" s="1" t="inlineStr"/>
+      <c r="F24" s="1" t="inlineStr"/>
+      <c r="G24" s="1" t="inlineStr"/>
+      <c r="H24" s="1" t="inlineStr">
+        <is>
+          <t>Check Use percent values. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I24" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J24" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K24" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L24" s="1" t="inlineStr"/>
+      <c r="M24" s="1" t="inlineStr"/>
+      <c r="N24" s="1" t="inlineStr"/>
+      <c r="O24" s="1" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="1" t="n">
+      <c r="A25" s="1" t="inlineStr"/>
+      <c r="B25" s="1" t="inlineStr"/>
+      <c r="C25" s="1" t="inlineStr"/>
+      <c r="D25" s="1" t="inlineStr"/>
+      <c r="E25" s="1" t="inlineStr"/>
+      <c r="F25" s="1" t="inlineStr"/>
+      <c r="G25" s="1" t="inlineStr"/>
+      <c r="H25" s="1" t="inlineStr">
+        <is>
+          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I25" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J25" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K25" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L25" s="1" t="inlineStr"/>
+      <c r="M25" s="1" t="inlineStr"/>
+      <c r="N25" s="1" t="inlineStr"/>
+      <c r="O25" s="1" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="2" t="inlineStr"/>
+      <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr"/>
+      <c r="M26" s="2" t="inlineStr"/>
+      <c r="N26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Material Files</t>
         </is>
       </c>
-      <c r="C25" s="1" t="inlineStr">
+      <c r="C27" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D25" s="1" t="inlineStr">
-        <is>
-          <t>LC_LP</t>
-        </is>
-      </c>
-      <c r="E25" s="1" t="inlineStr">
-        <is>
-          <t>It restarts on its own.</t>
-        </is>
-      </c>
-      <c r="F25" s="1" t="inlineStr"/>
-      <c r="G25" s="1" t="inlineStr">
+      <c r="D27" s="1" t="inlineStr">
+        <is>
+          <t>HC_LP</t>
+        </is>
+      </c>
+      <c r="E27" s="1" t="inlineStr">
+        <is>
+          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
+        </is>
+      </c>
+      <c r="F27" s="1" t="inlineStr"/>
+      <c r="G27" s="1" t="inlineStr">
         <is>
           <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
 2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
@@ -1370,107 +1448,41 @@
 6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
         </is>
       </c>
-      <c r="H25" s="1" t="inlineStr">
+      <c r="H27" s="1" t="inlineStr">
         <is>
           <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
         </is>
       </c>
-      <c r="I25" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J25" s="1" t="inlineStr">
+      <c r="I27" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J27" s="1" t="inlineStr">
         <is>
           <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
         </is>
       </c>
-      <c r="K25" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L25" s="1">
-        <f>IFERROR(COUNTIF(K25:K34,"CS")/COUNTA(K25:K34),"")</f>
+      <c r="K27" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L27" s="1">
+        <f>IFERROR(COUNTIF(K27:K32,"CS")/COUNTA(K27:K32),"")</f>
         <v/>
       </c>
-      <c r="M25" s="1">
-        <f>COUNTIF(K25:K34,"CS")/6</f>
+      <c r="M27" s="1">
+        <f>COUNTIF(K27:K32,"CS")/6</f>
         <v/>
       </c>
-      <c r="N25" s="1">
-        <f>IFERROR(2*(L25*M25)/(L25+M25),"")</f>
+      <c r="N27" s="1">
+        <f>IFERROR(2*(L27*M27)/(L27+M27),"")</f>
         <v/>
       </c>
-      <c r="O25" s="1" t="n">
+      <c r="O27" s="1" t="n">
         <v>6</v>
       </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="1" t="inlineStr"/>
-      <c r="B26" s="1" t="inlineStr"/>
-      <c r="C26" s="1" t="inlineStr"/>
-      <c r="D26" s="1" t="inlineStr"/>
-      <c r="E26" s="1" t="inlineStr"/>
-      <c r="F26" s="1" t="inlineStr"/>
-      <c r="G26" s="1" t="inlineStr"/>
-      <c r="H26" s="1" t="inlineStr">
-        <is>
-          <t>On the permission dialog, tap Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
-        </is>
-      </c>
-      <c r="I26" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J26" s="1" t="inlineStr">
-        <is>
-          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
-        </is>
-      </c>
-      <c r="K26" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L26" s="1" t="inlineStr"/>
-      <c r="M26" s="1" t="inlineStr"/>
-      <c r="N26" s="1" t="inlineStr"/>
-      <c r="O26" s="1" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="1" t="inlineStr"/>
-      <c r="B27" s="1" t="inlineStr"/>
-      <c r="C27" s="1" t="inlineStr"/>
-      <c r="D27" s="1" t="inlineStr"/>
-      <c r="E27" s="1" t="inlineStr"/>
-      <c r="F27" s="1" t="inlineStr"/>
-      <c r="G27" s="1" t="inlineStr"/>
-      <c r="H27" s="1" t="inlineStr">
-        <is>
-          <t>Open the navigation menu by tapping Navigate up. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
-        </is>
-      </c>
-      <c r="I27" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J27" s="1" t="inlineStr">
-        <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
-        </is>
-      </c>
-      <c r="K27" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L27" s="1" t="inlineStr"/>
-      <c r="M27" s="1" t="inlineStr"/>
-      <c r="N27" s="1" t="inlineStr"/>
-      <c r="O27" s="1" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="1" t="inlineStr"/>
@@ -1482,7 +1494,7 @@
       <c r="G28" s="1" t="inlineStr"/>
       <c r="H28" s="1" t="inlineStr">
         <is>
-          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+          <t>Grant the storage permission by tapping Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
         </is>
       </c>
       <c r="I28" s="1" t="inlineStr">
@@ -1492,7 +1504,7 @@
       </c>
       <c r="J28" s="1" t="inlineStr">
         <is>
-          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
         </is>
       </c>
       <c r="K28" s="1" t="inlineStr">
@@ -1515,7 +1527,7 @@
       <c r="G29" s="1" t="inlineStr"/>
       <c r="H29" s="1" t="inlineStr">
         <is>
-          <t>Tap the FTP server status switch while it is OFF to turn it ON. &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+          <t>Open the navigation drawer from the main Files screen. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="I29" s="1" t="inlineStr">
@@ -1525,7 +1537,7 @@
       </c>
       <c r="J29" s="1" t="inlineStr">
         <is>
-          <t>Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
         </is>
       </c>
       <c r="K29" s="1" t="inlineStr">
@@ -1548,7 +1560,7 @@
       <c r="G30" s="1" t="inlineStr"/>
       <c r="H30" s="1" t="inlineStr">
         <is>
-          <t>Tap the FTP server status switch while it is ON to turn it OFF. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
+          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="I30" s="1" t="inlineStr">
@@ -1558,7 +1570,7 @@
       </c>
       <c r="J30" s="1" t="inlineStr">
         <is>
-          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
+          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
         </is>
       </c>
       <c r="K30" s="1" t="inlineStr">
@@ -1581,18 +1593,22 @@
       <c r="G31" s="1" t="inlineStr"/>
       <c r="H31" s="1" t="inlineStr">
         <is>
-          <t>Leave the FTP server screen by tapping Navigate up. &lt;f5deb5a7a067fcecd183ba802aa26e2dfb3c5e38306d9407fd3b178866210afb&gt;</t>
+          <t>On the FTP server screen, tap the ON switch to stop the FTP server. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
         </is>
       </c>
       <c r="I31" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J31" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J31" s="1" t="inlineStr">
+        <is>
+          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
+        </is>
+      </c>
       <c r="K31" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L31" s="1" t="inlineStr"/>
@@ -1610,7 +1626,7 @@
       <c r="G32" s="1" t="inlineStr"/>
       <c r="H32" s="1" t="inlineStr">
         <is>
-          <t>Tap the list item to return to the FTP server screen path context. &lt;6766d1c12b54808176b7d8e110b78ee25e2843492f806acedcc0d8e1da70972c&gt;</t>
+          <t>Close the app by pressing Back from the FTP server screen. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
         </is>
       </c>
       <c r="I32" s="1" t="inlineStr">
@@ -1630,112 +1646,423 @@
       <c r="O32" s="1" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="1" t="inlineStr"/>
-      <c r="B33" s="1" t="inlineStr"/>
-      <c r="C33" s="1" t="inlineStr"/>
-      <c r="D33" s="1" t="inlineStr"/>
-      <c r="E33" s="1" t="inlineStr"/>
-      <c r="F33" s="1" t="inlineStr"/>
-      <c r="G33" s="1" t="inlineStr"/>
-      <c r="H33" s="1" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr"/>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr"/>
+      <c r="J33" s="2" t="inlineStr"/>
+      <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr"/>
+      <c r="M33" s="2" t="inlineStr"/>
+      <c r="N33" s="2" t="inlineStr"/>
+      <c r="O33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B34" s="1" t="inlineStr">
+        <is>
+          <t>Material Files</t>
+        </is>
+      </c>
+      <c r="C34" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D34" s="1" t="inlineStr">
+        <is>
+          <t>LC_LP</t>
+        </is>
+      </c>
+      <c r="E34" s="1" t="inlineStr">
+        <is>
+          <t>It restarts on its own.</t>
+        </is>
+      </c>
+      <c r="F34" s="1" t="inlineStr"/>
+      <c r="G34" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;
+2. Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;
+3. Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;
+4. Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;
+5. Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;
+6. Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="H34" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+        </is>
+      </c>
+      <c r="I34" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J34" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;aa09f6aef3409759f67d672c9efcbd64d8f3b0ee61cf3e8d197f0539e34430d2&gt;</t>
+        </is>
+      </c>
+      <c r="K34" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L34" s="1">
+        <f>IFERROR(COUNTIF(K34:K43,"CS")/COUNTA(K34:K43),"")</f>
+        <v/>
+      </c>
+      <c r="M34" s="1">
+        <f>COUNTIF(K34:K43,"CS")/6</f>
+        <v/>
+      </c>
+      <c r="N34" s="1">
+        <f>IFERROR(2*(L34*M34)/(L34+M34),"")</f>
+        <v/>
+      </c>
+      <c r="O34" s="1" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="1" t="inlineStr"/>
+      <c r="B35" s="1" t="inlineStr"/>
+      <c r="C35" s="1" t="inlineStr"/>
+      <c r="D35" s="1" t="inlineStr"/>
+      <c r="E35" s="1" t="inlineStr"/>
+      <c r="F35" s="1" t="inlineStr"/>
+      <c r="G35" s="1" t="inlineStr"/>
+      <c r="H35" s="1" t="inlineStr">
+        <is>
+          <t>On the permission dialog, tap Allow. &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+        </is>
+      </c>
+      <c r="I35" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J35" s="1" t="inlineStr">
+        <is>
+          <t>Click allow &lt;9253ef287211a96261d15d2522d1499f880b411f5e49851b98bae34f3403ab9d&gt;</t>
+        </is>
+      </c>
+      <c r="K35" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L35" s="1" t="inlineStr"/>
+      <c r="M35" s="1" t="inlineStr"/>
+      <c r="N35" s="1" t="inlineStr"/>
+      <c r="O35" s="1" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="1" t="inlineStr"/>
+      <c r="B36" s="1" t="inlineStr"/>
+      <c r="C36" s="1" t="inlineStr"/>
+      <c r="D36" s="1" t="inlineStr"/>
+      <c r="E36" s="1" t="inlineStr"/>
+      <c r="F36" s="1" t="inlineStr"/>
+      <c r="G36" s="1" t="inlineStr"/>
+      <c r="H36" s="1" t="inlineStr">
+        <is>
+          <t>Open the navigation menu by tapping Navigate up. &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
+        </is>
+      </c>
+      <c r="I36" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J36" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;3abd760d81519f7d0b2fe5daa74c918b40f9496bef2bf776dd7b0d8e95a47b49&gt;</t>
+        </is>
+      </c>
+      <c r="K36" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L36" s="1" t="inlineStr"/>
+      <c r="M36" s="1" t="inlineStr"/>
+      <c r="N36" s="1" t="inlineStr"/>
+      <c r="O36" s="1" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="1" t="inlineStr"/>
+      <c r="B37" s="1" t="inlineStr"/>
+      <c r="C37" s="1" t="inlineStr"/>
+      <c r="D37" s="1" t="inlineStr"/>
+      <c r="E37" s="1" t="inlineStr"/>
+      <c r="F37" s="1" t="inlineStr"/>
+      <c r="G37" s="1" t="inlineStr"/>
+      <c r="H37" s="1" t="inlineStr">
+        <is>
+          <t>Select FTP server from the navigation drawer. &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+        </is>
+      </c>
+      <c r="I37" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J37" s="1" t="inlineStr">
+        <is>
+          <t>Click FTP server &lt;ed4ddd149d2da1bda9c6a957048313602988bce3f183bd199efeacece662aeec&gt;</t>
+        </is>
+      </c>
+      <c r="K37" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L37" s="1" t="inlineStr"/>
+      <c r="M37" s="1" t="inlineStr"/>
+      <c r="N37" s="1" t="inlineStr"/>
+      <c r="O37" s="1" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="1" t="inlineStr"/>
+      <c r="B38" s="1" t="inlineStr"/>
+      <c r="C38" s="1" t="inlineStr"/>
+      <c r="D38" s="1" t="inlineStr"/>
+      <c r="E38" s="1" t="inlineStr"/>
+      <c r="F38" s="1" t="inlineStr"/>
+      <c r="G38" s="1" t="inlineStr"/>
+      <c r="H38" s="1" t="inlineStr">
+        <is>
+          <t>Tap the FTP server status switch while it is OFF to turn it ON. &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="I38" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J38" s="1" t="inlineStr">
+        <is>
+          <t>Click the status toggle button (switch server off) &lt;5f369cd30bd1e5644d294c31e5ff58277cad40b2633f69cc4105944721df8b1b&gt;</t>
+        </is>
+      </c>
+      <c r="K38" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L38" s="1" t="inlineStr"/>
+      <c r="M38" s="1" t="inlineStr"/>
+      <c r="N38" s="1" t="inlineStr"/>
+      <c r="O38" s="1" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="1" t="inlineStr"/>
+      <c r="B39" s="1" t="inlineStr"/>
+      <c r="C39" s="1" t="inlineStr"/>
+      <c r="D39" s="1" t="inlineStr"/>
+      <c r="E39" s="1" t="inlineStr"/>
+      <c r="F39" s="1" t="inlineStr"/>
+      <c r="G39" s="1" t="inlineStr"/>
+      <c r="H39" s="1" t="inlineStr">
+        <is>
+          <t>Tap the FTP server status switch while it is ON to turn it OFF. &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5&gt;</t>
+        </is>
+      </c>
+      <c r="I39" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J39" s="1" t="inlineStr">
+        <is>
+          <t>Click the status toggle button (switch server on) &lt;8453ee6186ad267c55c0f443ad2d1644911453cf4f005a06837b415345db6be5 &gt;</t>
+        </is>
+      </c>
+      <c r="K39" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L39" s="1" t="inlineStr"/>
+      <c r="M39" s="1" t="inlineStr"/>
+      <c r="N39" s="1" t="inlineStr"/>
+      <c r="O39" s="1" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="1" t="inlineStr"/>
+      <c r="B40" s="1" t="inlineStr"/>
+      <c r="C40" s="1" t="inlineStr"/>
+      <c r="D40" s="1" t="inlineStr"/>
+      <c r="E40" s="1" t="inlineStr"/>
+      <c r="F40" s="1" t="inlineStr"/>
+      <c r="G40" s="1" t="inlineStr"/>
+      <c r="H40" s="1" t="inlineStr">
+        <is>
+          <t>Leave the FTP server screen by tapping Navigate up. &lt;f5deb5a7a067fcecd183ba802aa26e2dfb3c5e38306d9407fd3b178866210afb&gt;</t>
+        </is>
+      </c>
+      <c r="I40" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J40" s="1" t="inlineStr"/>
+      <c r="K40" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L40" s="1" t="inlineStr"/>
+      <c r="M40" s="1" t="inlineStr"/>
+      <c r="N40" s="1" t="inlineStr"/>
+      <c r="O40" s="1" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="1" t="inlineStr"/>
+      <c r="B41" s="1" t="inlineStr"/>
+      <c r="C41" s="1" t="inlineStr"/>
+      <c r="D41" s="1" t="inlineStr"/>
+      <c r="E41" s="1" t="inlineStr"/>
+      <c r="F41" s="1" t="inlineStr"/>
+      <c r="G41" s="1" t="inlineStr"/>
+      <c r="H41" s="1" t="inlineStr">
+        <is>
+          <t>Tap the list item to return to the FTP server screen path context. &lt;6766d1c12b54808176b7d8e110b78ee25e2843492f806acedcc0d8e1da70972c&gt;</t>
+        </is>
+      </c>
+      <c r="I41" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J41" s="1" t="inlineStr"/>
+      <c r="K41" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L41" s="1" t="inlineStr"/>
+      <c r="M41" s="1" t="inlineStr"/>
+      <c r="N41" s="1" t="inlineStr"/>
+      <c r="O41" s="1" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="1" t="inlineStr"/>
+      <c r="B42" s="1" t="inlineStr"/>
+      <c r="C42" s="1" t="inlineStr"/>
+      <c r="D42" s="1" t="inlineStr"/>
+      <c r="E42" s="1" t="inlineStr"/>
+      <c r="F42" s="1" t="inlineStr"/>
+      <c r="G42" s="1" t="inlineStr"/>
+      <c r="H42" s="1" t="inlineStr">
         <is>
           <t>Open Recents using the system Back/Recents control. &lt;944abf1e97748f2436418aea5aa65a35e80ea307f807f0264ae85d2c80188e7c&gt;</t>
         </is>
       </c>
-      <c r="I33" s="1" t="inlineStr">
+      <c r="I42" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="J33" s="1" t="inlineStr"/>
-      <c r="K33" s="1" t="inlineStr">
+      <c r="J42" s="1" t="inlineStr"/>
+      <c r="K42" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="L33" s="1" t="inlineStr"/>
-      <c r="M33" s="1" t="inlineStr"/>
-      <c r="N33" s="1" t="inlineStr"/>
-      <c r="O33" s="1" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="1" t="inlineStr"/>
-      <c r="B34" s="1" t="inlineStr"/>
-      <c r="C34" s="1" t="inlineStr"/>
-      <c r="D34" s="1" t="inlineStr"/>
-      <c r="E34" s="1" t="inlineStr"/>
-      <c r="F34" s="1" t="inlineStr"/>
-      <c r="G34" s="1" t="inlineStr"/>
-      <c r="H34" s="1" t="inlineStr">
+      <c r="L42" s="1" t="inlineStr"/>
+      <c r="M42" s="1" t="inlineStr"/>
+      <c r="N42" s="1" t="inlineStr"/>
+      <c r="O42" s="1" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="1" t="inlineStr"/>
+      <c r="B43" s="1" t="inlineStr"/>
+      <c r="C43" s="1" t="inlineStr"/>
+      <c r="D43" s="1" t="inlineStr"/>
+      <c r="E43" s="1" t="inlineStr"/>
+      <c r="F43" s="1" t="inlineStr"/>
+      <c r="G43" s="1" t="inlineStr"/>
+      <c r="H43" s="1" t="inlineStr">
         <is>
           <t>Dismiss the Files app task from Recents. &lt;b05234dc13810ef197b494fe9ce3b3d6e6927d53c722ad904f3dc53e425da84c&gt;</t>
         </is>
       </c>
-      <c r="I34" s="1" t="inlineStr">
+      <c r="I43" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="J34" s="1" t="inlineStr"/>
-      <c r="K34" s="1" t="inlineStr">
+      <c r="J43" s="1" t="inlineStr"/>
+      <c r="K43" s="1" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="L34" s="1" t="inlineStr"/>
-      <c r="M34" s="1" t="inlineStr"/>
-      <c r="N34" s="1" t="inlineStr"/>
-      <c r="O34" s="1" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr"/>
-      <c r="B35" s="2" t="inlineStr"/>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-      <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
-      <c r="M35" s="2" t="inlineStr"/>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="1" t="n">
+      <c r="L43" s="1" t="inlineStr"/>
+      <c r="M43" s="1" t="inlineStr"/>
+      <c r="N43" s="1" t="inlineStr"/>
+      <c r="O43" s="1" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr"/>
+      <c r="J44" s="2" t="inlineStr"/>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="B36" s="1" t="inlineStr">
+      <c r="B45" s="1" t="inlineStr">
         <is>
           <t>Wikimedia Commons</t>
         </is>
       </c>
-      <c r="C36" s="1" t="inlineStr">
+      <c r="C45" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D36" s="1" t="inlineStr">
+      <c r="D45" s="1" t="inlineStr">
         <is>
           <t>HC_HP</t>
         </is>
       </c>
-      <c r="E36" s="1" t="inlineStr">
+      <c r="E45" s="1" t="inlineStr">
         <is>
           <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
-      <c r="F36" s="1" t="inlineStr">
+      <c r="F45" s="1" t="inlineStr">
         <is>
           <t>Title: Parent Categories tab opens a blank page on the category details screen
 Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
 Expected Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
-      <c r="G36" s="1" t="inlineStr">
+      <c r="G45" s="1" t="inlineStr">
         <is>
           <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
 2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
@@ -1754,330 +2081,41 @@
 15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
-      <c r="H36" s="1" t="inlineStr">
+      <c r="H45" s="1" t="inlineStr">
         <is>
           <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="I36" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J36" s="1" t="inlineStr">
+      <c r="I45" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J45" s="1" t="inlineStr">
         <is>
           <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="K36" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L36" s="1">
-        <f>IFERROR(COUNTIF(K36:K52,"CS")/COUNTA(K36:K52),"")</f>
+      <c r="K45" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L45" s="1">
+        <f>IFERROR(COUNTIF(K45:K61,"CS")/COUNTA(K45:K61),"")</f>
         <v/>
       </c>
-      <c r="M36" s="1">
-        <f>COUNTIF(K36:K52,"CS")/15</f>
+      <c r="M45" s="1">
+        <f>COUNTIF(K45:K61,"CS")/15</f>
         <v/>
       </c>
-      <c r="N36" s="1">
-        <f>IFERROR(2*(L36*M36)/(L36+M36),"")</f>
+      <c r="N45" s="1">
+        <f>IFERROR(2*(L45*M45)/(L45+M45),"")</f>
         <v/>
       </c>
-      <c r="O36" s="1" t="n">
+      <c r="O45" s="1" t="n">
         <v>15</v>
       </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="inlineStr"/>
-      <c r="B37" s="1" t="inlineStr"/>
-      <c r="C37" s="1" t="inlineStr"/>
-      <c r="D37" s="1" t="inlineStr"/>
-      <c r="E37" s="1" t="inlineStr"/>
-      <c r="F37" s="1" t="inlineStr"/>
-      <c r="G37" s="1" t="inlineStr"/>
-      <c r="H37" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="I37" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J37" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="K37" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L37" s="1" t="inlineStr"/>
-      <c r="M37" s="1" t="inlineStr"/>
-      <c r="N37" s="1" t="inlineStr"/>
-      <c r="O37" s="1" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr"/>
-      <c r="B38" s="1" t="inlineStr"/>
-      <c r="C38" s="1" t="inlineStr"/>
-      <c r="D38" s="1" t="inlineStr"/>
-      <c r="E38" s="1" t="inlineStr"/>
-      <c r="F38" s="1" t="inlineStr"/>
-      <c r="G38" s="1" t="inlineStr"/>
-      <c r="H38" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="I38" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J38" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="K38" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L38" s="1" t="inlineStr"/>
-      <c r="M38" s="1" t="inlineStr"/>
-      <c r="N38" s="1" t="inlineStr"/>
-      <c r="O38" s="1" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="inlineStr"/>
-      <c r="B39" s="1" t="inlineStr"/>
-      <c r="C39" s="1" t="inlineStr"/>
-      <c r="D39" s="1" t="inlineStr"/>
-      <c r="E39" s="1" t="inlineStr"/>
-      <c r="F39" s="1" t="inlineStr"/>
-      <c r="G39" s="1" t="inlineStr"/>
-      <c r="H39" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="I39" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J39" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="K39" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L39" s="1" t="inlineStr"/>
-      <c r="M39" s="1" t="inlineStr"/>
-      <c r="N39" s="1" t="inlineStr"/>
-      <c r="O39" s="1" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="1" t="inlineStr"/>
-      <c r="B40" s="1" t="inlineStr"/>
-      <c r="C40" s="1" t="inlineStr"/>
-      <c r="D40" s="1" t="inlineStr"/>
-      <c r="E40" s="1" t="inlineStr"/>
-      <c r="F40" s="1" t="inlineStr"/>
-      <c r="G40" s="1" t="inlineStr"/>
-      <c r="H40" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="I40" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J40" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="K40" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L40" s="1" t="inlineStr"/>
-      <c r="M40" s="1" t="inlineStr"/>
-      <c r="N40" s="1" t="inlineStr"/>
-      <c r="O40" s="1" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="1" t="inlineStr"/>
-      <c r="B41" s="1" t="inlineStr"/>
-      <c r="C41" s="1" t="inlineStr"/>
-      <c r="D41" s="1" t="inlineStr"/>
-      <c r="E41" s="1" t="inlineStr"/>
-      <c r="F41" s="1" t="inlineStr"/>
-      <c r="G41" s="1" t="inlineStr"/>
-      <c r="H41" s="1" t="inlineStr">
-        <is>
-          <t>Tap YES! on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="I41" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J41" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="K41" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L41" s="1" t="inlineStr"/>
-      <c r="M41" s="1" t="inlineStr"/>
-      <c r="N41" s="1" t="inlineStr"/>
-      <c r="O41" s="1" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="1" t="inlineStr"/>
-      <c r="B42" s="1" t="inlineStr"/>
-      <c r="C42" s="1" t="inlineStr"/>
-      <c r="D42" s="1" t="inlineStr"/>
-      <c r="E42" s="1" t="inlineStr"/>
-      <c r="F42" s="1" t="inlineStr"/>
-      <c r="G42" s="1" t="inlineStr"/>
-      <c r="H42" s="1" t="inlineStr">
-        <is>
-          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
-        </is>
-      </c>
-      <c r="I42" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J42" s="1" t="inlineStr"/>
-      <c r="K42" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L42" s="1" t="inlineStr"/>
-      <c r="M42" s="1" t="inlineStr"/>
-      <c r="N42" s="1" t="inlineStr"/>
-      <c r="O42" s="1" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="1" t="inlineStr"/>
-      <c r="B43" s="1" t="inlineStr"/>
-      <c r="C43" s="1" t="inlineStr"/>
-      <c r="D43" s="1" t="inlineStr"/>
-      <c r="E43" s="1" t="inlineStr"/>
-      <c r="F43" s="1" t="inlineStr"/>
-      <c r="G43" s="1" t="inlineStr"/>
-      <c r="H43" s="1" t="inlineStr">
-        <is>
-          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
-        </is>
-      </c>
-      <c r="I43" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J43" s="1" t="inlineStr"/>
-      <c r="K43" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L43" s="1" t="inlineStr"/>
-      <c r="M43" s="1" t="inlineStr"/>
-      <c r="N43" s="1" t="inlineStr"/>
-      <c r="O43" s="1" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="1" t="inlineStr"/>
-      <c r="B44" s="1" t="inlineStr"/>
-      <c r="C44" s="1" t="inlineStr"/>
-      <c r="D44" s="1" t="inlineStr"/>
-      <c r="E44" s="1" t="inlineStr"/>
-      <c r="F44" s="1" t="inlineStr"/>
-      <c r="G44" s="1" t="inlineStr"/>
-      <c r="H44" s="1" t="inlineStr">
-        <is>
-          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="I44" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J44" s="1" t="inlineStr">
-        <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="K44" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L44" s="1" t="inlineStr"/>
-      <c r="M44" s="1" t="inlineStr"/>
-      <c r="N44" s="1" t="inlineStr"/>
-      <c r="O44" s="1" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="inlineStr"/>
-      <c r="B45" s="1" t="inlineStr"/>
-      <c r="C45" s="1" t="inlineStr"/>
-      <c r="D45" s="1" t="inlineStr"/>
-      <c r="E45" s="1" t="inlineStr"/>
-      <c r="F45" s="1" t="inlineStr"/>
-      <c r="G45" s="1" t="inlineStr"/>
-      <c r="H45" s="1" t="inlineStr">
-        <is>
-          <t>Tap YES on the skip-login confirmation dialog. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="I45" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J45" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="K45" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L45" s="1" t="inlineStr"/>
-      <c r="M45" s="1" t="inlineStr"/>
-      <c r="N45" s="1" t="inlineStr"/>
-      <c r="O45" s="1" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="1" t="inlineStr"/>
@@ -2089,7 +2127,7 @@
       <c r="G46" s="1" t="inlineStr"/>
       <c r="H46" s="1" t="inlineStr">
         <is>
-          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+          <t>Swipe left on the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I46" s="1" t="inlineStr">
@@ -2099,7 +2137,7 @@
       </c>
       <c r="J46" s="1" t="inlineStr">
         <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K46" s="1" t="inlineStr">
@@ -2122,7 +2160,7 @@
       <c r="G47" s="1" t="inlineStr"/>
       <c r="H47" s="1" t="inlineStr">
         <is>
-          <t>Tap Explore in the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I47" s="1" t="inlineStr">
@@ -2132,7 +2170,7 @@
       </c>
       <c r="J47" s="1" t="inlineStr">
         <is>
-          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K47" s="1" t="inlineStr">
@@ -2155,7 +2193,7 @@
       <c r="G48" s="1" t="inlineStr"/>
       <c r="H48" s="1" t="inlineStr">
         <is>
-          <t>Tap a picture from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I48" s="1" t="inlineStr">
@@ -2165,7 +2203,7 @@
       </c>
       <c r="J48" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K48" s="1" t="inlineStr">
@@ -2188,7 +2226,7 @@
       <c r="G49" s="1" t="inlineStr"/>
       <c r="H49" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe left on the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I49" s="1" t="inlineStr">
@@ -2198,7 +2236,7 @@
       </c>
       <c r="J49" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K49" s="1" t="inlineStr">
@@ -2221,7 +2259,7 @@
       <c r="G50" s="1" t="inlineStr"/>
       <c r="H50" s="1" t="inlineStr">
         <is>
-          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Tap YES! on the final welcome screen. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I50" s="1" t="inlineStr">
@@ -2231,7 +2269,7 @@
       </c>
       <c r="J50" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="K50" s="1" t="inlineStr">
@@ -2254,22 +2292,18 @@
       <c r="G51" s="1" t="inlineStr"/>
       <c r="H51" s="1" t="inlineStr">
         <is>
-          <t>Tap a category in the media details metadata list. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
         </is>
       </c>
       <c r="I51" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J51" s="1" t="inlineStr">
-        <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J51" s="1" t="inlineStr"/>
       <c r="K51" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L51" s="1" t="inlineStr"/>
@@ -2287,22 +2321,18 @@
       <c r="G52" s="1" t="inlineStr"/>
       <c r="H52" s="1" t="inlineStr">
         <is>
-          <t>Tap the PARENT CATEGORIES tab on the category details screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
         </is>
       </c>
       <c r="I52" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J52" s="1" t="inlineStr">
-        <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J52" s="1" t="inlineStr"/>
       <c r="K52" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L52" s="1" t="inlineStr"/>
@@ -2311,48 +2341,345 @@
       <c r="O52" s="1" t="inlineStr"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="inlineStr"/>
-      <c r="B53" s="2" t="inlineStr"/>
-      <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-      <c r="H53" s="2" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr"/>
-      <c r="K53" s="2" t="inlineStr"/>
-      <c r="L53" s="2" t="inlineStr"/>
-      <c r="M53" s="2" t="inlineStr"/>
-      <c r="N53" s="2" t="inlineStr"/>
-      <c r="O53" s="2" t="inlineStr"/>
+      <c r="A53" s="1" t="inlineStr"/>
+      <c r="B53" s="1" t="inlineStr"/>
+      <c r="C53" s="1" t="inlineStr"/>
+      <c r="D53" s="1" t="inlineStr"/>
+      <c r="E53" s="1" t="inlineStr"/>
+      <c r="F53" s="1" t="inlineStr"/>
+      <c r="G53" s="1" t="inlineStr"/>
+      <c r="H53" s="1" t="inlineStr">
+        <is>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="I53" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J53" s="1" t="inlineStr">
+        <is>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="K53" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L53" s="1" t="inlineStr"/>
+      <c r="M53" s="1" t="inlineStr"/>
+      <c r="N53" s="1" t="inlineStr"/>
+      <c r="O53" s="1" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="1" t="n">
+      <c r="A54" s="1" t="inlineStr"/>
+      <c r="B54" s="1" t="inlineStr"/>
+      <c r="C54" s="1" t="inlineStr"/>
+      <c r="D54" s="1" t="inlineStr"/>
+      <c r="E54" s="1" t="inlineStr"/>
+      <c r="F54" s="1" t="inlineStr"/>
+      <c r="G54" s="1" t="inlineStr"/>
+      <c r="H54" s="1" t="inlineStr">
+        <is>
+          <t>Tap YES on the skip-login confirmation dialog. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="I54" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J54" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="K54" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L54" s="1" t="inlineStr"/>
+      <c r="M54" s="1" t="inlineStr"/>
+      <c r="N54" s="1" t="inlineStr"/>
+      <c r="O54" s="1" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="1" t="inlineStr"/>
+      <c r="B55" s="1" t="inlineStr"/>
+      <c r="C55" s="1" t="inlineStr"/>
+      <c r="D55" s="1" t="inlineStr"/>
+      <c r="E55" s="1" t="inlineStr"/>
+      <c r="F55" s="1" t="inlineStr"/>
+      <c r="G55" s="1" t="inlineStr"/>
+      <c r="H55" s="1" t="inlineStr">
+        <is>
+          <t>Open the navigation drawer from the Explore screen. &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
+      <c r="I55" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J55" s="1" t="inlineStr">
+        <is>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
+        </is>
+      </c>
+      <c r="K55" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L55" s="1" t="inlineStr"/>
+      <c r="M55" s="1" t="inlineStr"/>
+      <c r="N55" s="1" t="inlineStr"/>
+      <c r="O55" s="1" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="1" t="inlineStr"/>
+      <c r="B56" s="1" t="inlineStr"/>
+      <c r="C56" s="1" t="inlineStr"/>
+      <c r="D56" s="1" t="inlineStr"/>
+      <c r="E56" s="1" t="inlineStr"/>
+      <c r="F56" s="1" t="inlineStr"/>
+      <c r="G56" s="1" t="inlineStr"/>
+      <c r="H56" s="1" t="inlineStr">
+        <is>
+          <t>Tap Explore in the navigation drawer. &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+        </is>
+      </c>
+      <c r="I56" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J56" s="1" t="inlineStr">
+        <is>
+          <t>Click Explore &lt;2cb54b6b2c319fadcb77770ddc6f08bc1620d2ea99af5e4315a0e04d97476e34&gt;</t>
+        </is>
+      </c>
+      <c r="K56" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L56" s="1" t="inlineStr"/>
+      <c r="M56" s="1" t="inlineStr"/>
+      <c r="N56" s="1" t="inlineStr"/>
+      <c r="O56" s="1" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="1" t="inlineStr"/>
+      <c r="B57" s="1" t="inlineStr"/>
+      <c r="C57" s="1" t="inlineStr"/>
+      <c r="D57" s="1" t="inlineStr"/>
+      <c r="E57" s="1" t="inlineStr"/>
+      <c r="F57" s="1" t="inlineStr"/>
+      <c r="G57" s="1" t="inlineStr"/>
+      <c r="H57" s="1" t="inlineStr">
+        <is>
+          <t>Tap a picture from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="I57" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J57" s="1" t="inlineStr">
+        <is>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="K57" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L57" s="1" t="inlineStr"/>
+      <c r="M57" s="1" t="inlineStr"/>
+      <c r="N57" s="1" t="inlineStr"/>
+      <c r="O57" s="1" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="1" t="inlineStr"/>
+      <c r="B58" s="1" t="inlineStr"/>
+      <c r="C58" s="1" t="inlineStr"/>
+      <c r="D58" s="1" t="inlineStr"/>
+      <c r="E58" s="1" t="inlineStr"/>
+      <c r="F58" s="1" t="inlineStr"/>
+      <c r="G58" s="1" t="inlineStr"/>
+      <c r="H58" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up on the media details screen. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="I58" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J58" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="K58" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L58" s="1" t="inlineStr"/>
+      <c r="M58" s="1" t="inlineStr"/>
+      <c r="N58" s="1" t="inlineStr"/>
+      <c r="O58" s="1" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="1" t="inlineStr"/>
+      <c r="B59" s="1" t="inlineStr"/>
+      <c r="C59" s="1" t="inlineStr"/>
+      <c r="D59" s="1" t="inlineStr"/>
+      <c r="E59" s="1" t="inlineStr"/>
+      <c r="F59" s="1" t="inlineStr"/>
+      <c r="G59" s="1" t="inlineStr"/>
+      <c r="H59" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up again on the media details screen. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="I59" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J59" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="K59" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L59" s="1" t="inlineStr"/>
+      <c r="M59" s="1" t="inlineStr"/>
+      <c r="N59" s="1" t="inlineStr"/>
+      <c r="O59" s="1" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="1" t="inlineStr"/>
+      <c r="B60" s="1" t="inlineStr"/>
+      <c r="C60" s="1" t="inlineStr"/>
+      <c r="D60" s="1" t="inlineStr"/>
+      <c r="E60" s="1" t="inlineStr"/>
+      <c r="F60" s="1" t="inlineStr"/>
+      <c r="G60" s="1" t="inlineStr"/>
+      <c r="H60" s="1" t="inlineStr">
+        <is>
+          <t>Tap a category in the media details metadata list. &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="I60" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J60" s="1" t="inlineStr">
+        <is>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="K60" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L60" s="1" t="inlineStr"/>
+      <c r="M60" s="1" t="inlineStr"/>
+      <c r="N60" s="1" t="inlineStr"/>
+      <c r="O60" s="1" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="1" t="inlineStr"/>
+      <c r="B61" s="1" t="inlineStr"/>
+      <c r="C61" s="1" t="inlineStr"/>
+      <c r="D61" s="1" t="inlineStr"/>
+      <c r="E61" s="1" t="inlineStr"/>
+      <c r="F61" s="1" t="inlineStr"/>
+      <c r="G61" s="1" t="inlineStr"/>
+      <c r="H61" s="1" t="inlineStr">
+        <is>
+          <t>Tap the PARENT CATEGORIES tab on the category details screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I61" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J61" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K61" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L61" s="1" t="inlineStr"/>
+      <c r="M61" s="1" t="inlineStr"/>
+      <c r="N61" s="1" t="inlineStr"/>
+      <c r="O61" s="1" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr"/>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr"/>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr"/>
+      <c r="M62" s="2" t="inlineStr"/>
+      <c r="N62" s="2" t="inlineStr"/>
+      <c r="O62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="B54" s="1" t="inlineStr">
+      <c r="B63" s="1" t="inlineStr">
         <is>
           <t>Wikimedia Commons</t>
         </is>
       </c>
-      <c r="C54" s="1" t="inlineStr">
+      <c r="C63" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D54" s="1" t="inlineStr">
+      <c r="D63" s="1" t="inlineStr">
         <is>
           <t>LC_HP</t>
         </is>
       </c>
-      <c r="E54" s="1" t="inlineStr">
+      <c r="E63" s="1" t="inlineStr">
         <is>
           <t>The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
-      <c r="F54" s="1" t="inlineStr"/>
-      <c r="G54" s="1" t="inlineStr">
+      <c r="F63" s="1" t="inlineStr"/>
+      <c r="G63" s="1" t="inlineStr">
         <is>
           <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
 2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
@@ -2371,334 +2698,41 @@
 15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
-      <c r="H54" s="1" t="inlineStr">
+      <c r="H63" s="1" t="inlineStr">
         <is>
           <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="I54" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J54" s="1" t="inlineStr">
+      <c r="I63" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J63" s="1" t="inlineStr">
         <is>
           <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="K54" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L54" s="1">
-        <f>IFERROR(COUNTIF(K54:K68,"CS")/COUNTA(K54:K68),"")</f>
+      <c r="K63" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L63" s="1">
+        <f>IFERROR(COUNTIF(K63:K77,"CS")/COUNTA(K63:K77),"")</f>
         <v/>
       </c>
-      <c r="M54" s="1">
-        <f>COUNTIF(K54:K68,"CS")/15</f>
+      <c r="M63" s="1">
+        <f>COUNTIF(K63:K77,"CS")/15</f>
         <v/>
       </c>
-      <c r="N54" s="1">
-        <f>IFERROR(2*(L54*M54)/(L54+M54),"")</f>
+      <c r="N63" s="1">
+        <f>IFERROR(2*(L63*M63)/(L63+M63),"")</f>
         <v/>
       </c>
-      <c r="O54" s="1" t="n">
+      <c r="O63" s="1" t="n">
         <v>15</v>
       </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr"/>
-      <c r="B55" s="1" t="inlineStr"/>
-      <c r="C55" s="1" t="inlineStr"/>
-      <c r="D55" s="1" t="inlineStr"/>
-      <c r="E55" s="1" t="inlineStr"/>
-      <c r="F55" s="1" t="inlineStr"/>
-      <c r="G55" s="1" t="inlineStr"/>
-      <c r="H55" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="I55" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J55" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="K55" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L55" s="1" t="inlineStr"/>
-      <c r="M55" s="1" t="inlineStr"/>
-      <c r="N55" s="1" t="inlineStr"/>
-      <c r="O55" s="1" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="1" t="inlineStr"/>
-      <c r="B56" s="1" t="inlineStr"/>
-      <c r="C56" s="1" t="inlineStr"/>
-      <c r="D56" s="1" t="inlineStr"/>
-      <c r="E56" s="1" t="inlineStr"/>
-      <c r="F56" s="1" t="inlineStr"/>
-      <c r="G56" s="1" t="inlineStr"/>
-      <c r="H56" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="I56" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J56" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="K56" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L56" s="1" t="inlineStr"/>
-      <c r="M56" s="1" t="inlineStr"/>
-      <c r="N56" s="1" t="inlineStr"/>
-      <c r="O56" s="1" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="1" t="inlineStr"/>
-      <c r="B57" s="1" t="inlineStr"/>
-      <c r="C57" s="1" t="inlineStr"/>
-      <c r="D57" s="1" t="inlineStr"/>
-      <c r="E57" s="1" t="inlineStr"/>
-      <c r="F57" s="1" t="inlineStr"/>
-      <c r="G57" s="1" t="inlineStr"/>
-      <c r="H57" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="I57" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J57" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="K57" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L57" s="1" t="inlineStr"/>
-      <c r="M57" s="1" t="inlineStr"/>
-      <c r="N57" s="1" t="inlineStr"/>
-      <c r="O57" s="1" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="1" t="inlineStr"/>
-      <c r="B58" s="1" t="inlineStr"/>
-      <c r="C58" s="1" t="inlineStr"/>
-      <c r="D58" s="1" t="inlineStr"/>
-      <c r="E58" s="1" t="inlineStr"/>
-      <c r="F58" s="1" t="inlineStr"/>
-      <c r="G58" s="1" t="inlineStr"/>
-      <c r="H58" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="I58" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J58" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="K58" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L58" s="1" t="inlineStr"/>
-      <c r="M58" s="1" t="inlineStr"/>
-      <c r="N58" s="1" t="inlineStr"/>
-      <c r="O58" s="1" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="1" t="inlineStr"/>
-      <c r="B59" s="1" t="inlineStr"/>
-      <c r="C59" s="1" t="inlineStr"/>
-      <c r="D59" s="1" t="inlineStr"/>
-      <c r="E59" s="1" t="inlineStr"/>
-      <c r="F59" s="1" t="inlineStr"/>
-      <c r="G59" s="1" t="inlineStr"/>
-      <c r="H59" s="1" t="inlineStr">
-        <is>
-          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="I59" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J59" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="K59" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L59" s="1" t="inlineStr"/>
-      <c r="M59" s="1" t="inlineStr"/>
-      <c r="N59" s="1" t="inlineStr"/>
-      <c r="O59" s="1" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="1" t="inlineStr"/>
-      <c r="B60" s="1" t="inlineStr"/>
-      <c r="C60" s="1" t="inlineStr"/>
-      <c r="D60" s="1" t="inlineStr"/>
-      <c r="E60" s="1" t="inlineStr"/>
-      <c r="F60" s="1" t="inlineStr"/>
-      <c r="G60" s="1" t="inlineStr"/>
-      <c r="H60" s="1" t="inlineStr">
-        <is>
-          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="I60" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J60" s="1" t="inlineStr">
-        <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="K60" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L60" s="1" t="inlineStr"/>
-      <c r="M60" s="1" t="inlineStr"/>
-      <c r="N60" s="1" t="inlineStr"/>
-      <c r="O60" s="1" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="1" t="inlineStr"/>
-      <c r="B61" s="1" t="inlineStr"/>
-      <c r="C61" s="1" t="inlineStr"/>
-      <c r="D61" s="1" t="inlineStr"/>
-      <c r="E61" s="1" t="inlineStr"/>
-      <c r="F61" s="1" t="inlineStr"/>
-      <c r="G61" s="1" t="inlineStr"/>
-      <c r="H61" s="1" t="inlineStr">
-        <is>
-          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="I61" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J61" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="K61" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L61" s="1" t="inlineStr"/>
-      <c r="M61" s="1" t="inlineStr"/>
-      <c r="N61" s="1" t="inlineStr"/>
-      <c r="O61" s="1" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="1" t="inlineStr"/>
-      <c r="B62" s="1" t="inlineStr"/>
-      <c r="C62" s="1" t="inlineStr"/>
-      <c r="D62" s="1" t="inlineStr"/>
-      <c r="E62" s="1" t="inlineStr"/>
-      <c r="F62" s="1" t="inlineStr"/>
-      <c r="G62" s="1" t="inlineStr"/>
-      <c r="H62" s="1" t="inlineStr">
-        <is>
-          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
-        </is>
-      </c>
-      <c r="I62" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J62" s="1" t="inlineStr"/>
-      <c r="K62" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L62" s="1" t="inlineStr"/>
-      <c r="M62" s="1" t="inlineStr"/>
-      <c r="N62" s="1" t="inlineStr"/>
-      <c r="O62" s="1" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="1" t="inlineStr"/>
-      <c r="B63" s="1" t="inlineStr"/>
-      <c r="C63" s="1" t="inlineStr"/>
-      <c r="D63" s="1" t="inlineStr"/>
-      <c r="E63" s="1" t="inlineStr"/>
-      <c r="F63" s="1" t="inlineStr"/>
-      <c r="G63" s="1" t="inlineStr"/>
-      <c r="H63" s="1" t="inlineStr">
-        <is>
-          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
-        </is>
-      </c>
-      <c r="I63" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J63" s="1" t="inlineStr">
-        <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
-        </is>
-      </c>
-      <c r="K63" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L63" s="1" t="inlineStr"/>
-      <c r="M63" s="1" t="inlineStr"/>
-      <c r="N63" s="1" t="inlineStr"/>
-      <c r="O63" s="1" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="1" t="inlineStr"/>
@@ -2710,7 +2744,7 @@
       <c r="G64" s="1" t="inlineStr"/>
       <c r="H64" s="1" t="inlineStr">
         <is>
-          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe left through the first onboarding screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I64" s="1" t="inlineStr">
@@ -2720,7 +2754,7 @@
       </c>
       <c r="J64" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="K64" s="1" t="inlineStr">
@@ -2743,7 +2777,7 @@
       <c r="G65" s="1" t="inlineStr"/>
       <c r="H65" s="1" t="inlineStr">
         <is>
-          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I65" s="1" t="inlineStr">
@@ -2753,7 +2787,7 @@
       </c>
       <c r="J65" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K65" s="1" t="inlineStr">
@@ -2776,7 +2810,7 @@
       <c r="G66" s="1" t="inlineStr"/>
       <c r="H66" s="1" t="inlineStr">
         <is>
-          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I66" s="1" t="inlineStr">
@@ -2786,7 +2820,7 @@
       </c>
       <c r="J66" s="1" t="inlineStr">
         <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K66" s="1" t="inlineStr">
@@ -2809,7 +2843,7 @@
       <c r="G67" s="1" t="inlineStr"/>
       <c r="H67" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Swipe left through the next onboarding screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I67" s="1" t="inlineStr">
@@ -2819,7 +2853,7 @@
       </c>
       <c r="J67" s="1" t="inlineStr">
         <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K67" s="1" t="inlineStr">
@@ -2842,18 +2876,22 @@
       <c r="G68" s="1" t="inlineStr"/>
       <c r="H68" s="1" t="inlineStr">
         <is>
-          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
+          <t>Tap "YES!" to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I68" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J68" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J68" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
+        </is>
+      </c>
       <c r="K68" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L68" s="1" t="inlineStr"/>
@@ -2862,48 +2900,337 @@
       <c r="O68" s="1" t="inlineStr"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="inlineStr"/>
-      <c r="B69" s="2" t="inlineStr"/>
-      <c r="C69" s="2" t="inlineStr"/>
-      <c r="D69" s="2" t="inlineStr"/>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
-      <c r="H69" s="2" t="inlineStr"/>
-      <c r="I69" s="2" t="inlineStr"/>
-      <c r="J69" s="2" t="inlineStr"/>
-      <c r="K69" s="2" t="inlineStr"/>
-      <c r="L69" s="2" t="inlineStr"/>
-      <c r="M69" s="2" t="inlineStr"/>
-      <c r="N69" s="2" t="inlineStr"/>
-      <c r="O69" s="2" t="inlineStr"/>
+      <c r="A69" s="1" t="inlineStr"/>
+      <c r="B69" s="1" t="inlineStr"/>
+      <c r="C69" s="1" t="inlineStr"/>
+      <c r="D69" s="1" t="inlineStr"/>
+      <c r="E69" s="1" t="inlineStr"/>
+      <c r="F69" s="1" t="inlineStr"/>
+      <c r="G69" s="1" t="inlineStr"/>
+      <c r="H69" s="1" t="inlineStr">
+        <is>
+          <t>Tap "Skip" on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="I69" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J69" s="1" t="inlineStr">
+        <is>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
+        </is>
+      </c>
+      <c r="K69" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L69" s="1" t="inlineStr"/>
+      <c r="M69" s="1" t="inlineStr"/>
+      <c r="N69" s="1" t="inlineStr"/>
+      <c r="O69" s="1" t="inlineStr"/>
     </row>
     <row r="70">
-      <c r="A70" s="1" t="n">
+      <c r="A70" s="1" t="inlineStr"/>
+      <c r="B70" s="1" t="inlineStr"/>
+      <c r="C70" s="1" t="inlineStr"/>
+      <c r="D70" s="1" t="inlineStr"/>
+      <c r="E70" s="1" t="inlineStr"/>
+      <c r="F70" s="1" t="inlineStr"/>
+      <c r="G70" s="1" t="inlineStr"/>
+      <c r="H70" s="1" t="inlineStr">
+        <is>
+          <t>Tap "YES" to confirm skipping login. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="I70" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J70" s="1" t="inlineStr">
+        <is>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
+        </is>
+      </c>
+      <c r="K70" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L70" s="1" t="inlineStr"/>
+      <c r="M70" s="1" t="inlineStr"/>
+      <c r="N70" s="1" t="inlineStr"/>
+      <c r="O70" s="1" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="1" t="inlineStr"/>
+      <c r="B71" s="1" t="inlineStr"/>
+      <c r="C71" s="1" t="inlineStr"/>
+      <c r="D71" s="1" t="inlineStr"/>
+      <c r="E71" s="1" t="inlineStr"/>
+      <c r="F71" s="1" t="inlineStr"/>
+      <c r="G71" s="1" t="inlineStr"/>
+      <c r="H71" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up in Explore to reach a screen with a media item. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+        </is>
+      </c>
+      <c r="I71" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J71" s="1" t="inlineStr"/>
+      <c r="K71" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L71" s="1" t="inlineStr"/>
+      <c r="M71" s="1" t="inlineStr"/>
+      <c r="N71" s="1" t="inlineStr"/>
+      <c r="O71" s="1" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="1" t="inlineStr"/>
+      <c r="B72" s="1" t="inlineStr"/>
+      <c r="C72" s="1" t="inlineStr"/>
+      <c r="D72" s="1" t="inlineStr"/>
+      <c r="E72" s="1" t="inlineStr"/>
+      <c r="F72" s="1" t="inlineStr"/>
+      <c r="G72" s="1" t="inlineStr"/>
+      <c r="H72" s="1" t="inlineStr">
+        <is>
+          <t>Open a media item from Explore. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="I72" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J72" s="1" t="inlineStr">
+        <is>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+        </is>
+      </c>
+      <c r="K72" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L72" s="1" t="inlineStr"/>
+      <c r="M72" s="1" t="inlineStr"/>
+      <c r="N72" s="1" t="inlineStr"/>
+      <c r="O72" s="1" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="1" t="inlineStr"/>
+      <c r="B73" s="1" t="inlineStr"/>
+      <c r="C73" s="1" t="inlineStr"/>
+      <c r="D73" s="1" t="inlineStr"/>
+      <c r="E73" s="1" t="inlineStr"/>
+      <c r="F73" s="1" t="inlineStr"/>
+      <c r="G73" s="1" t="inlineStr"/>
+      <c r="H73" s="1" t="inlineStr">
+        <is>
+          <t>Swipe up in the media details screen to scroll toward the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="I73" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J73" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+        </is>
+      </c>
+      <c r="K73" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L73" s="1" t="inlineStr"/>
+      <c r="M73" s="1" t="inlineStr"/>
+      <c r="N73" s="1" t="inlineStr"/>
+      <c r="O73" s="1" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="1" t="inlineStr"/>
+      <c r="B74" s="1" t="inlineStr"/>
+      <c r="C74" s="1" t="inlineStr"/>
+      <c r="D74" s="1" t="inlineStr"/>
+      <c r="E74" s="1" t="inlineStr"/>
+      <c r="F74" s="1" t="inlineStr"/>
+      <c r="G74" s="1" t="inlineStr"/>
+      <c r="H74" s="1" t="inlineStr">
+        <is>
+          <t>Continue swiping up until the category entries are visible. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="I74" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J74" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+        </is>
+      </c>
+      <c r="K74" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L74" s="1" t="inlineStr"/>
+      <c r="M74" s="1" t="inlineStr"/>
+      <c r="N74" s="1" t="inlineStr"/>
+      <c r="O74" s="1" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="1" t="inlineStr"/>
+      <c r="B75" s="1" t="inlineStr"/>
+      <c r="C75" s="1" t="inlineStr"/>
+      <c r="D75" s="1" t="inlineStr"/>
+      <c r="E75" s="1" t="inlineStr"/>
+      <c r="F75" s="1" t="inlineStr"/>
+      <c r="G75" s="1" t="inlineStr"/>
+      <c r="H75" s="1" t="inlineStr">
+        <is>
+          <t>Tap the category "Focus stacking images of insects." &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="I75" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J75" s="1" t="inlineStr">
+        <is>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+        </is>
+      </c>
+      <c r="K75" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L75" s="1" t="inlineStr"/>
+      <c r="M75" s="1" t="inlineStr"/>
+      <c r="N75" s="1" t="inlineStr"/>
+      <c r="O75" s="1" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="1" t="inlineStr"/>
+      <c r="B76" s="1" t="inlineStr"/>
+      <c r="C76" s="1" t="inlineStr"/>
+      <c r="D76" s="1" t="inlineStr"/>
+      <c r="E76" s="1" t="inlineStr"/>
+      <c r="F76" s="1" t="inlineStr"/>
+      <c r="G76" s="1" t="inlineStr"/>
+      <c r="H76" s="1" t="inlineStr">
+        <is>
+          <t>Tap the "PARENT CATEGORIES" tab on the category screen. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="I76" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J76" s="1" t="inlineStr">
+        <is>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+        </is>
+      </c>
+      <c r="K76" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L76" s="1" t="inlineStr"/>
+      <c r="M76" s="1" t="inlineStr"/>
+      <c r="N76" s="1" t="inlineStr"/>
+      <c r="O76" s="1" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="1" t="inlineStr"/>
+      <c r="B77" s="1" t="inlineStr"/>
+      <c r="C77" s="1" t="inlineStr"/>
+      <c r="D77" s="1" t="inlineStr"/>
+      <c r="E77" s="1" t="inlineStr"/>
+      <c r="F77" s="1" t="inlineStr"/>
+      <c r="G77" s="1" t="inlineStr"/>
+      <c r="H77" s="1" t="inlineStr">
+        <is>
+          <t>Tap the "PARENT CATEGORIES" tab again. &lt;6be714d047ab21effd5c736c32506e18bd08b4c8e44ecb14442be1e47d5253a5&gt;</t>
+        </is>
+      </c>
+      <c r="I77" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J77" s="1" t="inlineStr"/>
+      <c r="K77" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L77" s="1" t="inlineStr"/>
+      <c r="M77" s="1" t="inlineStr"/>
+      <c r="N77" s="1" t="inlineStr"/>
+      <c r="O77" s="1" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr"/>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
+      <c r="I78" s="2" t="inlineStr"/>
+      <c r="J78" s="2" t="inlineStr"/>
+      <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr"/>
+      <c r="M78" s="2" t="inlineStr"/>
+      <c r="N78" s="2" t="inlineStr"/>
+      <c r="O78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="1" t="n">
         <v>135</v>
       </c>
-      <c r="B70" s="1" t="inlineStr">
+      <c r="B79" s="1" t="inlineStr">
         <is>
           <t>Wikimedia Commons</t>
         </is>
       </c>
-      <c r="C70" s="1" t="inlineStr">
+      <c r="C79" s="1" t="inlineStr">
         <is>
           <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
         </is>
       </c>
-      <c r="D70" s="1" t="inlineStr">
+      <c r="D79" s="1" t="inlineStr">
         <is>
           <t>MC_HP</t>
         </is>
       </c>
-      <c r="E70" s="1" t="inlineStr">
+      <c r="E79" s="1" t="inlineStr">
         <is>
           <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
-      <c r="F70" s="1" t="inlineStr"/>
-      <c r="G70" s="1" t="inlineStr">
+      <c r="F79" s="1" t="inlineStr"/>
+      <c r="G79" s="1" t="inlineStr">
         <is>
           <t>1. Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;
 2. Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;
@@ -2922,334 +3249,41 @@
 15. Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
-      <c r="H70" s="1" t="inlineStr">
+      <c r="H79" s="1" t="inlineStr">
         <is>
           <t>Open the app. &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="I70" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J70" s="1" t="inlineStr">
+      <c r="I79" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J79" s="1" t="inlineStr">
         <is>
           <t>Open App &lt;8e8c7133a537849ea1f09bcc2625161404e90d5f93d33e01c0e90230c92a5a7a&gt;</t>
         </is>
       </c>
-      <c r="K70" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L70" s="1">
-        <f>IFERROR(COUNTIF(K70:K85,"CS")/COUNTA(K70:K85),"")</f>
+      <c r="K79" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L79" s="1">
+        <f>IFERROR(COUNTIF(K79:K94,"CS")/COUNTA(K79:K94),"")</f>
         <v/>
       </c>
-      <c r="M70" s="1">
-        <f>COUNTIF(K70:K85,"CS")/15</f>
+      <c r="M79" s="1">
+        <f>COUNTIF(K79:K94,"CS")/15</f>
         <v/>
       </c>
-      <c r="N70" s="1">
-        <f>IFERROR(2*(L70*M70)/(L70+M70),"")</f>
+      <c r="N79" s="1">
+        <f>IFERROR(2*(L79*M79)/(L79+M79),"")</f>
         <v/>
       </c>
-      <c r="O70" s="1" t="n">
+      <c r="O79" s="1" t="n">
         <v>15</v>
       </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="1" t="inlineStr"/>
-      <c r="B71" s="1" t="inlineStr"/>
-      <c r="C71" s="1" t="inlineStr"/>
-      <c r="D71" s="1" t="inlineStr"/>
-      <c r="E71" s="1" t="inlineStr"/>
-      <c r="F71" s="1" t="inlineStr"/>
-      <c r="G71" s="1" t="inlineStr"/>
-      <c r="H71" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="I71" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J71" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
-        </is>
-      </c>
-      <c r="K71" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L71" s="1" t="inlineStr"/>
-      <c r="M71" s="1" t="inlineStr"/>
-      <c r="N71" s="1" t="inlineStr"/>
-      <c r="O71" s="1" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="1" t="inlineStr"/>
-      <c r="B72" s="1" t="inlineStr"/>
-      <c r="C72" s="1" t="inlineStr"/>
-      <c r="D72" s="1" t="inlineStr"/>
-      <c r="E72" s="1" t="inlineStr"/>
-      <c r="F72" s="1" t="inlineStr"/>
-      <c r="G72" s="1" t="inlineStr"/>
-      <c r="H72" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="I72" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J72" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
-        </is>
-      </c>
-      <c r="K72" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L72" s="1" t="inlineStr"/>
-      <c r="M72" s="1" t="inlineStr"/>
-      <c r="N72" s="1" t="inlineStr"/>
-      <c r="O72" s="1" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="1" t="inlineStr"/>
-      <c r="B73" s="1" t="inlineStr"/>
-      <c r="C73" s="1" t="inlineStr"/>
-      <c r="D73" s="1" t="inlineStr"/>
-      <c r="E73" s="1" t="inlineStr"/>
-      <c r="F73" s="1" t="inlineStr"/>
-      <c r="G73" s="1" t="inlineStr"/>
-      <c r="H73" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="I73" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J73" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
-        </is>
-      </c>
-      <c r="K73" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L73" s="1" t="inlineStr"/>
-      <c r="M73" s="1" t="inlineStr"/>
-      <c r="N73" s="1" t="inlineStr"/>
-      <c r="O73" s="1" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="1" t="inlineStr"/>
-      <c r="B74" s="1" t="inlineStr"/>
-      <c r="C74" s="1" t="inlineStr"/>
-      <c r="D74" s="1" t="inlineStr"/>
-      <c r="E74" s="1" t="inlineStr"/>
-      <c r="F74" s="1" t="inlineStr"/>
-      <c r="G74" s="1" t="inlineStr"/>
-      <c r="H74" s="1" t="inlineStr">
-        <is>
-          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="I74" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J74" s="1" t="inlineStr">
-        <is>
-          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
-        </is>
-      </c>
-      <c r="K74" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L74" s="1" t="inlineStr"/>
-      <c r="M74" s="1" t="inlineStr"/>
-      <c r="N74" s="1" t="inlineStr"/>
-      <c r="O74" s="1" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="1" t="inlineStr"/>
-      <c r="B75" s="1" t="inlineStr"/>
-      <c r="C75" s="1" t="inlineStr"/>
-      <c r="D75" s="1" t="inlineStr"/>
-      <c r="E75" s="1" t="inlineStr"/>
-      <c r="F75" s="1" t="inlineStr"/>
-      <c r="G75" s="1" t="inlineStr"/>
-      <c r="H75" s="1" t="inlineStr">
-        <is>
-          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="I75" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J75" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
-        </is>
-      </c>
-      <c r="K75" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L75" s="1" t="inlineStr"/>
-      <c r="M75" s="1" t="inlineStr"/>
-      <c r="N75" s="1" t="inlineStr"/>
-      <c r="O75" s="1" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="1" t="inlineStr"/>
-      <c r="B76" s="1" t="inlineStr"/>
-      <c r="C76" s="1" t="inlineStr"/>
-      <c r="D76" s="1" t="inlineStr"/>
-      <c r="E76" s="1" t="inlineStr"/>
-      <c r="F76" s="1" t="inlineStr"/>
-      <c r="G76" s="1" t="inlineStr"/>
-      <c r="H76" s="1" t="inlineStr">
-        <is>
-          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
-        </is>
-      </c>
-      <c r="I76" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J76" s="1" t="inlineStr">
-        <is>
-          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
-        </is>
-      </c>
-      <c r="K76" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L76" s="1" t="inlineStr"/>
-      <c r="M76" s="1" t="inlineStr"/>
-      <c r="N76" s="1" t="inlineStr"/>
-      <c r="O76" s="1" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="1" t="inlineStr"/>
-      <c r="B77" s="1" t="inlineStr"/>
-      <c r="C77" s="1" t="inlineStr"/>
-      <c r="D77" s="1" t="inlineStr"/>
-      <c r="E77" s="1" t="inlineStr"/>
-      <c r="F77" s="1" t="inlineStr"/>
-      <c r="G77" s="1" t="inlineStr"/>
-      <c r="H77" s="1" t="inlineStr">
-        <is>
-          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
-        </is>
-      </c>
-      <c r="I77" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J77" s="1" t="inlineStr"/>
-      <c r="K77" s="1" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="L77" s="1" t="inlineStr"/>
-      <c r="M77" s="1" t="inlineStr"/>
-      <c r="N77" s="1" t="inlineStr"/>
-      <c r="O77" s="1" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="1" t="inlineStr"/>
-      <c r="B78" s="1" t="inlineStr"/>
-      <c r="C78" s="1" t="inlineStr"/>
-      <c r="D78" s="1" t="inlineStr"/>
-      <c r="E78" s="1" t="inlineStr"/>
-      <c r="F78" s="1" t="inlineStr"/>
-      <c r="G78" s="1" t="inlineStr"/>
-      <c r="H78" s="1" t="inlineStr">
-        <is>
-          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="I78" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J78" s="1" t="inlineStr">
-        <is>
-          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
-        </is>
-      </c>
-      <c r="K78" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L78" s="1" t="inlineStr"/>
-      <c r="M78" s="1" t="inlineStr"/>
-      <c r="N78" s="1" t="inlineStr"/>
-      <c r="O78" s="1" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="1" t="inlineStr"/>
-      <c r="B79" s="1" t="inlineStr"/>
-      <c r="C79" s="1" t="inlineStr"/>
-      <c r="D79" s="1" t="inlineStr"/>
-      <c r="E79" s="1" t="inlineStr"/>
-      <c r="F79" s="1" t="inlineStr"/>
-      <c r="G79" s="1" t="inlineStr"/>
-      <c r="H79" s="1" t="inlineStr">
-        <is>
-          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="I79" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J79" s="1" t="inlineStr">
-        <is>
-          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
-        </is>
-      </c>
-      <c r="K79" s="1" t="inlineStr">
-        <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="L79" s="1" t="inlineStr"/>
-      <c r="M79" s="1" t="inlineStr"/>
-      <c r="N79" s="1" t="inlineStr"/>
-      <c r="O79" s="1" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="1" t="inlineStr"/>
@@ -3261,18 +3295,22 @@
       <c r="G80" s="1" t="inlineStr"/>
       <c r="H80" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
+          <t>Swipe left on the first welcome screen. &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
         </is>
       </c>
       <c r="I80" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J80" s="1" t="inlineStr">
+        <is>
+          <t>Swipe Left &lt;b3d177434c01973aefd635e9b2c077d1ba46bf4e2a80da4ed89474511160b63d&gt;</t>
+        </is>
+      </c>
       <c r="K80" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L80" s="1" t="inlineStr"/>
@@ -3290,7 +3328,7 @@
       <c r="G81" s="1" t="inlineStr"/>
       <c r="H81" s="1" t="inlineStr">
         <is>
-          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe left on the second welcome screen. &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="I81" s="1" t="inlineStr">
@@ -3300,7 +3338,7 @@
       </c>
       <c r="J81" s="1" t="inlineStr">
         <is>
-          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
+          <t>Swipe Left &lt;e0f12adac56be76acb79d37d0e90aa329ca9de72ca3481f451a5311f141027c4&gt;</t>
         </is>
       </c>
       <c r="K81" s="1" t="inlineStr">
@@ -3323,7 +3361,7 @@
       <c r="G82" s="1" t="inlineStr"/>
       <c r="H82" s="1" t="inlineStr">
         <is>
-          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe left on the third welcome screen. &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="I82" s="1" t="inlineStr">
@@ -3333,7 +3371,7 @@
       </c>
       <c r="J82" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
+          <t>Swipe Left &lt;8816181fdd2f34a86b06a3bc7208d741eee74c5da62d980f09630d2cf47f6df1&gt;</t>
         </is>
       </c>
       <c r="K82" s="1" t="inlineStr">
@@ -3356,7 +3394,7 @@
       <c r="G83" s="1" t="inlineStr"/>
       <c r="H83" s="1" t="inlineStr">
         <is>
-          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe left to the final welcome screen. &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="I83" s="1" t="inlineStr">
@@ -3366,7 +3404,7 @@
       </c>
       <c r="J83" s="1" t="inlineStr">
         <is>
-          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
+          <t>Swipe Left &lt;b71f779a1f0963d53f1859ce1784a17f4a319592a660124b62c8f18a53cf46e8&gt;</t>
         </is>
       </c>
       <c r="K83" s="1" t="inlineStr">
@@ -3389,7 +3427,7 @@
       <c r="G84" s="1" t="inlineStr"/>
       <c r="H84" s="1" t="inlineStr">
         <is>
-          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Tap the YES! button to finish onboarding. &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="I84" s="1" t="inlineStr">
@@ -3399,7 +3437,7 @@
       </c>
       <c r="J84" s="1" t="inlineStr">
         <is>
-          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
+          <t>Click YES &lt;9637973e88b508b265333dbf56463d16981017c2c09b4c69c5b9902e347d39e5&gt;</t>
         </is>
       </c>
       <c r="K84" s="1" t="inlineStr">
@@ -3422,7 +3460,7 @@
       <c r="G85" s="1" t="inlineStr"/>
       <c r="H85" s="1" t="inlineStr">
         <is>
-          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Open the navigation drawer from the Bookmarks screen. &lt;738b1be7acd4234c8f3960ed0b484e5f36707addded2ececa123a90c9fc1a1a6&gt;</t>
         </is>
       </c>
       <c r="I85" s="1" t="inlineStr">
@@ -3432,7 +3470,7 @@
       </c>
       <c r="J85" s="1" t="inlineStr">
         <is>
-          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
+          <t>Click the navigation drawer button, i.e., the menu option &lt;1d89fc61d139df7152892234c2a3f5174669a9b3b57a90c88ff95b811528ce5e&gt;</t>
         </is>
       </c>
       <c r="K85" s="1" t="inlineStr">
@@ -3446,62 +3484,45 @@
       <c r="O85" s="1" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="inlineStr"/>
-      <c r="B86" s="2" t="inlineStr"/>
-      <c r="C86" s="2" t="inlineStr"/>
-      <c r="D86" s="2" t="inlineStr"/>
-      <c r="E86" s="2" t="inlineStr"/>
-      <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
-      <c r="H86" s="2" t="inlineStr"/>
-      <c r="I86" s="2" t="inlineStr"/>
-      <c r="J86" s="2" t="inlineStr"/>
-      <c r="K86" s="2" t="inlineStr"/>
-      <c r="L86" s="2" t="inlineStr"/>
-      <c r="M86" s="2" t="inlineStr"/>
-      <c r="N86" s="2" t="inlineStr"/>
-      <c r="O86" s="2" t="inlineStr"/>
+      <c r="A86" s="1" t="inlineStr"/>
+      <c r="B86" s="1" t="inlineStr"/>
+      <c r="C86" s="1" t="inlineStr"/>
+      <c r="D86" s="1" t="inlineStr"/>
+      <c r="E86" s="1" t="inlineStr"/>
+      <c r="F86" s="1" t="inlineStr"/>
+      <c r="G86" s="1" t="inlineStr"/>
+      <c r="H86" s="1" t="inlineStr">
+        <is>
+          <t>Tap Log in in the navigation drawer. &lt;863b062d36cf4d96b243d1072ccaeab8367b05f9eb8d32b048e37b1b1fdf9c4e&gt;</t>
+        </is>
+      </c>
+      <c r="I86" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J86" s="1" t="inlineStr"/>
+      <c r="K86" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L86" s="1" t="inlineStr"/>
+      <c r="M86" s="1" t="inlineStr"/>
+      <c r="N86" s="1" t="inlineStr"/>
+      <c r="O86" s="1" t="inlineStr"/>
     </row>
     <row r="87">
-      <c r="A87" s="1" t="n">
-        <v>2</v>
-      </c>
-      <c r="B87" s="1" t="inlineStr">
-        <is>
-          <t>Family Finance</t>
-        </is>
-      </c>
-      <c r="C87" s="1" t="inlineStr">
-        <is>
-          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
-        </is>
-      </c>
-      <c r="D87" s="1" t="inlineStr">
-        <is>
-          <t>HC_HP</t>
-        </is>
-      </c>
-      <c r="E87" s="1" t="inlineStr">
-        <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
-        </is>
-      </c>
+      <c r="A87" s="1" t="inlineStr"/>
+      <c r="B87" s="1" t="inlineStr"/>
+      <c r="C87" s="1" t="inlineStr"/>
+      <c r="D87" s="1" t="inlineStr"/>
+      <c r="E87" s="1" t="inlineStr"/>
       <c r="F87" s="1" t="inlineStr"/>
-      <c r="G87" s="1" t="inlineStr">
-        <is>
-          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
-2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
-3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
-4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
-5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
-6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
-7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
-8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
-        </is>
-      </c>
+      <c r="G87" s="1" t="inlineStr"/>
       <c r="H87" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Tap Skip on the login screen. &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="I87" s="1" t="inlineStr">
@@ -3511,7 +3532,7 @@
       </c>
       <c r="J87" s="1" t="inlineStr">
         <is>
-          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+          <t>Click Skip &lt;bb009cd969fdfffc3f5842081f292334289f80d5b8fc399d1fce7ec4972173c4&gt;</t>
         </is>
       </c>
       <c r="K87" s="1" t="inlineStr">
@@ -3519,21 +3540,10 @@
           <t>CS</t>
         </is>
       </c>
-      <c r="L87" s="1">
-        <f>IFERROR(COUNTIF(K87:K94,"CS")/COUNTA(K87:K94),"")</f>
-        <v/>
-      </c>
-      <c r="M87" s="1">
-        <f>COUNTIF(K87:K94,"CS")/8</f>
-        <v/>
-      </c>
-      <c r="N87" s="1">
-        <f>IFERROR(2*(L87*M87)/(L87+M87),"")</f>
-        <v/>
-      </c>
-      <c r="O87" s="1" t="n">
-        <v>8</v>
-      </c>
+      <c r="L87" s="1" t="inlineStr"/>
+      <c r="M87" s="1" t="inlineStr"/>
+      <c r="N87" s="1" t="inlineStr"/>
+      <c r="O87" s="1" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="1" t="inlineStr"/>
@@ -3545,7 +3555,7 @@
       <c r="G88" s="1" t="inlineStr"/>
       <c r="H88" s="1" t="inlineStr">
         <is>
-          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Confirm skipping login by tapping YES. &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="I88" s="1" t="inlineStr">
@@ -3555,7 +3565,7 @@
       </c>
       <c r="J88" s="1" t="inlineStr">
         <is>
-          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+          <t>Click YES &lt;a15358162dfdc9d6068f688c1a95276f63e1788b93f9311047afa58f7e695b0b&gt;</t>
         </is>
       </c>
       <c r="K88" s="1" t="inlineStr">
@@ -3578,22 +3588,18 @@
       <c r="G89" s="1" t="inlineStr"/>
       <c r="H89" s="1" t="inlineStr">
         <is>
-          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Swipe up on the Explore screen. &lt;8a5e9e75126660d60392ee6c2946d0f28be30676865462118ea818c1459fda98&gt;</t>
         </is>
       </c>
       <c r="I89" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
-        </is>
-      </c>
-      <c r="J89" s="1" t="inlineStr">
-        <is>
-          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
-        </is>
-      </c>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J89" s="1" t="inlineStr"/>
       <c r="K89" s="1" t="inlineStr">
         <is>
-          <t>CS</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="L89" s="1" t="inlineStr"/>
@@ -3611,7 +3617,7 @@
       <c r="G90" s="1" t="inlineStr"/>
       <c r="H90" s="1" t="inlineStr">
         <is>
-          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
+          <t>Select a media item from the Explore grid. &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="I90" s="1" t="inlineStr">
@@ -3621,7 +3627,7 @@
       </c>
       <c r="J90" s="1" t="inlineStr">
         <is>
-          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Click a picture &lt;eeb2dcc5b038a5365fc5e3968862c3ae476f8c007955b49e9585b8a8b05bc0c1&gt;</t>
         </is>
       </c>
       <c r="K90" s="1" t="inlineStr">
@@ -3644,7 +3650,7 @@
       <c r="G91" s="1" t="inlineStr"/>
       <c r="H91" s="1" t="inlineStr">
         <is>
-          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe up on the media details screen to reach the categories section. &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="I91" s="1" t="inlineStr">
@@ -3654,7 +3660,7 @@
       </c>
       <c r="J91" s="1" t="inlineStr">
         <is>
-          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Swipe Up &lt;d84994fbe18eaf7d76f1dfe454496f07db5e6a0c2213452558c14661322567ac&gt;</t>
         </is>
       </c>
       <c r="K91" s="1" t="inlineStr">
@@ -3677,7 +3683,7 @@
       <c r="G92" s="1" t="inlineStr"/>
       <c r="H92" s="1" t="inlineStr">
         <is>
-          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Swipe up again to reveal the category entry. &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="I92" s="1" t="inlineStr">
@@ -3687,7 +3693,7 @@
       </c>
       <c r="J92" s="1" t="inlineStr">
         <is>
-          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
+          <t>Swipe Up &lt;44efd4db46c1a856f86f5f10423f5a596b37a4499b0d7f8dbc4036eba4edddf7&gt;</t>
         </is>
       </c>
       <c r="K92" s="1" t="inlineStr">
@@ -3710,7 +3716,7 @@
       <c r="G93" s="1" t="inlineStr"/>
       <c r="H93" s="1" t="inlineStr">
         <is>
-          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Tap the category link "Focus stacking images of insects". &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="I93" s="1" t="inlineStr">
@@ -3720,7 +3726,7 @@
       </c>
       <c r="J93" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Click a category &lt;f855240a7c5488e1a1fd483c6fec3b99757ca2940f7ceba50517a42c5e6211dc&gt;</t>
         </is>
       </c>
       <c r="K93" s="1" t="inlineStr">
@@ -3743,7 +3749,7 @@
       <c r="G94" s="1" t="inlineStr"/>
       <c r="H94" s="1" t="inlineStr">
         <is>
-          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Tap the PARENT CATEGORIES tab. &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="I94" s="1" t="inlineStr">
@@ -3753,7 +3759,7 @@
       </c>
       <c r="J94" s="1" t="inlineStr">
         <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Click parent Categories &lt;31951cb9f29b46f435d8f75ccd1b6f6cc6ead9febe61faa81dad6e547e91a68f&gt;</t>
         </is>
       </c>
       <c r="K94" s="1" t="inlineStr">
@@ -3799,12 +3805,12 @@
       </c>
       <c r="D96" s="1" t="inlineStr">
         <is>
-          <t>MC_MP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E96" s="1" t="inlineStr">
         <is>
-          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
         </is>
       </c>
       <c r="F96" s="1" t="inlineStr"/>
@@ -3822,7 +3828,7 @@
       </c>
       <c r="H96" s="1" t="inlineStr">
         <is>
-          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+          <t>Open the app. &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
         </is>
       </c>
       <c r="I96" s="1" t="inlineStr">
@@ -3841,11 +3847,11 @@
         </is>
       </c>
       <c r="L96" s="1">
-        <f>IFERROR(COUNTIF(K96:K102,"CS")/COUNTA(K96:K102),"")</f>
+        <f>IFERROR(COUNTIF(K96:K103,"CS")/COUNTA(K96:K103),"")</f>
         <v/>
       </c>
       <c r="M96" s="1">
-        <f>COUNTIF(K96:K102,"CS")/8</f>
+        <f>COUNTIF(K96:K103,"CS")/8</f>
         <v/>
       </c>
       <c r="N96" s="1">
@@ -3866,18 +3872,22 @@
       <c r="G97" s="1" t="inlineStr"/>
       <c r="H97" s="1" t="inlineStr">
         <is>
-          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+          <t>Tap Allow on the SMS permission dialog. &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
         </is>
       </c>
       <c r="I97" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="J97" s="1" t="inlineStr"/>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J97" s="1" t="inlineStr">
+        <is>
+          <t>Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;</t>
+        </is>
+      </c>
       <c r="K97" s="1" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>CS</t>
         </is>
       </c>
       <c r="L97" s="1" t="inlineStr"/>
@@ -3895,7 +3905,7 @@
       <c r="G98" s="1" t="inlineStr"/>
       <c r="H98" s="1" t="inlineStr">
         <is>
-          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+          <t>Tap Reports from the main screen. &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
         </is>
       </c>
       <c r="I98" s="1" t="inlineStr">
@@ -3928,7 +3938,7 @@
       <c r="G99" s="1" t="inlineStr"/>
       <c r="H99" s="1" t="inlineStr">
         <is>
-          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+          <t>Select the Incomes by Articles tab. &lt;2965c3b4debc48c038e78f98002ad0883abcdd8571e00c1287e80981331ef5b4&gt;</t>
         </is>
       </c>
       <c r="I99" s="1" t="inlineStr">
@@ -3961,7 +3971,7 @@
       <c r="G100" s="1" t="inlineStr"/>
       <c r="H100" s="1" t="inlineStr">
         <is>
-          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+          <t>Tap Display to open the Display of Incomes by Articles dialog. &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
         </is>
       </c>
       <c r="I100" s="1" t="inlineStr">
@@ -3994,7 +4004,7 @@
       <c r="G101" s="1" t="inlineStr"/>
       <c r="H101" s="1" t="inlineStr">
         <is>
-          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Check the View values option. &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
         </is>
       </c>
       <c r="I101" s="1" t="inlineStr">
@@ -4004,7 +4014,7 @@
       </c>
       <c r="J101" s="1" t="inlineStr">
         <is>
-          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+          <t>Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;</t>
         </is>
       </c>
       <c r="K101" s="1" t="inlineStr">
@@ -4027,7 +4037,7 @@
       <c r="G102" s="1" t="inlineStr"/>
       <c r="H102" s="1" t="inlineStr">
         <is>
-          <t>Tap "OK" to confirm the change. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Check the Use percent values option. &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
         </is>
       </c>
       <c r="I102" s="1" t="inlineStr">
@@ -4037,7 +4047,7 @@
       </c>
       <c r="J102" s="1" t="inlineStr">
         <is>
-          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
         </is>
       </c>
       <c r="K102" s="1" t="inlineStr">
@@ -4049,6 +4059,323 @@
       <c r="M102" s="1" t="inlineStr"/>
       <c r="N102" s="1" t="inlineStr"/>
       <c r="O102" s="1" t="inlineStr"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="1" t="inlineStr"/>
+      <c r="B103" s="1" t="inlineStr"/>
+      <c r="C103" s="1" t="inlineStr"/>
+      <c r="D103" s="1" t="inlineStr"/>
+      <c r="E103" s="1" t="inlineStr"/>
+      <c r="F103" s="1" t="inlineStr"/>
+      <c r="G103" s="1" t="inlineStr"/>
+      <c r="H103" s="1" t="inlineStr">
+        <is>
+          <t>Tap OK. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I103" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J103" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K103" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L103" s="1" t="inlineStr"/>
+      <c r="M103" s="1" t="inlineStr"/>
+      <c r="N103" s="1" t="inlineStr"/>
+      <c r="O103" s="1" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr"/>
+      <c r="B104" s="2" t="inlineStr"/>
+      <c r="C104" s="2" t="inlineStr"/>
+      <c r="D104" s="2" t="inlineStr"/>
+      <c r="E104" s="2" t="inlineStr"/>
+      <c r="F104" s="2" t="inlineStr"/>
+      <c r="G104" s="2" t="inlineStr"/>
+      <c r="H104" s="2" t="inlineStr"/>
+      <c r="I104" s="2" t="inlineStr"/>
+      <c r="J104" s="2" t="inlineStr"/>
+      <c r="K104" s="2" t="inlineStr"/>
+      <c r="L104" s="2" t="inlineStr"/>
+      <c r="M104" s="2" t="inlineStr"/>
+      <c r="N104" s="2" t="inlineStr"/>
+      <c r="O104" s="2" t="inlineStr"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B105" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C105" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D105" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E105" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F105" s="1" t="inlineStr"/>
+      <c r="G105" s="1" t="inlineStr">
+        <is>
+          <t>1. Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;
+2. Click allow button &lt;8407e328c4a9d75304cf3edee19af6616ae654caca4e79229e0df0c827909816&gt;
+3. Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88
+4. Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;
+5. Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;
+6. Click view values checkbox &lt;dc01c666d81db01f9ceb751ff256033bcc27f75ab0951ef2f9eff49e39233d64&gt;
+7. Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;
+8. Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="H105" s="1" t="inlineStr">
+        <is>
+          <t>Open the app. &lt;24f7aef009bd7a8b145fd2acabd46d79833f775339f82b7248b75b22eb407522&gt;</t>
+        </is>
+      </c>
+      <c r="I105" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J105" s="1" t="inlineStr">
+        <is>
+          <t>Open app &lt;fa8baa4de2d1015dd5da60a38bcc25a725e918d25bafb6b4b8bafe8f727ccfcf&gt;</t>
+        </is>
+      </c>
+      <c r="K105" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L105" s="1">
+        <f>IFERROR(COUNTIF(K105:K111,"CS")/COUNTA(K105:K111),"")</f>
+        <v/>
+      </c>
+      <c r="M105" s="1">
+        <f>COUNTIF(K105:K111,"CS")/8</f>
+        <v/>
+      </c>
+      <c r="N105" s="1">
+        <f>IFERROR(2*(L105*M105)/(L105+M105),"")</f>
+        <v/>
+      </c>
+      <c r="O105" s="1" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="1" t="inlineStr"/>
+      <c r="B106" s="1" t="inlineStr"/>
+      <c r="C106" s="1" t="inlineStr"/>
+      <c r="D106" s="1" t="inlineStr"/>
+      <c r="E106" s="1" t="inlineStr"/>
+      <c r="F106" s="1" t="inlineStr"/>
+      <c r="G106" s="1" t="inlineStr"/>
+      <c r="H106" s="1" t="inlineStr">
+        <is>
+          <t>On the initial permission screen, tap "DENY". &lt;2b209a3d55050bc8611e4799d186aac1ed51a780062d43e781082427e0523b10&gt;</t>
+        </is>
+      </c>
+      <c r="I106" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="J106" s="1" t="inlineStr"/>
+      <c r="K106" s="1" t="inlineStr">
+        <is>
+          <t>ES</t>
+        </is>
+      </c>
+      <c r="L106" s="1" t="inlineStr"/>
+      <c r="M106" s="1" t="inlineStr"/>
+      <c r="N106" s="1" t="inlineStr"/>
+      <c r="O106" s="1" t="inlineStr"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="1" t="inlineStr"/>
+      <c r="B107" s="1" t="inlineStr"/>
+      <c r="C107" s="1" t="inlineStr"/>
+      <c r="D107" s="1" t="inlineStr"/>
+      <c r="E107" s="1" t="inlineStr"/>
+      <c r="F107" s="1" t="inlineStr"/>
+      <c r="G107" s="1" t="inlineStr"/>
+      <c r="H107" s="1" t="inlineStr">
+        <is>
+          <t>On the dashboard, tap "Reports". &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88&gt;</t>
+        </is>
+      </c>
+      <c r="I107" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J107" s="1" t="inlineStr">
+        <is>
+          <t>Click Report &lt;9a4f389ec16dc06bc51519fd35159ab49c667d2cae3e0323df9bf08cd98bda88</t>
+        </is>
+      </c>
+      <c r="K107" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L107" s="1" t="inlineStr"/>
+      <c r="M107" s="1" t="inlineStr"/>
+      <c r="N107" s="1" t="inlineStr"/>
+      <c r="O107" s="1" t="inlineStr"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="1" t="inlineStr"/>
+      <c r="B108" s="1" t="inlineStr"/>
+      <c r="C108" s="1" t="inlineStr"/>
+      <c r="D108" s="1" t="inlineStr"/>
+      <c r="E108" s="1" t="inlineStr"/>
+      <c r="F108" s="1" t="inlineStr"/>
+      <c r="G108" s="1" t="inlineStr"/>
+      <c r="H108" s="1" t="inlineStr">
+        <is>
+          <t>On the Reports screen, open "Incomes by Articles". &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="I108" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J108" s="1" t="inlineStr">
+        <is>
+          <t>Click Incomes By Articles or expenses by articles &lt;c010db1badf9deb0564b10c46916ad505c7d1acca0f840fdc12c4867c81990d0&gt;</t>
+        </is>
+      </c>
+      <c r="K108" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L108" s="1" t="inlineStr"/>
+      <c r="M108" s="1" t="inlineStr"/>
+      <c r="N108" s="1" t="inlineStr"/>
+      <c r="O108" s="1" t="inlineStr"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="1" t="inlineStr"/>
+      <c r="B109" s="1" t="inlineStr"/>
+      <c r="C109" s="1" t="inlineStr"/>
+      <c r="D109" s="1" t="inlineStr"/>
+      <c r="E109" s="1" t="inlineStr"/>
+      <c r="F109" s="1" t="inlineStr"/>
+      <c r="G109" s="1" t="inlineStr"/>
+      <c r="H109" s="1" t="inlineStr">
+        <is>
+          <t>On the Incomes by Articles report screen, tap "Display". &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="I109" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J109" s="1" t="inlineStr">
+        <is>
+          <t>Click View Button &lt;c7c181b4d07f85b6731edefa0c51eca8637b088e992c8d07e2349379db3cd413&gt;</t>
+        </is>
+      </c>
+      <c r="K109" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L109" s="1" t="inlineStr"/>
+      <c r="M109" s="1" t="inlineStr"/>
+      <c r="N109" s="1" t="inlineStr"/>
+      <c r="O109" s="1" t="inlineStr"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="1" t="inlineStr"/>
+      <c r="B110" s="1" t="inlineStr"/>
+      <c r="C110" s="1" t="inlineStr"/>
+      <c r="D110" s="1" t="inlineStr"/>
+      <c r="E110" s="1" t="inlineStr"/>
+      <c r="F110" s="1" t="inlineStr"/>
+      <c r="G110" s="1" t="inlineStr"/>
+      <c r="H110" s="1" t="inlineStr">
+        <is>
+          <t>In the display dialog, tap "Use percent values". &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="I110" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J110" s="1" t="inlineStr">
+        <is>
+          <t>Click use percent values checkbox &lt;c3292f1abb084883da9f0bf06776dd33343b186505d53bedfbb8b83717e4b319&gt;</t>
+        </is>
+      </c>
+      <c r="K110" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L110" s="1" t="inlineStr"/>
+      <c r="M110" s="1" t="inlineStr"/>
+      <c r="N110" s="1" t="inlineStr"/>
+      <c r="O110" s="1" t="inlineStr"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="1" t="inlineStr"/>
+      <c r="B111" s="1" t="inlineStr"/>
+      <c r="C111" s="1" t="inlineStr"/>
+      <c r="D111" s="1" t="inlineStr"/>
+      <c r="E111" s="1" t="inlineStr"/>
+      <c r="F111" s="1" t="inlineStr"/>
+      <c r="G111" s="1" t="inlineStr"/>
+      <c r="H111" s="1" t="inlineStr">
+        <is>
+          <t>Tap "OK" to confirm the change. &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="I111" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="J111" s="1" t="inlineStr">
+        <is>
+          <t>Click OK &lt;26c0ae2d76021672cf80c07928394773aec07f5be831f91ab09b5f7c2392b6aa&gt;</t>
+        </is>
+      </c>
+      <c r="K111" s="1" t="inlineStr">
+        <is>
+          <t>CS</t>
+        </is>
+      </c>
+      <c r="L111" s="1" t="inlineStr"/>
+      <c r="M111" s="1" t="inlineStr"/>
+      <c r="N111" s="1" t="inlineStr"/>
+      <c r="O111" s="1" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4061,7 +4388,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L16"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -4224,11 +4551,11 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>Material Files</t>
+          <t>Family Finance</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
@@ -4238,29 +4565,35 @@
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>HC_LP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr">
         <is>
-          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
-        </is>
-      </c>
-      <c r="F4" s="1" t="inlineStr"/>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Title: App crashes when applying both View values and Use percent values in the Display of Incomes by Articles dialog
+Observed Behavior: On the Display of Incomes by Articles pop-up of the Reports screen, if the user checks View values, checks Use percent values, and taps OK, the application crashes.
+Expected Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
       <c r="G4" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the server restarts automatically
-Triggering GUI Interaction: stops the FTP server and then closes the app
-Triggering Screen Reference: FTP server screen
-Correct Behavior: The FTP server should remain stopped</t>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
+Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
+Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
         </is>
       </c>
       <c r="H4" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the FTP server restarts automatically after stopping it and closing the app
-Triggering GUI Interactions: the user turns off the FTP server switch and then closes the app
-Triggering Screen Reference: On the FTP server screen
-Correct Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
+Triggering Screen Reference: On the Display of Incomes by Articles pop-up of the Reports screen
+Correct Behavior: The appearance of the report should be changed to use percent values.</t>
         </is>
       </c>
       <c r="I4" s="1" t="inlineStr">
@@ -4314,12 +4647,12 @@
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>LC_LP</t>
+          <t>HC_LP</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr">
         <is>
-          <t>It restarts on its own.</t>
+          <t>On the FTP server screen, stopping it and closing the app makes the server restart, even though it should stay stopped.</t>
         </is>
       </c>
       <c r="F6" s="1" t="inlineStr"/>
@@ -4333,10 +4666,10 @@
       </c>
       <c r="H6" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the FTP server is restarting on its own
-Triggering GUI Interactions: turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents
+          <t>Buggy Behavior: the FTP server restarts automatically after stopping it and closing the app
+Triggering GUI Interactions: the user turns off the FTP server switch and then closes the app
 Triggering Screen Reference: On the FTP server screen
-Correct Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
+Correct Behavior: The FTP server should stay stopped after stopping it and closing the app.</t>
         </is>
       </c>
       <c r="I6" s="1" t="inlineStr">
@@ -4376,11 +4709,11 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>135</v>
+        <v>10</v>
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>Wikimedia Commons</t>
+          <t>Material Files</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
@@ -4390,35 +4723,29 @@
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>HC_HP</t>
+          <t>LC_LP</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr">
         <is>
-          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F8" s="1" t="inlineStr">
-        <is>
-          <t>Title: Parent Categories tab opens a blank page on the category details screen
-Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
-Expected Behavior: The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
+          <t>It restarts on its own.</t>
+        </is>
+      </c>
+      <c r="F8" s="1" t="inlineStr"/>
       <c r="G8" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: see a blank page
-Triggering GUI Interaction: clicks the Parent Categories tab
-Triggering Screen Reference: Category screen, Parent Categories tab
-Correct Behavior: The Parent Categories of the current category should be displayed</t>
+          <t>Buggy Behavior: the server restarts automatically
+Triggering GUI Interaction: stops the FTP server and then closes the app
+Triggering Screen Reference: FTP server screen
+Correct Behavior: The FTP server should remain stopped</t>
         </is>
       </c>
       <c r="H8" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: a blank page is shown
-Triggering GUI Interactions: taps the PARENT CATEGORIES tab
-Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
-Correct Behavior: The Parent Categories of the current category should be displayed</t>
+          <t>Buggy Behavior: the FTP server is restarting on its own
+Triggering GUI Interactions: turns the server on, turns it off, leaves the FTP server screen, and then swipes the app away from Recents
+Triggering Screen Reference: On the FTP server screen
+Correct Behavior: The FTP server should remain off after the user toggles it off and leaves the FTP server screen, and it should not restart automatically on its own.</t>
         </is>
       </c>
       <c r="I8" s="1" t="inlineStr">
@@ -4472,15 +4799,21 @@
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>LC_HP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr">
         <is>
-          <t>The Parent Categories of the current category should be displayed.</t>
-        </is>
-      </c>
-      <c r="F10" s="1" t="inlineStr"/>
+          <t>Open App, swipe left four times, tap YES, tap Skip, tap YES, open the navigation drawer, select Explore, tap a picture, swipe up twice, tap a category, and tap Parent Categories to reach the Category screen in the Parent Categories tab; clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
+      <c r="F10" s="1" t="inlineStr">
+        <is>
+          <t>Title: Parent Categories tab opens a blank page on the category details screen
+Observed Behavior: On the Category Details screen in the Parent Categories tab, if the user taps the PARENT CATEGORIES tab, a blank page is shown.
+Expected Behavior: The Parent Categories of the current category should be displayed.</t>
+        </is>
+      </c>
       <c r="G10" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: see a blank page
@@ -4491,10 +4824,10 @@
       </c>
       <c r="H10" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the parent categories of the current category are not displayed
-Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
-Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
-Correct Behavior: The parent categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: a blank page is shown
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen in the Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
         </is>
       </c>
       <c r="I10" s="1" t="inlineStr">
@@ -4509,7 +4842,7 @@
       </c>
       <c r="K10" s="1" t="inlineStr">
         <is>
-          <t>Incomplete</t>
+          <t>Correct</t>
         </is>
       </c>
       <c r="L10" s="1" t="inlineStr">
@@ -4548,12 +4881,12 @@
       </c>
       <c r="D12" s="1" t="inlineStr">
         <is>
-          <t>MC_HP</t>
+          <t>LC_HP</t>
         </is>
       </c>
       <c r="E12" s="1" t="inlineStr">
         <is>
-          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
+          <t>The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F12" s="1" t="inlineStr"/>
@@ -4567,10 +4900,10 @@
       </c>
       <c r="H12" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the app results in a blank page
-Triggering GUI Interactions: taps the PARENT CATEGORIES tab
-Triggering Screen Reference: On the Category Details screen
-Correct Behavior: The Parent Categories of the current category should be displayed.</t>
+          <t>Buggy Behavior: the parent categories of the current category are not displayed
+Triggering GUI Interactions: taps the "PARENT CATEGORIES" tab
+Triggering Screen Reference: On the category details screen for "Focus stacking images of insects,"
+Correct Behavior: The parent categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I12" s="1" t="inlineStr">
@@ -4610,11 +4943,11 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>2</v>
+        <v>135</v>
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>Family Finance</t>
+          <t>Wikimedia Commons</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
@@ -4624,29 +4957,29 @@
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>HC_HP</t>
+          <t>MC_HP</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr">
         <is>
-          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
+          <t>Clicking the Parent Categories tab results in a blank page, but the Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="F14" s="1" t="inlineStr"/>
       <c r="G14" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the application crashes
-Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
-Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
-Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+          <t>Buggy Behavior: see a blank page
+Triggering GUI Interaction: clicks the Parent Categories tab
+Triggering Screen Reference: Category screen, Parent Categories tab
+Correct Behavior: The Parent Categories of the current category should be displayed</t>
         </is>
       </c>
       <c r="H14" s="1" t="inlineStr">
         <is>
-          <t>Buggy Behavior: the application crashes
-Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
-Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
-Correct Behavior: The appearance of the report should be changed to use percent values.</t>
+          <t>Buggy Behavior: the app results in a blank page
+Triggering GUI Interactions: taps the PARENT CATEGORIES tab
+Triggering Screen Reference: On the Category Details screen
+Correct Behavior: The Parent Categories of the current category should be displayed.</t>
         </is>
       </c>
       <c r="I14" s="1" t="inlineStr">
@@ -4661,7 +4994,7 @@
       </c>
       <c r="K14" s="1" t="inlineStr">
         <is>
-          <t>Correct</t>
+          <t>Incomplete</t>
         </is>
       </c>
       <c r="L14" s="1" t="inlineStr">
@@ -4700,12 +5033,12 @@
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>MC_MP</t>
+          <t>HC_HP</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr">
         <is>
-          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+          <t>On Display of Incomes by Articles pop-up of the Reports screen changing the report appearance from 'view values' to 'use percent values' causes the application to crash, but the appearance of the report should be changed to 'use percent values'. I took these steps: Open the app, tap Allow, select Report, choose Incomes By Articles or Expenses By Articles, tap View, check 'view values', check 'use percent values', and tap OK.</t>
         </is>
       </c>
       <c r="F16" s="1" t="inlineStr"/>
@@ -4720,27 +5053,103 @@
       <c r="H16" s="1" t="inlineStr">
         <is>
           <t>Buggy Behavior: the application crashes
+Triggering GUI Interactions: checks View values, checks Use percent values, and taps OK
+Triggering Screen Reference: On the Display of Incomes by Articles dialog of the Reports screen
+Correct Behavior: The appearance of the report should be changed to use percent values.</t>
+        </is>
+      </c>
+      <c r="I16" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="J16" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="K16" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+      <c r="L16" s="1" t="inlineStr">
+        <is>
+          <t>Correct</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr"/>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr"/>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B18" s="1" t="inlineStr">
+        <is>
+          <t>Family Finance</t>
+        </is>
+      </c>
+      <c r="C18" s="1" t="inlineStr">
+        <is>
+          <t>bugscribe_mutli-candidate_transitions_and_screen_descriptions</t>
+        </is>
+      </c>
+      <c r="D18" s="1" t="inlineStr">
+        <is>
+          <t>MC_MP</t>
+        </is>
+      </c>
+      <c r="E18" s="1" t="inlineStr">
+        <is>
+          <t>Changing the report appearance from 'view values' to 'use percent values' results in the application crashing.</t>
+        </is>
+      </c>
+      <c r="F18" s="1" t="inlineStr"/>
+      <c r="G18" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
+Triggering GUI Interaction: changes the appearance of the report from 'view values' to use percent values'
+Triggering Screen Reference: Display of Incomes by Articles pop-up of the Reports screen
+Correct Behavior: The appearance of the report should be changed to 'use percent values'</t>
+        </is>
+      </c>
+      <c r="H18" s="1" t="inlineStr">
+        <is>
+          <t>Buggy Behavior: the application crashes
 Triggering GUI Interactions: the user taps the "Use percent values" checkbox
 Triggering Screen Reference: On the Display of Incomes by Articles dialog
 Correct Behavior: The application should change the report appearance to use percent values without crashing.</t>
         </is>
       </c>
-      <c r="I16" s="1" t="inlineStr">
+      <c r="I18" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="J16" s="1" t="inlineStr">
+      <c r="J18" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="K16" s="1" t="inlineStr">
+      <c r="K18" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
       </c>
-      <c r="L16" s="1" t="inlineStr">
+      <c r="L18" s="1" t="inlineStr">
         <is>
           <t>Correct</t>
         </is>
@@ -4911,16 +5320,16 @@
         <v/>
       </c>
       <c r="M2" t="n">
-        <v>73273.75</v>
+        <v>71972.11111111111</v>
       </c>
       <c r="N2" t="n">
-        <v>32.391268</v>
+        <v>28.520764</v>
       </c>
       <c r="O2" t="n">
-        <v>32.391268</v>
+        <v>28.520764</v>
       </c>
       <c r="P2" t="n">
-        <v>1.375</v>
+        <v>1.333333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>